<commit_message>
Canon: starting convoy and boss drops for player equipment
weapons.convoy_qty: what the shared convoy holds at the start of a playthrough
(one mid-tier weapon per art; the overlap weapons start at 0).
encounter_spawns.drop_weapon_id: the weapon a defeated enemy adds to the
convoy, once per spawn per playthrough. Drafted: Act 1 non-trivial bosses drop
a mid-tier weapon, Act 2+ bosses and the paralogues the high tier, and the two
Billmen the halberd -- the only source of an overlap weapon. 22 drops.

canon_validate.py c07h: convoy_qty must be a non-negative integer and
drop_weapon_id must resolve (negative-tested: 2 deliberate errors, 2 blocking).
build_sqlite.py: drop_weapon_id FK, convoy_qty numeric. Validator baseline
unchanged (0 blocking / 19 warning / 5 info), foreign_key_check 0.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -911,8 +911,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J113"/>
+  <dimension ref="A1:K113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="18" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="26" t="inlineStr">
@@ -963,6 +966,11 @@
       <c r="J1" s="26" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="K1" s="26" t="inlineStr">
+        <is>
+          <t>drop_weapon_id</t>
         </is>
       </c>
     </row>
@@ -1159,6 +1167,11 @@
           <t>Guards the reliquary from one tile north.</t>
         </is>
       </c>
+      <c r="K6" s="17" t="inlineStr">
+        <is>
+          <t>wpn_bow_mid</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -1545,6 +1558,11 @@
           <t>Reuses the generic miniboss template (not a new named character -- no identity is named in map_x11's design_note) at the west crossing, matching 'two simultaneous timed objectives at opposite edges.'</t>
         </is>
       </c>
+      <c r="K16" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_high</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -3105,6 +3123,11 @@
           <t>end_perverse: 'the party fights HIM directly.' ea_warlord (the generic boss-tier template) is the closest existing fit -- no unique stat line invented for him specifically, that's real future content. No den, matching this map's own design_note ('reads as a direct, personal fight... not an attritional one').</t>
         </is>
       </c>
+      <c r="K56" s="17" t="inlineStr">
+        <is>
+          <t>wpn_sword_high</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
@@ -3615,6 +3638,11 @@
           <t>Closing chapter of the invented War arc -- ea_warlord (boss-tier template) reused for 'where it finally stops,' the arc's toughest fight.</t>
         </is>
       </c>
+      <c r="K69" s="17" t="inlineStr">
+        <is>
+          <t>wpn_axe_high</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="17" t="inlineStr">
@@ -3695,6 +3723,11 @@
           <t>npcs.npc_macuil: 'paralogue capstone.' ea_warlord reused for capstone-tier difficulty. Repositioned (2026-09-24) to row5/col12 -- dry shoreline ground at the map's new eastern shore, next to the regrounded seize tile, not in the lake patch the old row5/col8 coordinate now falls inside.</t>
         </is>
       </c>
+      <c r="K71" s="17" t="inlineStr">
+        <is>
+          <t>wpn_axe_high</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="inlineStr">
@@ -3733,6 +3766,11 @@
           <t>npcs.npc_indech: 'paralogue capstone,' same treatment as map_p_macuil.</t>
         </is>
       </c>
+      <c r="K72" s="17" t="inlineStr">
+        <is>
+          <t>wpn_axe_high</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="17" t="inlineStr">
@@ -3769,6 +3807,11 @@
           <t>locations.loc_lowest_terrace / named.nmd_shadhavar: the creature itself, placed mid-terrace, one tile east of the seize tile at row4/col8 (see game/data/maps/map_p_shadhavar.txt) -- same adjacent-not-overlapping placement used for spn_pmacuil_boss after that map's own correction.</t>
         </is>
       </c>
+      <c r="K73" s="17" t="inlineStr">
+        <is>
+          <t>wpn_reason_high</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="17" t="inlineStr">
@@ -3805,6 +3848,11 @@
           <t>locations.loc_simurgh_nest / named.nmd_simurgh: the creature at her nest, one tile east of the seize tile at row6/col8 (see game/data/maps/map_p_simurgh.txt) -- same adjacent-not-overlapping placement used for spn_pmacuil_boss and spn_pshadhavar_boss.</t>
         </is>
       </c>
+      <c r="K74" s="17" t="inlineStr">
+        <is>
+          <t>wpn_faith_high</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="17" t="inlineStr">
@@ -3841,6 +3889,11 @@
           <t>locations.loc_dove_colony / named.nmd_karkadann: the creature guarding the clearing's center, one tile east of the seize tile at row4/col8 (see game/data/maps/map_p_karkadann.txt) -- same adjacent-not-overlapping placement used for every other Named stand-in this session.</t>
         </is>
       </c>
+      <c r="K75" s="17" t="inlineStr">
+        <is>
+          <t>wpn_brawl_high</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="17" t="inlineStr">
@@ -3877,6 +3930,11 @@
           <t>locations.loc_flats_interior / named.nmd_anzu: the creature standing alone in the open flat, one tile east of the seize tile at row6/col9 (see game/data/maps/map_p_anzu.txt) -- same adjacent-not-overlapping placement used for every other Named stand-in this session.</t>
         </is>
       </c>
+      <c r="K76" s="17" t="inlineStr">
+        <is>
+          <t>wpn_bow_high</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="17" t="inlineStr">
@@ -3985,6 +4043,11 @@
           <t>No named identity, same reuse ch_v21's own encounter_spawns row already used ea_hardened_veteran for -- 'complicit hands' generally, the works' overseer guarding the archive doorway.</t>
         </is>
       </c>
+      <c r="K79" s="17" t="inlineStr">
+        <is>
+          <t>wpn_sword_mid</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="17" t="inlineStr">
@@ -4201,6 +4264,11 @@
           <t>A mobile raiding party leader, matching 'punishes slow armies' by being fast itself.</t>
         </is>
       </c>
+      <c r="K85" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_mid</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="17" t="inlineStr">
@@ -4345,6 +4413,11 @@
           <t>The gate captain -- 'the Unstained will not talk to you' means this is the answer instead.</t>
         </is>
       </c>
+      <c r="K89" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_mid</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="17" t="inlineStr">
@@ -4525,6 +4598,11 @@
           <t>A mobile Plains raiding party leader threatening the frontier city.</t>
         </is>
       </c>
+      <c r="K94" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_mid</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="17" t="inlineStr">
@@ -4597,6 +4675,11 @@
           <t>Escarpment fighting -- an organized veteran force holding the cliff edge.</t>
         </is>
       </c>
+      <c r="K96" s="17" t="inlineStr">
+        <is>
+          <t>wpn_sword_mid</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="17" t="inlineStr">
@@ -4705,6 +4788,11 @@
           <t>The chapel's defender captain, mirroring ch_d10's gate captain.</t>
         </is>
       </c>
+      <c r="K99" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_mid</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="17" t="inlineStr">
@@ -4777,6 +4865,11 @@
           <t>Act3 tier per this session's own precedent (order/paragon-tier reuse, not commoner mooks) -- the district's defending captain.</t>
         </is>
       </c>
+      <c r="K101" s="17" t="inlineStr">
+        <is>
+          <t>wpn_axe_high</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="17" t="inlineStr">
@@ -4849,6 +4942,11 @@
           <t>Paragon-tier capstone for the district's climax, guarding the colossus's base.</t>
         </is>
       </c>
+      <c r="K103" s="17" t="inlineStr">
+        <is>
+          <t>wpn_axe_high</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="17" t="inlineStr">
@@ -4993,6 +5091,11 @@
           <t>The pass's garrison captain -- 'held by whoever taxes it' reads as an organized force, not bandits.</t>
         </is>
       </c>
+      <c r="K107" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lance_high</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="17" t="inlineStr">
@@ -5029,6 +5132,11 @@
           <t>A contesting force at the reunion point itself.</t>
         </is>
       </c>
+      <c r="K108" s="17" t="inlineStr">
+        <is>
+          <t>wpn_sword_high</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="17" t="inlineStr">
@@ -5137,6 +5245,11 @@
           <t>A halberd line behind the pass's captain -- the pass is 'held by whoever taxes it', and a toll garrison keeps polearm infantry against riders. Drafted 2026-10-02.</t>
         </is>
       </c>
+      <c r="K111" s="17" t="inlineStr">
+        <is>
+          <t>wpn_halberd</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="17" t="inlineStr">
@@ -5173,11 +5286,16 @@
           <t>One halberd-bearer with the contesting force at the reunion point; see spn_tp19_billman. Drafted 2026-10-02.</t>
         </is>
       </c>
+      <c r="K112" s="17" t="inlineStr">
+        <is>
+          <t>wpn_halberd</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft, review before treating as canon. row/col are grid coordinates in the corresponding map_*.txt file (0-indexed, row0=top). kind: 'boss'/'mook' spawn once at map load; 'den' spawns wave_size new enemy_id units every spawn_interval turns, up to max_waves (null = forever). Positions are placement choices grounded in each map's own text where possible (Boyan on the defend point, Vitomir/the relic hunter den by the reliquary) but the exact tile coordinates themselves are invented, not sourced. Drafted by a Claude Code session, 2026-09-23. ADDENDUM: 12 rows added for map_d01/d03/x11/b15. None of these four maps name a specific antagonist the way map_a02/a03 do -- every row here reuses an existing grounded archetype (ea_looter, ea_conscript_levy, ea_privateer, ea_war_captain) rather than inventing new named characters, per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 2: 9 rows added for map_d02/a01/d05 -- the last three maps in the maps tab without a scene. All three reuse archetypes whose own first_seen_map_id already points at these exact maps (ea_conscript_levy/d02, ea_looter/a01, ea_privateer/d05), the closest grounding this tab gets short of a named individual. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 3: 17 rows added fleshing out the 6 Act2 skeleton maps (v21/v22/c21/m21/m22/r16) into playable content. All reuse existing archetypes -- none of these six name a specific individual antagonist the way map_a02/a03 do -- per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 4: 22 rows added fleshing out the 10 Act3/paralogue skeleton maps into playable content. Act3's tougher tier is reflected by reusing ea_war_captain/ea_warlord (the miniboss/boss templates) throughout rather than Act1/2's commoner-tier mooks -- no new archetypes invented, same discipline as every prior addendum. Drafted by a Claude Code session, 2026-09-23.</t>
+          <t>NOTE -- draft, review before treating as canon. row/col are grid coordinates in the corresponding map_*.txt file (0-indexed, row0=top). kind: 'boss'/'mook' spawn once at map load; 'den' spawns wave_size new enemy_id units every spawn_interval turns, up to max_waves (null = forever). Positions are placement choices grounded in each map's own text where possible (Boyan on the defend point, Vitomir/the relic hunter den by the reliquary) but the exact tile coordinates themselves are invented, not sourced. Drafted by a Claude Code session, 2026-09-23. ADDENDUM: 12 rows added for map_d01/d03/x11/b15. None of these four maps name a specific antagonist the way map_a02/a03 do -- every row here reuses an existing grounded archetype (ea_looter, ea_conscript_levy, ea_privateer, ea_war_captain) rather than inventing new named characters, per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 2: 9 rows added for map_d02/a01/d05 -- the last three maps in the maps tab without a scene. All three reuse archetypes whose own first_seen_map_id already points at these exact maps (ea_conscript_levy/d02, ea_looter/a01, ea_privateer/d05), the closest grounding this tab gets short of a named individual. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 3: 17 rows added fleshing out the 6 Act2 skeleton maps (v21/v22/c21/m21/m22/r16) into playable content. All reuse existing archetypes -- none of these six name a specific individual antagonist the way map_a02/a03 do -- per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 4: 22 rows added fleshing out the 10 Act3/paralogue skeleton maps into playable content. Act3's tougher tier is reflected by reusing ea_war_captain/ea_warlord (the miniboss/boss templates) throughout rather than Act1/2's commoner-tier mooks -- no new archetypes invented, same discipline as every prior addendum. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 5 (2026-10-03): added drop_weapon_id -- the weapon this enemy adds to the player's convoy when defeated, once per spawn_id per playthrough. Drafted: Act 1 non-trivial bosses drop a mid-tier weapon, Act 2+ bosses and the paralogues the high tier, and the two Billmen the halberd (the only way to get an overlap weapon). Nobody in the roster can wield a halberd yet (it needs cls_billman) -- it just waits in the convoy.</t>
         </is>
       </c>
     </row>
@@ -20094,7 +20212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="1" max="1"/>
@@ -20111,6 +20229,7 @@
     <col width="40" customWidth="1" style="18" min="12" max="12"/>
     <col width="14" customWidth="1" style="18" min="13" max="13"/>
     <col width="14" customWidth="1" style="18" min="14" max="14"/>
+    <col width="12" customWidth="1" style="18" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -20184,6 +20303,11 @@
           <t>effective_vs</t>
         </is>
       </c>
+      <c r="O1" s="26" t="inlineStr">
+        <is>
+          <t>convoy_qty</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -20227,6 +20351,9 @@
       <c r="K2" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
@@ -20270,6 +20397,9 @@
       <c r="K3" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
@@ -20313,6 +20443,9 @@
       <c r="K4" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -20356,6 +20489,9 @@
       <c r="K5" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -20399,6 +20535,9 @@
       <c r="K6" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
@@ -20442,6 +20581,9 @@
       <c r="K7" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
@@ -20485,6 +20627,9 @@
       <c r="K8" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="17" t="inlineStr">
@@ -20528,6 +20673,9 @@
       <c r="K9" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
@@ -20571,6 +20719,9 @@
       <c r="K10" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
@@ -20614,6 +20765,9 @@
       <c r="K11" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -20657,6 +20811,9 @@
       <c r="K12" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O12" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="17" t="inlineStr">
@@ -20700,6 +20857,9 @@
       <c r="K13" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
@@ -20743,6 +20903,9 @@
       <c r="K14" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
@@ -20786,6 +20949,9 @@
       <c r="K15" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O15" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
@@ -20829,6 +20995,9 @@
       <c r="K16" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="17" t="inlineStr">
@@ -20872,6 +21041,9 @@
       <c r="K17" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -20915,6 +21087,9 @@
       <c r="K18" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O18" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
@@ -20958,6 +21133,9 @@
       <c r="K19" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
@@ -21001,6 +21179,9 @@
       <c r="K20" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
@@ -21044,6 +21225,9 @@
       <c r="K21" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O21" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
@@ -21087,6 +21271,9 @@
       <c r="K22" s="17" t="n">
         <v>2</v>
       </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
@@ -21135,6 +21322,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
@@ -21183,6 +21373,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="17" t="inlineStr">
@@ -21231,6 +21424,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
@@ -21279,6 +21475,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="17" t="inlineStr">
@@ -21327,6 +21526,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
@@ -21375,6 +21577,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -21423,6 +21628,9 @@
           <t>Below Iron -- scavenged/broken-in gear, not a tuned tier like basic/mid/high.</t>
         </is>
       </c>
+      <c r="O29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -21471,15 +21679,18 @@
           <t>OVERLAP WEAPON (drafted 2026-10-02). Wielder needs BOTH axe and lance proficiency (req_arts) -- no class has that pair yet, cls_billman is the drafted one. Triangle-neutral (it hedges both faces, so no advantage and no penalty). Deliberately slow: weight 12 against a typical str of 7 costs 5 attack speed, so most wielders get doubled. Effective vs riding (might x2 in Combat.EFFECTIVE_MULT) -- the answer to cavalry that the plain triangle doesn't have.</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
+      <c r="M30" s="17" t="inlineStr">
         <is>
           <t>axe|lance</t>
         </is>
       </c>
-      <c r="N30" t="inlineStr">
+      <c r="N30" s="17" t="inlineStr">
         <is>
           <t>riding</t>
         </is>
+      </c>
+      <c r="O30" s="17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -21529,15 +21740,18 @@
           <t>OVERLAP WEAPON (drafted 2026-10-02). Needs axe AND brawl (cls_jaguar_knight today). Triangle-neutral. Heavy and inaccurate but hits hard; effective vs armor (heavy-armor movement type), the mirror of the halberd's anti-cavalry role.</t>
         </is>
       </c>
-      <c r="M31" t="inlineStr">
+      <c r="M31" s="17" t="inlineStr">
         <is>
           <t>axe|brawl</t>
         </is>
       </c>
-      <c r="N31" t="inlineStr">
+      <c r="N31" s="17" t="inlineStr">
         <is>
           <t>armor</t>
         </is>
+      </c>
+      <c r="O31" s="17" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="32">
@@ -21587,16 +21801,19 @@
           <t>OVERLAP WEAPON (drafted 2026-10-02). Needs reason AND faith (cls_miasma_warden today). Magic (mag/res), range 1-2, triangle-neutral. No effectiveness trait: its edge is that one weapon spans both magic arts. Attack speed burdens against mag, not str, like every magic weapon.</t>
         </is>
       </c>
-      <c r="M32" t="inlineStr">
+      <c r="M32" s="17" t="inlineStr">
         <is>
           <t>reason|faith</t>
         </is>
+      </c>
+      <c r="O32" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft weapons table, review before treating as canon. Covers ordinary equipment only -- forges/materials' 5 legendary drops (3-of-5 cap) are a separate system above this tier, per forges' own note that the common smith 'arms lances and axes: the common soldier's tools, not the officer's.' Three tiers per art (basic/mid/high, flavor-named Iron/Steel/Silver) x 7 arts = 21 weapons. Might/hit/crit/weight/uses follow the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises) -- this design's own stated lineage per PROJECT_HANDOFF.md, not sourced from anything in canon.xlsx. Range: melee arts (sword/lance/axe/brawl) = 1, bow = 2, reason/faith = 1-2 (standard FE magic range). Names are placeholder and mechanical on purpose (e.g. 'Iron Tome', 'Iron Rite') -- real flavor-naming consistent with the setting's Byzantine/Near-East register is a writing pass for later, not attempted here. No weapon-rank/proficiency gating system exists yet (who can use which tier) -- units' single art_primary/secondary per class implicitly limits which art a unit fights with, but nothing yet gates basic vs. mid vs. high within that art. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: 'worn' tier added below basic -- might 1, hit 55, one art each. Built for the prologue's conquered-army soldiers (enemy_archetypes.ea_conquered_soldier): veteran-level troops equipped with whatever's left after a siege, not a new balance tier anyone is meant to fight through progression. Numbers are a judgment call (roughly basic tier's might/hit at a fifth to two-thirds), not derived from anything in canon.xlsx. Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-09-25): crit calibration pass. This row's own text already said crit 'follows the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises)' but every weapon actually shipped with crit=0, flat across all 4 tiers -- never filled in despite the stated intent. Extended the same tier-scaling might/hit/weight/uses already use: worn=0, basic=0 (unchanged -- starter/scavenged gear staying crit-free matches genre convention), mid=5, high=10. Simulated the resulting crit_chance() output (weapon_crit + attacker.dex - defender.lck, this session's own 2026-09-25 formula calibration) against all 1,056 ordered unit/enemy attacker-defender combos per tier: basic/worn stays at the formula's own baseline (57.5% nonzero, mean 3.4%, max 21%); mid roughly doubles presence (86.8% nonzero, mean 7.1%, max 26%); high makes crit a real threat without ever approaching a coinflip (97.3% nonzero, mean 11.9%, max 31%, only 2 of 1,056 combos clear 30%). Kept the crit value uniform across all 7 arts, matching every other column on this table already being purely tier-based, not art-based -- nothing here or in canon.xlsx supports giving e.g. bows a crit edge over axes. ADDENDUM (2026-10-02): added req_arts (pipe-delimited arts a wielder must ALL be proficient in; blank = just the weapon's own art) and effective_vs (pipe-delimited movement types the weapon deals x2 might to), plus 3 overlap weapons (halberd, maul, censer). A weapon with 2+ req_arts is triangle-neutral. Attack speed = spd - max(0, weight - str) (mag for magic arts); a unit doubles at +4 speed. See combat.gd.</t>
+          <t>NOTE -- draft weapons table, review before treating as canon. Covers ordinary equipment only -- forges/materials' 5 legendary drops (3-of-5 cap) are a separate system above this tier, per forges' own note that the common smith 'arms lances and axes: the common soldier's tools, not the officer's.' Three tiers per art (basic/mid/high, flavor-named Iron/Steel/Silver) x 7 arts = 21 weapons. Might/hit/crit/weight/uses follow the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises) -- this design's own stated lineage per PROJECT_HANDOFF.md, not sourced from anything in canon.xlsx. Range: melee arts (sword/lance/axe/brawl) = 1, bow = 2, reason/faith = 1-2 (standard FE magic range). Names are placeholder and mechanical on purpose (e.g. 'Iron Tome', 'Iron Rite') -- real flavor-naming consistent with the setting's Byzantine/Near-East register is a writing pass for later, not attempted here. No weapon-rank/proficiency gating system exists yet (who can use which tier) -- units' single art_primary/secondary per class implicitly limits which art a unit fights with, but nothing yet gates basic vs. mid vs. high within that art. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: 'worn' tier added below basic -- might 1, hit 55, one art each. Built for the prologue's conquered-army soldiers (enemy_archetypes.ea_conquered_soldier): veteran-level troops equipped with whatever's left after a siege, not a new balance tier anyone is meant to fight through progression. Numbers are a judgment call (roughly basic tier's might/hit at a fifth to two-thirds), not derived from anything in canon.xlsx. Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-09-25): crit calibration pass. This row's own text already said crit 'follows the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises)' but every weapon actually shipped with crit=0, flat across all 4 tiers -- never filled in despite the stated intent. Extended the same tier-scaling might/hit/weight/uses already use: worn=0, basic=0 (unchanged -- starter/scavenged gear staying crit-free matches genre convention), mid=5, high=10. Simulated the resulting crit_chance() output (weapon_crit + attacker.dex - defender.lck, this session's own 2026-09-25 formula calibration) against all 1,056 ordered unit/enemy attacker-defender combos per tier: basic/worn stays at the formula's own baseline (57.5% nonzero, mean 3.4%, max 21%); mid roughly doubles presence (86.8% nonzero, mean 7.1%, max 26%); high makes crit a real threat without ever approaching a coinflip (97.3% nonzero, mean 11.9%, max 31%, only 2 of 1,056 combos clear 30%). Kept the crit value uniform across all 7 arts, matching every other column on this table already being purely tier-based, not art-based -- nothing here or in canon.xlsx supports giving e.g. bows a crit edge over axes. ADDENDUM (2026-10-02): added req_arts (pipe-delimited arts a wielder must ALL be proficient in; blank = just the weapon's own art) and effective_vs (pipe-delimited movement types the weapon deals x2 might to), plus 3 overlap weapons (halberd, maul, censer). A weapon with 2+ req_arts is triangle-neutral. Attack speed = spd - max(0, weight - str) (mag for magic arts); a unit doubles at +4 speed. See combat.gd. ADDENDUM 2 (2026-10-03): added convoy_qty -- how many of each weapon the shared convoy holds at the start of a playthrough (one mid-tier weapon per art; the overlap weapons start at 0 and arrive as drops). Every unit also starts with the basic weapon of its art (Equipment.ensure_loadout). `uses` is now spent: 1 per strike made, the weapon breaks at 0, no repair (map_f00's design note).</t>
         </is>
       </c>
     </row>
@@ -40355,7 +40572,7 @@
           <t>map_tp19</t>
         </is>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R17" s="17" t="inlineStr">
         <is>
           <t>wpn_halberd</t>
         </is>

</xml_diff>

<commit_message>
Add the Capture action and the capture deed
Units whose class carries classes.map_actions=capture (Gunnar's bounty hunter,
the Pardoner) can press C to take a weakened (<=50% HP), non-boss enemy alive:
no exchange, no drop, kill-level EXP, 25 gold ransom at the end of the map.
Each capture counts toward ep_capture, earned at epithets.count_needed (5).

Canon: epithets.count_needed, classes.map_actions, ep_capture tracked,
capture_hp_pct and income_per_capture parameters; validator checks.
Forecast shows a Capture line; barracks shows progress. test_capture (60).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -9184,7 +9184,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9194,6 +9194,7 @@
     <col width="14" customWidth="1" style="17" min="5" max="5"/>
     <col width="18" customWidth="1" style="17" min="6" max="6"/>
     <col width="10" customWidth="1" style="18" min="7" max="7"/>
+    <col width="14" customWidth="1" style="18" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -9232,6 +9233,11 @@
           <t>tracked</t>
         </is>
       </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>count_needed</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -9269,6 +9275,9 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -9306,6 +9315,9 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -9343,6 +9355,9 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="H4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -9380,6 +9395,9 @@
           <t>no</t>
         </is>
       </c>
+      <c r="H5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -9417,6 +9435,9 @@
           <t>no</t>
         </is>
       </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -9454,6 +9475,9 @@
           <t>no</t>
         </is>
       </c>
+      <c r="H7" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -9491,6 +9515,9 @@
           <t>no</t>
         </is>
       </c>
+      <c r="H8" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -9525,15 +9552,17 @@
       </c>
       <c r="G9" s="32" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+    </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection.</t>
+          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection. ADDENDUM (2026-10-07): count_needed = how many times a deed must be recorded before it is earned (1 for most; ep_capture 5). ep_capture is now tracked (the Capture action).</t>
         </is>
       </c>
     </row>
@@ -21880,7 +21909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="17" min="1" max="1"/>
@@ -21894,6 +21923,7 @@
     <col width="18" customWidth="1" style="17" min="9" max="9"/>
     <col width="30" customWidth="1" style="17" min="10" max="10"/>
     <col width="18" customWidth="1" style="18" min="11" max="11"/>
+    <col width="14" customWidth="1" style="18" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -21952,6 +21982,11 @@
           <t>unlock_map_id</t>
         </is>
       </c>
+      <c r="L1" s="21" t="inlineStr">
+        <is>
+          <t>map_actions</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -23666,6 +23701,11 @@
           <t>map_h33_mercy</t>
         </is>
       </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>capture</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="18">
       <c r="A37" s="23" t="inlineStr">
@@ -24096,6 +24136,11 @@
           <t>Gunnar; Capture + Shove mercy kit</t>
         </is>
       </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>capture</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="18">
       <c r="A46" s="23" t="inlineStr">
@@ -24608,7 +24653,7 @@
           <t>lv30+, deed-gated</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
+      <c r="K56" s="17" t="inlineStr">
         <is>
           <t>map_p_simurgh</t>
         </is>
@@ -33441,7 +33486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -33992,7 +34037,7 @@
           <t>prm_paragon_min_level</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="17" t="n">
         <v>30</v>
       </c>
       <c r="C36" s="17" t="n"/>
@@ -34008,7 +34053,7 @@
           <t>prm_paragon_deeds_required</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C37" s="17" t="n"/>
@@ -34024,7 +34069,7 @@
           <t>prm_paragon_fee_base</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="17" t="n">
         <v>1000</v>
       </c>
       <c r="C38" s="17" t="n"/>
@@ -34040,7 +34085,7 @@
           <t>prm_paragon_fee_per_level</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="17" t="n">
         <v>150</v>
       </c>
       <c r="C39" s="17" t="n"/>
@@ -34056,7 +34101,7 @@
           <t>prm_paragon_growth_bonus</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="17" t="n">
         <v>5</v>
       </c>
       <c r="C40" s="17" t="n"/>
@@ -34072,7 +34117,7 @@
           <t>prm_paragon_slots</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="17" t="n">
         <v>1</v>
       </c>
       <c r="C41" s="17" t="n"/>
@@ -34088,7 +34133,7 @@
           <t>prm_solo_hold_phases</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="17" t="n">
         <v>3</v>
       </c>
       <c r="C42" s="17" t="n"/>
@@ -34104,7 +34149,7 @@
           <t>prm_solo_hold_radius</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="17" t="n">
         <v>2</v>
       </c>
       <c r="C43" s="17" t="n"/>
@@ -34120,7 +34165,7 @@
           <t>prm_paragon_jump_hp</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="17" t="n">
         <v>5</v>
       </c>
       <c r="C44" s="17" t="n"/>
@@ -34136,7 +34181,7 @@
           <t>prm_paragon_jump_str</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="17" t="n">
         <v>4</v>
       </c>
       <c r="C45" s="17" t="n"/>
@@ -34152,7 +34197,7 @@
           <t>prm_paragon_jump_mag</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="17" t="n">
         <v>3</v>
       </c>
       <c r="C46" s="17" t="n"/>
@@ -34168,7 +34213,7 @@
           <t>prm_paragon_jump_dex</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="17" t="n">
         <v>4</v>
       </c>
       <c r="C47" s="17" t="n"/>
@@ -34184,7 +34229,7 @@
           <t>prm_paragon_jump_spd</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="17" t="n">
         <v>4</v>
       </c>
       <c r="C48" s="17" t="n"/>
@@ -34200,7 +34245,7 @@
           <t>prm_paragon_jump_lck</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="17" t="n">
         <v>3</v>
       </c>
       <c r="C49" s="17" t="n"/>
@@ -34216,7 +34261,7 @@
           <t>prm_paragon_jump_def</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="17" t="n">
         <v>4</v>
       </c>
       <c r="C50" s="17" t="n"/>
@@ -34232,7 +34277,7 @@
           <t>prm_paragon_jump_res</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="17" t="n">
         <v>3</v>
       </c>
       <c r="C51" s="17" t="n"/>
@@ -34245,7 +34290,39 @@
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds.</t>
+          <t>prm_capture_hp_pct</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C52" s="17" t="n"/>
+      <c r="D52" s="17" t="inlineStr">
+        <is>
+          <t>Capture: an enemy can be captured once its HP is at or below this percent of its maximum. Bosses cannot be captured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>prm_income_per_capture</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C53" s="17" t="n"/>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>Ransom: extra gold per enemy captured rather than defeated (a defeat is worth income_per_kill, so mercy pays better but drops no weapon).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Shove and Smite: a push action that upgrades on certification
S then an arrow key / click pushes an adjacent unit straight back: 1 tile for
Shove (Gunnar), 2 for Smite (Housecarl natively; Gunnar once certified). Walls,
the map edge and units stop it; bosses are never pushed; armor resists a tile.
Works on friends too, costs the action, deals no damage.

Canon: classes.map_actions gains shove/smite; shove_distance, smite_distance
and shove_armor_resist parameters. Barracks notes the upgrade. test_shove (48).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -9275,7 +9275,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9315,7 +9315,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9355,7 +9355,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9395,7 +9395,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9475,7 +9475,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9515,7 +9515,7 @@
           <t>no</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -9555,7 +9555,7 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="17" t="n">
         <v>5</v>
       </c>
     </row>
@@ -22851,6 +22851,11 @@
           <t>lv15+, pair-certified</t>
         </is>
       </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>smite</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="18">
       <c r="A20" s="23" t="inlineStr">
@@ -23701,7 +23706,7 @@
           <t>map_h33_mercy</t>
         </is>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L36" s="17" t="inlineStr">
         <is>
           <t>capture</t>
         </is>
@@ -24136,9 +24141,9 @@
           <t>Gunnar; Capture + Shove mercy kit</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>capture</t>
+      <c r="L45" s="17" t="inlineStr">
+        <is>
+          <t>capture|shove</t>
         </is>
       </c>
     </row>
@@ -33486,7 +33491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D54"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -34322,7 +34327,55 @@
     <row r="54">
       <c r="A54" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture).</t>
+          <t>prm_shove_distance</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" s="17" t="n"/>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>Shove (map action): tiles an adjacent unit is pushed straight away from the shover. Gunnar starts with this; it upgrades to Smite once he is certified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="17" t="inlineStr">
+        <is>
+          <t>prm_smite_distance</t>
+        </is>
+      </c>
+      <c r="B55" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" s="17" t="n"/>
+      <c r="D55" s="17" t="inlineStr">
+        <is>
+          <t>Smite (map action): the same push, one tile further. A class with 'smite' in classes.map_actions (the Housecarl) has it from the start; a shove unit gains it on certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="17" t="inlineStr">
+        <is>
+          <t>prm_shove_armor_resist</t>
+        </is>
+      </c>
+      <c r="B56" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C56" s="17" t="n"/>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>Tiles an armor-movement target resists a Shove/Smite (so a plain Shove cannot move armor at all, a Smite moves it one). Bosses are never pushed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add collision damage to Shove/Smite
A push that meets a wall, the map's edge or another unit collides: the pushed
unit takes a tenth of its own max HP (rounded down), and so does a unit it
hits. Never lethal (stops at 1 HP). A collision spends the action even when
nothing moves; armor resisting a push is not a collision. Enemies hurt by a
slam count as damaged by the pusher (boss single-combat deed).

Canon: promotion_rules.collision_pct = 10. test_shove now 72 checks.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -22851,7 +22851,7 @@
           <t>lv15+, pair-certified</t>
         </is>
       </c>
-      <c r="L19" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr">
         <is>
           <t>smite</t>
         </is>
@@ -33491,7 +33491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D57"/>
+  <dimension ref="A1:D58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -34375,7 +34375,23 @@
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist).</t>
+          <t>prm_collision_pct</t>
+        </is>
+      </c>
+      <c r="B57" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C57" s="17" t="n"/>
+      <c r="D57" s="17" t="inlineStr">
+        <is>
+          <t>Shove/Smite collision: a pushed unit that hits a wall, the map edge or another unit takes this percent of its own max HP (rounded down); a unit it hits takes the same of its own. Never lethal: it stops at 1 HP.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Kheldar's Bribe: pay to turn an adjacent enemy neutral
B then an arrow key / click on an adjacent enemy: 40 gold + 10 a level, one a
map, no bosses. A neutral enemy stops acting and can't be attacked or captured,
but stays put (it blocks, and can still be shoved). Not a kill or capture, so
it pays no income. Kheldar's Factor class gains map_actions=bribe.

Canon: bribe_cost_base, bribe_cost_per_level, bribe_per_map. test_bribe (39).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -24097,6 +24097,11 @@
           <t>Kheldar; end-map income, bribe one enemy to neutral</t>
         </is>
       </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>bribe</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="18">
       <c r="A45" s="23" t="inlineStr">
@@ -33491,7 +33496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -34391,7 +34396,55 @@
     <row r="58">
       <c r="A58" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage).</t>
+          <t>prm_bribe_cost_base</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="C58" s="17" t="n"/>
+      <c r="D58" s="17" t="inlineStr">
+        <is>
+          <t>Bribe (Kheldar's map action): gold base price to turn an adjacent enemy neutral for the rest of the map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>prm_bribe_cost_per_level</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C59" s="17" t="n"/>
+      <c r="D59" s="17" t="inlineStr">
+        <is>
+          <t>Bribe: extra gold per level of the enemy (a level-5 levy costs 90, a level-10 billman 140).</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>prm_bribe_per_map</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C60" s="17" t="n"/>
+      <c r="D60" s="17" t="inlineStr">
+        <is>
+          <t>Bribe: how many enemies Kheldar can turn per map (canon: 'bribe one enemy to neutral'). Bosses cannot be bribed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace the linear overworld with a walkable world map
Locations are nodes at canon coordinates (locations.map_x/map_y), world_paths
joins them, and the party marker walks the shortest chain of paths to wherever
you click. Chapters are placed at locations (chapters.location_id) and open as
you win others (chapters.unlock_after, any-of); Enter plays the next open
chapter where you stand. The Ur-Nashet prologue is a memory in the corner with
no road. Where the party stands is saved (GameState.world_location).

Canon: world_paths tab (38), location coordinates, chapter placement and
unlock chain; validator rule c07j. test_overworld (87).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -55,6 +55,7 @@
     <sheet name="supports" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="promotion_rules" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="abilities" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="world_paths" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -6373,7 +6374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L52"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="17" min="1" max="1"/>
@@ -6387,6 +6388,8 @@
     <col width="44" customWidth="1" style="17" min="10" max="10"/>
     <col width="16" customWidth="1" style="17" min="11" max="11"/>
     <col width="22" customWidth="1" style="17" min="12" max="12"/>
+    <col width="14" customWidth="1" style="18" min="13" max="13"/>
+    <col width="14" customWidth="1" style="18" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -6450,6 +6453,16 @@
           <t>teaches_system</t>
         </is>
       </c>
+      <c r="M1" s="21" t="inlineStr">
+        <is>
+          <t>location_id</t>
+        </is>
+      </c>
+      <c r="N1" s="21" t="inlineStr">
+        <is>
+          <t>unlock_after</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -6502,6 +6515,16 @@
           <t>positioning</t>
         </is>
       </c>
+      <c r="M2" s="17" t="inlineStr">
+        <is>
+          <t>loc_tally_house</t>
+        </is>
+      </c>
+      <c r="N2" s="17" t="inlineStr">
+        <is>
+          <t>ch_f00</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -6554,6 +6577,16 @@
           <t>green levies</t>
         </is>
       </c>
+      <c r="M3" s="17" t="inlineStr">
+        <is>
+          <t>loc_weighbridge</t>
+        </is>
+      </c>
+      <c r="N3" s="17" t="inlineStr">
+        <is>
+          <t>ch_d01</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -6606,6 +6639,16 @@
           <t>escort + cargo</t>
         </is>
       </c>
+      <c r="M4" s="17" t="inlineStr">
+        <is>
+          <t>loc_grain_road</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>ch_d02</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -6658,6 +6701,16 @@
           <t>terrain hazard</t>
         </is>
       </c>
+      <c r="M5" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_gate</t>
+        </is>
+      </c>
+      <c r="N5" s="17" t="inlineStr">
+        <is>
+          <t>ch_f00</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -6714,6 +6767,16 @@
           <t>talk / capture / disperse</t>
         </is>
       </c>
+      <c r="M6" s="17" t="inlineStr">
+        <is>
+          <t>loc_still_town</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>ch_a01</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -6768,6 +6831,16 @@
       <c r="L7" s="24" t="inlineStr">
         <is>
           <t>reinforcement pressure</t>
+        </is>
+      </c>
+      <c r="M7" s="17" t="inlineStr">
+        <is>
+          <t>loc_chapterhouse</t>
+        </is>
+      </c>
+      <c r="N7" s="17" t="inlineStr">
+        <is>
+          <t>ch_a02</t>
         </is>
       </c>
     </row>
@@ -6822,6 +6895,16 @@
           <t>the commission split</t>
         </is>
       </c>
+      <c r="M8" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>ch_d10|ch_a10</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -6876,6 +6959,16 @@
       <c r="L9" s="24" t="inlineStr">
         <is>
           <t>purchase objective</t>
+        </is>
+      </c>
+      <c r="M9" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="N9" s="17" t="inlineStr">
+        <is>
+          <t>ch_c21</t>
         </is>
       </c>
     </row>
@@ -6930,6 +7023,16 @@
           <t>boarding / grapple-dens</t>
         </is>
       </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>loc_salt_ford</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="inlineStr">
+        <is>
+          <t>ch_d04</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="23" t="inlineStr">
@@ -6982,6 +7085,11 @@
           <t>movement, terrain cost, weapon triangle</t>
         </is>
       </c>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t>loc_ur_nashet</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
@@ -7038,6 +7146,16 @@
           <t>no-talk chapters</t>
         </is>
       </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="inlineStr">
+        <is>
+          <t>ch_x11</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="23" t="inlineStr">
@@ -7094,6 +7212,16 @@
           <t>ritual defense</t>
         </is>
       </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>ch_v21</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="23" t="inlineStr">
@@ -7150,6 +7278,16 @@
           <t>home-front ambush</t>
         </is>
       </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_chapel</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>ch_v22|ch_m22</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -7206,6 +7344,16 @@
           <t>ongoing prophecy pressure</t>
         </is>
       </c>
+      <c r="M15" s="17" t="inlineStr">
+        <is>
+          <t>loc_lake_shore</t>
+        </is>
+      </c>
+      <c r="N15" s="17" t="inlineStr">
+        <is>
+          <t>ch_x11</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
@@ -7262,6 +7410,16 @@
           <t>archive standoff</t>
         </is>
       </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="inlineStr">
+        <is>
+          <t>ch_m21</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
@@ -7318,6 +7476,16 @@
           <t>redemption-as-purchase</t>
         </is>
       </c>
+      <c r="M17" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="inlineStr">
+        <is>
+          <t>ch_b15</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
@@ -7374,6 +7542,16 @@
           <t>consequences accumulate</t>
         </is>
       </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="inlineStr">
+        <is>
+          <t>ch_k22</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -7430,6 +7608,16 @@
           <t>the good ending still costs something</t>
         </is>
       </c>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>ch_e31</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
@@ -7486,6 +7674,16 @@
           <t>false godhood, assembled not born</t>
         </is>
       </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>ch_e31</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
@@ -7542,6 +7740,16 @@
           <t>conquest, not villainy</t>
         </is>
       </c>
+      <c r="M21" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="N21" s="17" t="inlineStr">
+        <is>
+          <t>ch_k22</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
@@ -7594,6 +7802,16 @@
           <t>the trial IS the system</t>
         </is>
       </c>
+      <c r="M22" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="N22" s="17" t="inlineStr">
+        <is>
+          <t>ch_h31</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
@@ -7650,6 +7868,16 @@
           <t>mercy has a bill too</t>
         </is>
       </c>
+      <c r="M23" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="N23" s="17" t="inlineStr">
+        <is>
+          <t>ch_h32</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
@@ -7706,6 +7934,16 @@
           <t>attrition, not spectacle</t>
         </is>
       </c>
+      <c r="M24" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="N24" s="17" t="inlineStr">
+        <is>
+          <t>ch_h32</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
@@ -7762,6 +8000,16 @@
           <t>the front keeps moving, there's no fixed line to hold</t>
         </is>
       </c>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>loc_glass_edge</t>
+        </is>
+      </c>
+      <c r="N25" s="17" t="inlineStr">
+        <is>
+          <t>ch_h34_war1</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
@@ -7818,6 +8066,16 @@
           <t>the cost lands on the world</t>
         </is>
       </c>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="N26" s="17" t="inlineStr">
+        <is>
+          <t>ch_h34_war2</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
@@ -7874,6 +8132,16 @@
           <t>a saint who will not judge</t>
         </is>
       </c>
+      <c r="M27" s="17" t="inlineStr">
+        <is>
+          <t>loc_north_wind</t>
+        </is>
+      </c>
+      <c r="N27" s="17" t="inlineStr">
+        <is>
+          <t>ch_a05|ch_d05</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="23" t="inlineStr">
@@ -7930,6 +8198,16 @@
           <t>a saint who will not judge</t>
         </is>
       </c>
+      <c r="M28" s="17" t="inlineStr">
+        <is>
+          <t>loc_hermit_lake</t>
+        </is>
+      </c>
+      <c r="N28" s="17" t="inlineStr">
+        <is>
+          <t>ch_a06|ch_d06</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -7985,6 +8263,16 @@
           <t>a pact that cannot be turned off</t>
         </is>
       </c>
+      <c r="M29" s="17" t="inlineStr">
+        <is>
+          <t>loc_lowest_terrace</t>
+        </is>
+      </c>
+      <c r="N29" s="17" t="inlineStr">
+        <is>
+          <t>ch_a06|ch_d06</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -8040,6 +8328,16 @@
           <t>help you cannot simply ask for</t>
         </is>
       </c>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>loc_simurgh_nest</t>
+        </is>
+      </c>
+      <c r="N30" s="17" t="inlineStr">
+        <is>
+          <t>ch_a05|ch_d05</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -8095,6 +8393,16 @@
           <t>a guardian whose terms are simple and absolute</t>
         </is>
       </c>
+      <c r="M31" s="17" t="inlineStr">
+        <is>
+          <t>loc_dove_colony</t>
+        </is>
+      </c>
+      <c r="N31" s="17" t="inlineStr">
+        <is>
+          <t>ch_a10|ch_d10</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
@@ -8150,6 +8458,16 @@
           <t>a pact you must be able to read to keep</t>
         </is>
       </c>
+      <c r="M32" s="17" t="inlineStr">
+        <is>
+          <t>loc_flats_interior</t>
+        </is>
+      </c>
+      <c r="N32" s="17" t="inlineStr">
+        <is>
+          <t>ch_x11</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
@@ -8205,6 +8523,16 @@
           <t>a blessing that was never yours to keep</t>
         </is>
       </c>
+      <c r="M33" s="17" t="inlineStr">
+        <is>
+          <t>loc_open_road</t>
+        </is>
+      </c>
+      <c r="N33" s="17" t="inlineStr">
+        <is>
+          <t>ch_x11</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
@@ -8260,6 +8588,16 @@
           <t>what a shrine is built to bury</t>
         </is>
       </c>
+      <c r="M34" s="17" t="inlineStr">
+        <is>
+          <t>loc_buried_works</t>
+        </is>
+      </c>
+      <c r="N34" s="17" t="inlineStr">
+        <is>
+          <t>ch_a10|ch_d10</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
@@ -8310,6 +8648,16 @@
           <t>defend under a deadline</t>
         </is>
       </c>
+      <c r="M35" s="17" t="inlineStr">
+        <is>
+          <t>loc_thessala</t>
+        </is>
+      </c>
+      <c r="N35" s="17" t="inlineStr">
+        <is>
+          <t>ch_d03</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
@@ -8360,6 +8708,16 @@
           <t>riding-blocked elevation</t>
         </is>
       </c>
+      <c r="M36" s="17" t="inlineStr">
+        <is>
+          <t>loc_anthe</t>
+        </is>
+      </c>
+      <c r="N36" s="17" t="inlineStr">
+        <is>
+          <t>ch_d05</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
@@ -8410,6 +8768,16 @@
           <t>a ruin with residents who are not the enemy</t>
         </is>
       </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>loc_stranded_harbour</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>ch_d06</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
@@ -8460,6 +8828,16 @@
           <t>no cover, no terrain to lean on</t>
         </is>
       </c>
+      <c r="M38" s="17" t="inlineStr">
+        <is>
+          <t>loc_dry_country</t>
+        </is>
+      </c>
+      <c r="N38" s="17" t="inlineStr">
+        <is>
+          <t>ch_d07</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
@@ -8510,6 +8888,16 @@
           <t>a chokepoint road, no fixed objective</t>
         </is>
       </c>
+      <c r="M39" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_road</t>
+        </is>
+      </c>
+      <c r="N39" s="17" t="inlineStr">
+        <is>
+          <t>ch_d08</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
@@ -8560,6 +8948,16 @@
           <t>a door that answers with force, not words</t>
         </is>
       </c>
+      <c r="M40" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="N40" s="17" t="inlineStr">
+        <is>
+          <t>ch_d09</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
@@ -8610,6 +9008,16 @@
           <t>a harbour trade, no crowd this time</t>
         </is>
       </c>
+      <c r="M41" s="17" t="inlineStr">
+        <is>
+          <t>loc_halder</t>
+        </is>
+      </c>
+      <c r="N41" s="17" t="inlineStr">
+        <is>
+          <t>ch_a03</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
@@ -8660,6 +9068,16 @@
           <t>a drowned landmark, walkable around it</t>
         </is>
       </c>
+      <c r="M42" s="17" t="inlineStr">
+        <is>
+          <t>loc_lake_shore</t>
+        </is>
+      </c>
+      <c r="N42" s="17" t="inlineStr">
+        <is>
+          <t>ch_a04</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -8710,6 +9128,16 @@
           <t>a frontier city, open approach</t>
         </is>
       </c>
+      <c r="M43" s="17" t="inlineStr">
+        <is>
+          <t>loc_ostrova</t>
+        </is>
+      </c>
+      <c r="N43" s="17" t="inlineStr">
+        <is>
+          <t>ch_a05</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
@@ -8760,6 +9188,16 @@
           <t>a cliff edge as a wall</t>
         </is>
       </c>
+      <c r="M44" s="17" t="inlineStr">
+        <is>
+          <t>loc_upper_scar</t>
+        </is>
+      </c>
+      <c r="N44" s="17" t="inlineStr">
+        <is>
+          <t>ch_a06</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
@@ -8810,6 +9248,16 @@
           <t>canopy blocks flight, ground fights normal</t>
         </is>
       </c>
+      <c r="M45" s="17" t="inlineStr">
+        <is>
+          <t>loc_timber_road</t>
+        </is>
+      </c>
+      <c r="N45" s="17" t="inlineStr">
+        <is>
+          <t>ch_a07</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
@@ -8860,6 +9308,16 @@
           <t>a shrine that keeps writing itself</t>
         </is>
       </c>
+      <c r="M46" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="N46" s="17" t="inlineStr">
+        <is>
+          <t>ch_a08</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
@@ -8910,6 +9368,16 @@
           <t>a loyalist home front, first contact</t>
         </is>
       </c>
+      <c r="M47" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_chapel</t>
+        </is>
+      </c>
+      <c r="N47" s="17" t="inlineStr">
+        <is>
+          <t>ch_a09</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
@@ -8965,6 +9433,16 @@
           <t>a home front, not a frontier</t>
         </is>
       </c>
+      <c r="M48" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="N48" s="17" t="inlineStr">
+        <is>
+          <t>ch_rf20</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
@@ -9020,6 +9498,16 @@
           <t>what a false godhood is actually made of</t>
         </is>
       </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="N49" s="17" t="inlineStr">
+        <is>
+          <t>ch_k21</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="17" t="inlineStr">
@@ -9070,6 +9558,16 @@
           <t>an ash crossing, no fixed foe</t>
         </is>
       </c>
+      <c r="M50" s="17" t="inlineStr">
+        <is>
+          <t>loc_cinder_track</t>
+        </is>
+      </c>
+      <c r="N50" s="17" t="inlineStr">
+        <is>
+          <t>ch_c21</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
@@ -9120,6 +9618,16 @@
           <t>a toll held by force, not by law</t>
         </is>
       </c>
+      <c r="M51" s="17" t="inlineStr">
+        <is>
+          <t>loc_throat_pass</t>
+        </is>
+      </c>
+      <c r="N51" s="17" t="inlineStr">
+        <is>
+          <t>ch_b15</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
@@ -9168,6 +9676,16 @@
       <c r="L52" s="17" t="inlineStr">
         <is>
           <t>what each side kept, what each side lost</t>
+        </is>
+      </c>
+      <c r="M52" s="17" t="inlineStr">
+        <is>
+          <t>loc_reunion_field</t>
+        </is>
+      </c>
+      <c r="N52" s="17" t="inlineStr">
+        <is>
+          <t>ch_tp19|ch_ct19</t>
         </is>
       </c>
     </row>
@@ -14006,7 +14524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="17" min="1" max="1"/>
@@ -14016,6 +14534,8 @@
     <col width="14" customWidth="1" style="17" min="5" max="5"/>
     <col width="12" customWidth="1" style="17" min="6" max="6"/>
     <col width="62" customWidth="1" style="17" min="7" max="7"/>
+    <col width="14" customWidth="1" style="18" min="8" max="8"/>
+    <col width="14" customWidth="1" style="18" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -14054,6 +14574,16 @@
           <t>what_the_ground_is_for</t>
         </is>
       </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>map_x</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>map_y</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -14091,6 +14621,12 @@
           <t>night docks, neutral porters; where the avatar starts as a clerk</t>
         </is>
       </c>
+      <c r="H2" s="17" t="n">
+        <v>450</v>
+      </c>
+      <c r="I2" s="17" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -14128,6 +14664,12 @@
           <t>hedgerow country; a requisition writ enforced on a reluctant house</t>
         </is>
       </c>
+      <c r="H3" s="17" t="n">
+        <v>545</v>
+      </c>
+      <c r="I3" s="17" t="n">
+        <v>335</v>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -14165,6 +14707,12 @@
           <t>bridge choke and a foot-only ford; wagons move 4</t>
         </is>
       </c>
+      <c r="H4" s="17" t="n">
+        <v>625</v>
+      </c>
+      <c r="I4" s="17" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -14202,6 +14750,12 @@
           <t>south coast; grain bought abroad, unloaded under protest</t>
         </is>
       </c>
+      <c r="H5" s="17" t="n">
+        <v>650</v>
+      </c>
+      <c r="I5" s="17" t="n">
+        <v>440</v>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -14239,6 +14793,12 @@
           <t>the rift crossed where it is shallow; the only southern crossing</t>
         </is>
       </c>
+      <c r="H6" s="17" t="n">
+        <v>540</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>420</v>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -14276,6 +14836,12 @@
           <t>a port stranded above its own water; three levels of street</t>
         </is>
       </c>
+      <c r="H7" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>435</v>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -14313,6 +14879,12 @@
           <t>ruin on the middle terrace; the renunciants live in it</t>
         </is>
       </c>
+      <c r="H8" s="17" t="n">
+        <v>210</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>365</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -14350,6 +14922,12 @@
           <t>open ground, no cover, the map that punishes slow armies</t>
         </is>
       </c>
+      <c r="H9" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>365</v>
+      </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="18">
       <c r="A10" s="23" t="inlineStr">
@@ -14387,6 +14965,12 @@
           <t>the single road east; lava fans narrow it to one lane in places</t>
         </is>
       </c>
+      <c r="H10" s="17" t="n">
+        <v>790</v>
+      </c>
+      <c r="I10" s="17" t="n">
+        <v>330</v>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="23" t="inlineStr">
@@ -14424,6 +15008,12 @@
           <t>the occupied seat; the Unstained will not talk to you</t>
         </is>
       </c>
+      <c r="H11" s="17" t="n">
+        <v>890</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <v>290</v>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="18">
       <c r="A12" s="23" t="inlineStr">
@@ -14461,6 +15051,12 @@
           <t>medicine cart to a gate; civilians chase it, looters follow</t>
         </is>
       </c>
+      <c r="H12" s="17" t="n">
+        <v>280</v>
+      </c>
+      <c r="I12" s="17" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="18">
       <c r="A13" s="23" t="inlineStr">
@@ -14498,6 +15094,12 @@
           <t>three streets of different widths; a preacher converting one a turn</t>
         </is>
       </c>
+      <c r="H13" s="17" t="n">
+        <v>350</v>
+      </c>
+      <c r="I13" s="17" t="n">
+        <v>170</v>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="18">
       <c r="A14" s="23" t="inlineStr">
@@ -14535,6 +15137,12 @@
           <t>escape map; relic hunters reinforce forever; a reliquary to take or give</t>
         </is>
       </c>
+      <c r="H14" s="17" t="n">
+        <v>440</v>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="18">
       <c r="A15" s="23" t="inlineStr">
@@ -14572,6 +15180,12 @@
           <t>north coast; exotic medicines bought from people who know it</t>
         </is>
       </c>
+      <c r="H15" s="17" t="n">
+        <v>400</v>
+      </c>
+      <c r="I15" s="17" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="16" ht="15" customHeight="1" s="18">
       <c r="A16" s="23" t="inlineStr">
@@ -14609,6 +15223,12 @@
           <t>the drowned town; a bell tower breaking the surface in dry years</t>
         </is>
       </c>
+      <c r="H16" s="17" t="n">
+        <v>520</v>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>80</v>
+      </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="18">
       <c r="A17" s="23" t="inlineStr">
@@ -14646,6 +15266,12 @@
           <t>steppe edge; the Assembly's eastern city, closer to the Plains than to Vetch</t>
         </is>
       </c>
+      <c r="H17" s="17" t="n">
+        <v>680</v>
+      </c>
+      <c r="I17" s="17" t="n">
+        <v>70</v>
+      </c>
     </row>
     <row r="18" ht="15" customHeight="1" s="18">
       <c r="A18" s="23" t="inlineStr">
@@ -14683,6 +15309,12 @@
           <t>escarpment fighting; the rift where it is still a cliff</t>
         </is>
       </c>
+      <c r="H18" s="17" t="n">
+        <v>770</v>
+      </c>
+      <c r="I18" s="17" t="n">
+        <v>135</v>
+      </c>
     </row>
     <row r="19" ht="15" customHeight="1" s="18">
       <c r="A19" s="23" t="inlineStr">
@@ -14720,6 +15352,12 @@
           <t>forest; the map where fliers are worthless and archers are not</t>
         </is>
       </c>
+      <c r="H19" s="17" t="n">
+        <v>690</v>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>190</v>
+      </c>
     </row>
     <row r="20" ht="15" customHeight="1" s="18">
       <c r="A20" s="23" t="inlineStr">
@@ -14757,6 +15395,12 @@
           <t>living prophecy; a sect that thinks revelation never stopped</t>
         </is>
       </c>
+      <c r="H20" s="17" t="n">
+        <v>580</v>
+      </c>
+      <c r="I20" s="17" t="n">
+        <v>175</v>
+      </c>
     </row>
     <row r="21" ht="15" customHeight="1" s="18">
       <c r="A21" s="23" t="inlineStr">
@@ -14794,6 +15438,12 @@
           <t>the court sect at home; obedience belongs to the throne</t>
         </is>
       </c>
+      <c r="H21" s="17" t="n">
+        <v>230</v>
+      </c>
+      <c r="I21" s="17" t="n">
+        <v>190</v>
+      </c>
     </row>
     <row r="22" ht="15" customHeight="1" s="18">
       <c r="A22" s="23" t="inlineStr">
@@ -14831,6 +15481,12 @@
           <t>largest map; whole army deployed once; two timed objectives, one force</t>
         </is>
       </c>
+      <c r="H22" s="17" t="n">
+        <v>600</v>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>230</v>
+      </c>
     </row>
     <row r="23" ht="15" customHeight="1" s="18">
       <c r="A23" s="23" t="inlineStr">
@@ -14868,6 +15524,12 @@
           <t>column A; ash underfoot, bad air, the Karkadann's country</t>
         </is>
       </c>
+      <c r="H23" s="17" t="n">
+        <v>830</v>
+      </c>
+      <c r="I23" s="17" t="n">
+        <v>400</v>
+      </c>
     </row>
     <row r="24" ht="15" customHeight="1" s="18">
       <c r="A24" s="23" t="inlineStr">
@@ -14905,6 +15567,12 @@
           <t>column B; prices rise every turn a fight is visible in the bazaar</t>
         </is>
       </c>
+      <c r="H24" s="17" t="n">
+        <v>1010</v>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>330</v>
+      </c>
     </row>
     <row r="25" ht="15" customHeight="1" s="18">
       <c r="A25" s="23" t="inlineStr">
@@ -14942,6 +15610,12 @@
           <t>column B; the road east, held by whoever taxes it this year</t>
         </is>
       </c>
+      <c r="H25" s="17" t="n">
+        <v>1060</v>
+      </c>
+      <c r="I25" s="17" t="n">
+        <v>430</v>
+      </c>
     </row>
     <row r="26" ht="15" customHeight="1" s="18">
       <c r="A26" s="23" t="inlineStr">
@@ -14979,6 +15653,12 @@
           <t>column A; straight-edged fused ground, nothing grows, nobody agrees why</t>
         </is>
       </c>
+      <c r="H26" s="17" t="n">
+        <v>780</v>
+      </c>
+      <c r="I26" s="17" t="n">
+        <v>480</v>
+      </c>
     </row>
     <row r="27" ht="15" customHeight="1" s="18">
       <c r="A27" s="23" t="inlineStr">
@@ -15016,6 +15696,12 @@
           <t>columns meet; whatever each lost is visible in what each brings</t>
         </is>
       </c>
+      <c r="H27" s="17" t="n">
+        <v>700</v>
+      </c>
+      <c r="I27" s="17" t="n">
+        <v>360</v>
+      </c>
     </row>
     <row r="28" ht="15" customHeight="1" s="18">
       <c r="A28" s="23" t="inlineStr">
@@ -15053,6 +15739,12 @@
           <t>the capital as a battlefield; the synod's colossus is fed from here</t>
         </is>
       </c>
+      <c r="H28" s="17" t="n">
+        <v>500</v>
+      </c>
+      <c r="I28" s="17" t="n">
+        <v>270</v>
+      </c>
     </row>
     <row r="29" ht="15" customHeight="1" s="18">
       <c r="A29" s="23" t="inlineStr">
@@ -15090,6 +15782,12 @@
           <t>the Simurgh; a foster-mother who answers whoever holds the feather</t>
         </is>
       </c>
+      <c r="H29" s="17" t="n">
+        <v>600</v>
+      </c>
+      <c r="I29" s="17" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="18">
       <c r="A30" s="23" t="inlineStr">
@@ -15127,6 +15825,12 @@
           <t>the Karkadann; it guards what it has decided to guard</t>
         </is>
       </c>
+      <c r="H30" s="17" t="n">
+        <v>930</v>
+      </c>
+      <c r="I30" s="17" t="n">
+        <v>435</v>
+      </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="18">
       <c r="A31" s="23" t="inlineStr">
@@ -15164,6 +15868,12 @@
           <t>the Anzu; arrows come apart, and it reads what you cannot</t>
         </is>
       </c>
+      <c r="H31" s="17" t="n">
+        <v>880</v>
+      </c>
+      <c r="I31" s="17" t="n">
+        <v>505</v>
+      </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="18">
       <c r="A32" s="23" t="inlineStr">
@@ -15201,6 +15911,12 @@
           <t>the Shadhavar; the song pulls the nearest enemy one tile a turn</t>
         </is>
       </c>
+      <c r="H32" s="17" t="n">
+        <v>190</v>
+      </c>
+      <c r="I32" s="17" t="n">
+        <v>470</v>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="18">
       <c r="A33" s="23" t="inlineStr">
@@ -15238,6 +15954,12 @@
           <t>the Huma; it never lands, so it belongs to a road, not a place</t>
         </is>
       </c>
+      <c r="H33" s="17" t="n">
+        <v>980</v>
+      </c>
+      <c r="I33" s="17" t="n">
+        <v>495</v>
+      </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="18">
       <c r="A34" s="23" t="inlineStr">
@@ -15275,6 +15997,12 @@
           <t>a hermit who refuses to adjudicate; fisher cult around him</t>
         </is>
       </c>
+      <c r="H34" s="17" t="n">
+        <v>105</v>
+      </c>
+      <c r="I34" s="17" t="n">
+        <v>410</v>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="18">
       <c r="A35" s="23" t="inlineStr">
@@ -15312,6 +16040,12 @@
           <t>the second hermit; likewise refuses</t>
         </is>
       </c>
+      <c r="H35" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="I35" s="17" t="n">
+        <v>45</v>
+      </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="18">
       <c r="A36" s="23" t="inlineStr">
@@ -15349,11 +16083,56 @@
           <t>records, complicit clerks, a shrine built over a facility</t>
         </is>
       </c>
-    </row>
+      <c r="H36" s="17" t="n">
+        <v>960</v>
+      </c>
+      <c r="I36" s="17" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="18">
-      <c r="A38" s="25" t="inlineStr">
-        <is>
-          <t>Comma-separated chapter numbers mean the ground is re-staged. Act 3 fights over Act 1's own fords and roads at army scale, so the player recognises the terrain they escorted a grain wagon across in chapter 3. 'P' = paralogue, unlocked through the supply network rather than the writ, so some stay dark in any given run. 34 locations against 30 chapters plus paralogues -- the world has the capacity, with room to cut.</t>
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>loc_ur_nashet</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Ur-Nashet, the last night (a memory)</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
+        <is>
+          <t>prologue</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>a flashback, 800 years early, in a city that no longer exists: not on the world map; the overworld draws it as a memory in the corner</t>
+        </is>
+      </c>
+      <c r="H38" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="I38" s="17" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="inlineStr">
+        <is>
+          <t>Comma-separated chapter numbers mean the ground is re-staged. Act 3 fights over Act 1's own fords and roads at army scale, so the player recognises the terrain they escorted a grain wagon across in chapter 3. 'P' = paralogue, unlocked through the supply network rather than the writ, so some stay dark in any given run. 34 locations against 30 chapters plus paralogues -- the world has the capacity, with room to cut. ADDENDUM (2026-10-11): map_x/map_y are overworld screen coordinates (a 1152x540 canvas, drafted: regions follow regions.direction, nothing is to scale); loc_ur_nashet is a flashback, not a place on the map.</t>
         </is>
       </c>
     </row>
@@ -24097,7 +24876,7 @@
           <t>Kheldar; end-map income, bribe one enemy to neutral</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" s="17" t="inlineStr">
         <is>
           <t>bribe</t>
         </is>
@@ -36588,6 +37367,1104 @@
       <c r="A42" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft ability table, review before treating as canon. pool is pipe-delimited tags a unit's class must match one of: 'any', 'art:&lt;art&gt;', 'move:&lt;movement&gt;', 'tier:&lt;tier&gt;', 'class:&lt;class_id&gt;'. cond: always | hp_full | hp_low (&lt;= half HP) | vs_&lt;movement&gt; (the foe's movement type) | art:&lt;art&gt; (the wielded weapon's art). Effects are flat: hit/avoid/crit/dodge points, dmg added to damage dealt, guard subtracted from damage taken, speed added to attack speed, exp_pct EXP percent. Passive combat effects only: canon's map-action skills (Shove, Steal, Refresh, Provoke...) need systems that don't exist. Slots come from promotion_rules (slots_*). Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): the six paragon signature skills (Astra, Deadeye, Fierce Iron Fist, Colossus, Stun, Corrosion) and Charge now also listed for the Bogatyr.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" style="18" min="1" max="1"/>
+    <col width="22" customWidth="1" style="18" min="2" max="2"/>
+    <col width="22" customWidth="1" style="18" min="3" max="3"/>
+    <col width="22" customWidth="1" style="18" min="4" max="4"/>
+    <col width="22" customWidth="1" style="18" min="5" max="5"/>
+    <col width="22" customWidth="1" style="18" min="6" max="6"/>
+    <col width="22" customWidth="1" style="18" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>path_id</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>from_location_id</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>to_location_id</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="E1" s="17" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="F1" s="17" t="inlineStr">
+        <is>
+          <t>waypoints</t>
+        </is>
+      </c>
+      <c r="G1" s="17" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>path_tally_house_weighbridge</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>loc_tally_house</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>loc_weighbridge</t>
+        </is>
+      </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>path_weighbridge_grain_road</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>loc_weighbridge</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>loc_grain_road</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>path_grain_road_thessala</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>loc_grain_road</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>loc_thessala</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>path_thessala_salt_ford</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>loc_thessala</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>loc_salt_ford</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>path_salt_ford_anthe</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>loc_salt_ford</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>loc_anthe</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>path_anthe_stranded_harbour</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>loc_anthe</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>loc_stranded_harbour</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>path_stranded_harbour_dry_country</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>loc_stranded_harbour</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>loc_dry_country</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>path_dry_country_vashti_road</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>loc_dry_country</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_road</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>520,392;690,392</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>path_vashti_road_vashti_gate</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_road</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
+        <is>
+          <t>diadem</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>path_vetch_gate_still_town</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_gate</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>loc_still_town</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>path_still_town_chapterhouse</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>loc_still_town</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>loc_chapterhouse</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>path_chapterhouse_halder</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>loc_chapterhouse</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>loc_halder</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>path_halder_lake_shore</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>loc_halder</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>loc_lake_shore</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>path_lake_shore_ostrova</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>loc_lake_shore</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>loc_ostrova</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>path_ostrova_upper_scar</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>loc_ostrova</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>loc_upper_scar</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>path_upper_scar_timber_road</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>loc_upper_scar</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>loc_timber_road</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>path_timber_road_march_shrine</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>loc_timber_road</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>path_march_shrine_vetch_chapel</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_chapel</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>path_vetch_chapel_vetch_gate</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_chapel</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>loc_vetch_gate</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
+        <is>
+          <t>assembly</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>path_tally_house_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>loc_tally_house</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>path_kaisareia_walls_muster_field</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>loc_kaisareia_walls</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>path_vashti_gate_muster_field</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>path_march_shrine_muster_field</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>loc_march_shrine</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>path_muster_field_cinder_track</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>loc_muster_field</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>loc_cinder_track</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>path_cinder_track_glass_edge</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>loc_cinder_track</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>loc_glass_edge</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>path_glass_edge_reunion_field</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>loc_glass_edge</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>loc_reunion_field</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>path_reunion_field_grain_road</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>loc_reunion_field</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>loc_grain_road</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>path_cinder_track_caravanserai</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>loc_cinder_track</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>path_caravanserai_throat_pass</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>loc_caravanserai</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>loc_throat_pass</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E30" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>path_throat_pass_glass_edge</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>loc_throat_pass</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>loc_glass_edge</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>path_lake_shore_simurgh_nest</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>loc_lake_shore</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>loc_simurgh_nest</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E32" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>path_halder_north_wind</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>loc_halder</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>loc_north_wind</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>path_cinder_track_dove_colony</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>loc_cinder_track</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>loc_dove_colony</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E34" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>path_vashti_gate_buried_works</t>
+        </is>
+      </c>
+      <c r="B35" s="17" t="inlineStr">
+        <is>
+          <t>loc_vashti_gate</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>loc_buried_works</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>path_glass_edge_flats_interior</t>
+        </is>
+      </c>
+      <c r="B36" s="17" t="inlineStr">
+        <is>
+          <t>loc_glass_edge</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>loc_flats_interior</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E36" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>path_anthe_lowest_terrace</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>loc_anthe</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>loc_lowest_terrace</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>path_stranded_harbour_hermit_lake</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>loc_stranded_harbour</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>loc_hermit_lake</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>path_throat_pass_open_road</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>loc_throat_pass</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>loc_open_road</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>trail</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>NOTE -- draft overworld paths (2026-10-11). The overworld is a graph, Super-Mario-World style: locations are nodes, each row here is a two-way path between two of them. The party walks the shortest chain of paths to any location you pick; a location with no path at all (the Ur-Nashet flashback) is reached by memory. route: diadem/assembly/both (how the line is drawn); kind: road/trail; waypoints: optional 'x,y;x,y' bends so a line doesn't cut through other places. Not to scale and not canon geography beyond regions.direction.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the miasma and delivery deeds, and cargo units for delivery
Miasma: a main unit that ends the player turn on miasma counts one; the deed is
earned at 5 (epithets.count_needed, deed_terrain = ter_miasma). Delivery needed
cargo: canon gains cargo_units and maps.cargo_needed (d03's three wagons, 2 to
deliver; a01's cart). On a cargo map only cargo delivers, enemies and hazards
hit it, losing too much loses the map, and units within 2 tiles of the goal
when a wagon arrives earn the deed. [W] selects the next cargo unit.

The barracks lists non-gating tracked deeds under 'Other deeds'. Validator
rule c07k. test_cargo_miasma (59).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -56,6 +56,7 @@
     <sheet name="promotion_rules" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="abilities" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="world_paths" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="cargo_units" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -9702,7 +9703,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9713,6 +9714,7 @@
     <col width="18" customWidth="1" style="17" min="6" max="6"/>
     <col width="10" customWidth="1" style="18" min="7" max="7"/>
     <col width="14" customWidth="1" style="18" min="8" max="8"/>
+    <col width="14" customWidth="1" style="18" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -9756,6 +9758,11 @@
           <t>count_needed</t>
         </is>
       </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>deed_terrain</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -9910,11 +9917,16 @@
       </c>
       <c r="G5" s="32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H5" s="17" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>ter_miasma</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
@@ -9950,7 +9962,7 @@
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H6" s="17" t="n">
@@ -10080,7 +10092,7 @@
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection. ADDENDUM (2026-10-07): count_needed = how many times a deed must be recorded before it is earned (1 for most; ep_capture 5). ep_capture is now tracked (the Capture action).</t>
+          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection. ADDENDUM (2026-10-07): count_needed = how many times a deed must be recorded before it is earned (1 for most; ep_capture 5). ep_capture is now tracked (the Capture action). ADDENDUM (2026-10-12): deed_terrain names the terrain_costs row a terrain deed counts turn-ends on (ep_miasma: ter_miasma, 5 times). ep_miasma and ep_delivery are now tracked; neither gates paragon (forge vocabulary only).</t>
         </is>
       </c>
     </row>
@@ -16090,7 +16102,6 @@
         <v>220</v>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="18">
       <c r="A38" s="17" t="inlineStr">
         <is>
@@ -34275,7 +34286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -35223,7 +35234,23 @@
     <row r="61">
       <c r="A61" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map).</t>
+          <t>prm_delivery_radius</t>
+        </is>
+      </c>
+      <c r="B61" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C61" s="17" t="n"/>
+      <c r="D61" s="17" t="inlineStr">
+        <is>
+          <t>ep_delivery: a unit 'escorts' a cargo unit if it is alive and within this many tiles of the goal when the cargo is delivered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius.</t>
         </is>
       </c>
     </row>
@@ -37645,7 +37672,7 @@
           <t>road</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>520,392;690,392</t>
         </is>
@@ -38462,7 +38489,7 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft overworld paths (2026-10-11). The overworld is a graph, Super-Mario-World style: locations are nodes, each row here is a two-way path between two of them. The party walks the shortest chain of paths to any location you pick; a location with no path at all (the Ur-Nashet flashback) is reached by memory. route: diadem/assembly/both (how the line is drawn); kind: road/trail; waypoints: optional 'x,y;x,y' bends so a line doesn't cut through other places. Not to scale and not canon geography beyond regions.direction.</t>
         </is>
@@ -38890,6 +38917,249 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="18" min="1" max="1"/>
+    <col width="18" customWidth="1" style="18" min="2" max="2"/>
+    <col width="18" customWidth="1" style="18" min="3" max="3"/>
+    <col width="18" customWidth="1" style="18" min="4" max="4"/>
+    <col width="18" customWidth="1" style="18" min="5" max="5"/>
+    <col width="18" customWidth="1" style="18" min="6" max="6"/>
+    <col width="18" customWidth="1" style="18" min="7" max="7"/>
+    <col width="18" customWidth="1" style="18" min="8" max="8"/>
+    <col width="18" customWidth="1" style="18" min="9" max="9"/>
+    <col width="18" customWidth="1" style="18" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>cargo_id</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>map_id</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
+      <c r="E1" s="26" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="F1" s="26" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="H1" s="26" t="inlineStr">
+        <is>
+          <t>spawn_row</t>
+        </is>
+      </c>
+      <c r="I1" s="26" t="inlineStr">
+        <is>
+          <t>spawn_col</t>
+        </is>
+      </c>
+      <c r="J1" s="26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cargo_d03_wagon1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>map_d03</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Grain wagon (north)</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>13</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>map_d03: escort 2 of 3 wagons, move 4 -- armor movement, so a wagon cannot take the foot-only ford</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cargo_d03_wagon2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>map_d03</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Grain wagon (centre)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I3" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cargo_d03_wagon3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>map_d03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Grain wagon (south)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>13</v>
+      </c>
+      <c r="I4" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cargo_a01_cart</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>map_a01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>The medicine cart</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>24</v>
+      </c>
+      <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>11</v>
+      </c>
+      <c r="I5" t="n">
+        <v>8</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>map_a01: the winter dole's cart; civilians chasing it aren't modelled</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>NOTE -- draft cargo units (2026-10-12). A cargo unit is a player-side unit that cannot fight and must be walked to its map's escort tile (the 'E' symbol); delivering one is what the escort objective now means on a map with cargo (maps.cargo_needed delivered to win; if too few remain alive the map is lost) and what ep_delivery counts. Wagon and cart stats are first-pass guesses. d03's 'escort 2 of 3' is canon; the cart's hp and the wagons' defence are mine.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -40801,7 +41071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R53"/>
+  <dimension ref="A1:S53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="17" min="1" max="1"/>
@@ -40820,6 +41090,7 @@
     <col width="22" customWidth="1" style="17" min="16" max="16"/>
     <col width="12" customWidth="1" style="17" min="17" max="17"/>
     <col width="28" customWidth="1" style="17" min="18" max="18"/>
+    <col width="14" customWidth="1" style="18" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -40913,6 +41184,11 @@
           <t>approaches</t>
         </is>
       </c>
+      <c r="S1" s="21" t="inlineStr">
+        <is>
+          <t>cargo_needed</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -41129,6 +41405,9 @@
           <t>bridge choke|southern ford (foot only)|north bank escort line</t>
         </is>
       </c>
+      <c r="S4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -41200,6 +41479,9 @@
         <is>
           <t>the dole road|the ice (risky, fast)</t>
         </is>
+      </c>
+      <c r="S5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">

</xml_diff>

<commit_message>
Add the dispersal and talk deeds: routing levies and the Talk action
Routing: enemy_archetypes.flees_below_pct (50 for the conscript levy, per
map_d02's note) makes a non-boss below that HP break in the enemy phase and run
for the map edge; reaching it takes it off the field unkilled. Whoever dealt the
blow that broke it is credited; 3 routs earn ep_dispersal.

Talk: T then an arrow / click on an adjacent enemy rolls a chance (40 + 3 Lck +
2 per level gap + the enemy's talk_mod, 5-95%). A yielded enemy leaves unharmed
with its talk_line, pays 20 gold and earns ep_talk; a boss that yields ends a
defend map (Boyan's 'answer' path). A failure spends the action and that enemy
stops listening. Income now pays 10 a rout and 20 a talk.

Canon: flees_below_pct / talk_mod / talk_line, talk and income parameters,
validator rule c07l. test_dispersal_talk (62).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -9923,7 +9923,7 @@
       <c r="H5" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>ter_miasma</t>
         </is>
@@ -10002,11 +10002,11 @@
       </c>
       <c r="G7" s="32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H7" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
@@ -10042,7 +10042,7 @@
       </c>
       <c r="G8" s="32" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="H8" s="17" t="n">
@@ -10092,7 +10092,7 @@
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection. ADDENDUM (2026-10-07): count_needed = how many times a deed must be recorded before it is earned (1 for most; ep_capture 5). ep_capture is now tracked (the Capture action). ADDENDUM (2026-10-12): deed_terrain names the terrain_costs row a terrain deed counts turn-ends on (ep_miasma: ter_miasma, 5 times). ep_miasma and ep_delivery are now tracked; neither gates paragon (forge vocabulary only).</t>
+          <t>Pure performance telemetry, no rubber-banding. Feeds Paragon gating, forge vocabulary, Venerated evidence, boss pre-battle screens, and the deputy selection. ADDENDUM (2026-10-07): count_needed = how many times a deed must be recorded before it is earned (1 for most; ep_capture 5). ep_capture is now tracked (the Capture action). ADDENDUM (2026-10-12): deed_terrain names the terrain_costs row a terrain deed counts turn-ends on (ep_miasma: ter_miasma, 5 times). ep_miasma and ep_delivery are now tracked; neither gates paragon (forge vocabulary only). ADDENDUM (2026-10-13): ep_dispersal (3 levies routed) and ep_talk (1 enemy talked down) are now tracked; neither gates paragon.</t>
         </is>
       </c>
     </row>
@@ -34286,7 +34286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D62"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -35250,7 +35250,119 @@
     <row r="62">
       <c r="A62" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius.</t>
+          <t>prm_talk_base</t>
+        </is>
+      </c>
+      <c r="B62" s="17" t="n">
+        <v>40</v>
+      </c>
+      <c r="C62" s="17" t="n"/>
+      <c r="D62" s="17" t="inlineStr">
+        <is>
+          <t>Talk (map action): base chance in percent that an adjacent talkable enemy yields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>prm_talk_lck</t>
+        </is>
+      </c>
+      <c r="B63" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" s="17" t="n"/>
+      <c r="D63" s="17" t="inlineStr">
+        <is>
+          <t>Talk: + this many percent per point of the speaker's Lck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="17" t="inlineStr">
+        <is>
+          <t>prm_talk_level</t>
+        </is>
+      </c>
+      <c r="B64" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C64" s="17" t="n"/>
+      <c r="D64" s="17" t="inlineStr">
+        <is>
+          <t>Talk: + this many percent per level the speaker is above the enemy (minus per level below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="17" t="inlineStr">
+        <is>
+          <t>prm_talk_min</t>
+        </is>
+      </c>
+      <c r="B65" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C65" s="17" t="n"/>
+      <c r="D65" s="17" t="inlineStr">
+        <is>
+          <t>Talk: the chance never drops below this percent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>prm_talk_max</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="n">
+        <v>95</v>
+      </c>
+      <c r="C66" s="17" t="n"/>
+      <c r="D66" s="17" t="inlineStr">
+        <is>
+          <t>Talk: the chance never rises above this percent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>prm_income_per_rout</t>
+        </is>
+      </c>
+      <c r="B67" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="C67" s="17" t="n"/>
+      <c r="D67" s="17" t="inlineStr">
+        <is>
+          <t>Extra gold per enemy that fled the field (routed) rather than being defeated, captured or talked down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>prm_income_per_talk</t>
+        </is>
+      </c>
+      <c r="B68" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C68" s="17" t="n"/>
+      <c r="D68" s="17" t="inlineStr">
+        <is>
+          <t>Extra gold per enemy talked down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates.</t>
         </is>
       </c>
     </row>
@@ -38994,165 +39106,165 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>cargo_d03_wagon1</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>map_d03</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>Grain wagon (north)</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>armor</t>
         </is>
       </c>
-      <c r="E2" t="n">
+      <c r="E2" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="17" t="inlineStr">
         <is>
           <t>map_d03: escort 2 of 3 wagons, move 4 -- armor movement, so a wagon cannot take the foot-only ford</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>cargo_d03_wagon2</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>map_d03</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>Grain wagon (centre)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>armor</t>
         </is>
       </c>
-      <c r="E3" t="n">
+      <c r="E3" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="17" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>cargo_d03_wagon3</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>map_d03</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Grain wagon (south)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>armor</t>
         </is>
       </c>
-      <c r="E4" t="n">
+      <c r="E4" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" s="17" t="n">
         <v>13</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="17" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>cargo_a01_cart</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>map_a01</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>The medicine cart</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>armor</t>
         </is>
       </c>
-      <c r="E5" t="n">
+      <c r="E5" s="17" t="n">
         <v>24</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" s="17" t="n">
         <v>11</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>map_a01: the winter dole's cart; civilians chasing it aren't modelled</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft cargo units (2026-10-12). A cargo unit is a player-side unit that cannot fight and must be walked to its map's escort tile (the 'E' symbol); delivering one is what the escort objective now means on a map with cargo (maps.cargo_needed delivered to win; if too few remain alive the map is lost) and what ep_delivery counts. Wagon and cart stats are first-pass guesses. d03's 'escort 2 of 3' is canon; the cart's hp and the wagons' defence are mine.</t>
         </is>
@@ -41405,7 +41517,7 @@
           <t>bridge choke|southern ford (foot only)|north bank escort line</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="S4" s="17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -41480,7 +41592,7 @@
           <t>the dole road|the ice (risky, fast)</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="S5" s="17" t="n">
         <v>1</v>
       </c>
     </row>
@@ -44775,7 +44887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R18"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="18" min="1" max="1"/>
@@ -44795,6 +44907,9 @@
     <col width="55" customWidth="1" style="18" min="15" max="15"/>
     <col width="14" customWidth="1" style="18" min="16" max="16"/>
     <col width="16" customWidth="1" style="18" min="18" max="18"/>
+    <col width="14" customWidth="1" style="18" min="19" max="19"/>
+    <col width="14" customWidth="1" style="18" min="20" max="20"/>
+    <col width="40" customWidth="1" style="18" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -44888,6 +45003,21 @@
           <t>weapon_id</t>
         </is>
       </c>
+      <c r="S1" s="26" t="inlineStr">
+        <is>
+          <t>flees_below_pct</t>
+        </is>
+      </c>
+      <c r="T1" s="26" t="inlineStr">
+        <is>
+          <t>talk_mod</t>
+        </is>
+      </c>
+      <c r="U1" s="26" t="inlineStr">
+        <is>
+          <t>talk_line</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -44957,6 +45087,14 @@
           <t>map_f00</t>
         </is>
       </c>
+      <c r="T2" t="n">
+        <v>30</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>We were told it was a drill. ... It isn't, is it.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
@@ -45026,6 +45164,17 @@
           <t>map_d02</t>
         </is>
       </c>
+      <c r="S3" t="n">
+        <v>50</v>
+      </c>
+      <c r="T3" t="n">
+        <v>20</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>I never wanted this spear. Tell them you never saw me.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
@@ -45566,6 +45715,14 @@
           <t>map_a02</t>
         </is>
       </c>
+      <c r="T11" t="n">
+        <v>-10</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>You answered the still night, and the night answers you. Go on, then.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="17" t="inlineStr">
@@ -45989,7 +46146,7 @@
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft enemy archetypes, review before treating as canon. These are the only enemy TYPES actually named anywhere in canon.xlsx (scattered across maps.design_note for d02/a01/a02/a03, plus f00's own garrison) -- this tab just gives them mechanical stats, it does not invent new enemy types. Stats reuse unit_base_stats' exact tier baselines (commoner/trained) rather than new numbers, so a generic enemy naturally reads as somewhat weaker than an average player unit of the same tier -- player units get baseline + a growth_profile-derived bonus, these get baseline alone, with no growth_profile to add from since they're static mooks, not growing units. ea_garrison is the one deliberate exception: knocked further below even the commoner floor because 'fatigued and not a threat' is explicit design language, not just tier-average. weapon_art is stored directly (not derived via a base_class_id lookup) since 'commoner' tier classes have no art_primary in the classes tab -- same reason prologue_roster carries movement_type directly instead of relying solely on a class link. No per-chapter difficulty scaling exists yet (these are flat reference stats at each archetype's tier baseline level, not tuned per-map); that's a separate system for whenever real encounters get built. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: ea_privateer added for map_d05, the only other place canon.xlsx names a distinct enemy identity (weapon_art/movement_type are invented -- 'boards' implies melee, nothing pins down which art or foot-vs-other -- everything else reuses the trained-tier baseline like ea_relic_hunter). map_b15's 'green levies' are the same call already made for map_a02 in ea_conscript_levy's own note above -- not a new archetype. map_d01/d03/x11 name no enemy identity at all in their design_note text, so nothing to ground a new row in there yet. Drafted by a Claude Code session, 2026-09-16. ADDENDUM 2: ea_conquered_soldier, ea_hardened_veteran, ea_war_captain, and ea_warlord added per a direct request for a prologue-soldier archetype plus generic sidequest/miniboss/boss power-tier templates. These break from the rest of this tab in two ways, both explained on each row's own behavior text: (1) they're the first rows using the new weapon_tier column (worn/mid/high instead of every prior row's implicit basic) and (2) three of the four (hardened_veteran/war_captain/warlord) have no first_seen_map_id -- they're reusable templates, not tied to any written encounter, unlike every other row in this tab so far. Drafted by a Claude Code session, 2026-09-16. ADDENDUM 3: ea_preacher_boyan (map_a02) and ea_relic_hunter_captain (map_a03) added -- the first named-individual reskins of the generic sidequest/miniboss templates, tied to a specific map the way the original 5 rows are (unlike ADDENDUM 2's three unassigned templates). Both rows' own behavior text spells out exactly what's grounded (the map/chapter design_notes, recruit rosters, force-deploys) versus invented (names, exact stat tuning, and one speculative narrative thread on the a03 row explicitly flagged as unconfirmed). Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-10-02): added weapon_id (optional: blank means wpn_&lt;weapon_art&gt;_&lt;weapon_tier&gt;; set it for overlap weapons whose id doesn't follow that pattern) and ea_billman, the first archetype with an overlap weapon.</t>
+          <t>NOTE -- draft enemy archetypes, review before treating as canon. These are the only enemy TYPES actually named anywhere in canon.xlsx (scattered across maps.design_note for d02/a01/a02/a03, plus f00's own garrison) -- this tab just gives them mechanical stats, it does not invent new enemy types. Stats reuse unit_base_stats' exact tier baselines (commoner/trained) rather than new numbers, so a generic enemy naturally reads as somewhat weaker than an average player unit of the same tier -- player units get baseline + a growth_profile-derived bonus, these get baseline alone, with no growth_profile to add from since they're static mooks, not growing units. ea_garrison is the one deliberate exception: knocked further below even the commoner floor because 'fatigued and not a threat' is explicit design language, not just tier-average. weapon_art is stored directly (not derived via a base_class_id lookup) since 'commoner' tier classes have no art_primary in the classes tab -- same reason prologue_roster carries movement_type directly instead of relying solely on a class link. No per-chapter difficulty scaling exists yet (these are flat reference stats at each archetype's tier baseline level, not tuned per-map); that's a separate system for whenever real encounters get built. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: ea_privateer added for map_d05, the only other place canon.xlsx names a distinct enemy identity (weapon_art/movement_type are invented -- 'boards' implies melee, nothing pins down which art or foot-vs-other -- everything else reuses the trained-tier baseline like ea_relic_hunter). map_b15's 'green levies' are the same call already made for map_a02 in ea_conscript_levy's own note above -- not a new archetype. map_d01/d03/x11 name no enemy identity at all in their design_note text, so nothing to ground a new row in there yet. Drafted by a Claude Code session, 2026-09-16. ADDENDUM 2: ea_conquered_soldier, ea_hardened_veteran, ea_war_captain, and ea_warlord added per a direct request for a prologue-soldier archetype plus generic sidequest/miniboss/boss power-tier templates. These break from the rest of this tab in two ways, both explained on each row's own behavior text: (1) they're the first rows using the new weapon_tier column (worn/mid/high instead of every prior row's implicit basic) and (2) three of the four (hardened_veteran/war_captain/warlord) have no first_seen_map_id -- they're reusable templates, not tied to any written encounter, unlike every other row in this tab so far. Drafted by a Claude Code session, 2026-09-16. ADDENDUM 3: ea_preacher_boyan (map_a02) and ea_relic_hunter_captain (map_a03) added -- the first named-individual reskins of the generic sidequest/miniboss templates, tied to a specific map the way the original 5 rows are (unlike ADDENDUM 2's three unassigned templates). Both rows' own behavior text spells out exactly what's grounded (the map/chapter design_notes, recruit rosters, force-deploys) versus invented (names, exact stat tuning, and one speculative narrative thread on the a03 row explicitly flagged as unconfirmed). Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-10-02): added weapon_id (optional: blank means wpn_&lt;weapon_art&gt;_&lt;weapon_tier&gt;; set it for overlap weapons whose id doesn't follow that pattern) and ea_billman, the first archetype with an overlap weapon. ADDENDUM (2026-10-13): flees_below_pct = the HP percent below which a non-boss of this type routs (blank = never; the conscript levy, per map_d02's own note). talk_mod = how receptive it is to being talked down (blank = cannot be talked to; added to the speaker's chance), talk_line = what it says when it yields. Both are first-pass guesses.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add the Krivis, a drafted faith paragon class
Canon's paragon list had a class for every art but faith, so no faith unit could
take the second tier. cls_krivis (Baltic, faith art, infantry) fills the gap with
the signature skill Verdict (ab_verdict: +6 hit, +6 avoid, +4 dodge, +3 guard).
The engine already offered paragons by art, so faith units, and hybrids with a
faith second art, now see it. Tests that asserted 'faith has no paragon class'
now check the Krivis end to end.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -22699,7 +22699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="17" min="1" max="1"/>
@@ -25462,61 +25462,110 @@
     <row r="57">
       <c r="A57" s="23" t="inlineStr">
         <is>
+          <t>cls_krivis</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>Krivis</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="inlineStr">
+        <is>
+          <t>paragon</t>
+        </is>
+      </c>
+      <c r="D57" s="23" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="E57" s="23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F57" s="23" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="G57" s="23" t="n"/>
+      <c r="H57" s="23" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="I57" s="23" t="inlineStr">
+        <is>
+          <t>Baltic</t>
+        </is>
+      </c>
+      <c r="J57" s="23" t="inlineStr">
+        <is>
+          <t>lv30+, deed-gated. ADDED 2026-10-14 to fill the faith gap: canon's paragon list (Bogatyr, Fianna, Donso, Toa, Jaguar knight, Eagle knight, Tzitzimitl) had no faith class, so no faith unit could take the paragon tier. The Krivis is the Baltic high priest, a judge as much as a priest -- the paragon of a faith that rules on the dead and the living, set against the hermits' refusal to adjudicate. Name, culture, infantry movement and the signature skill are all drafted; none is setting canon.</t>
+        </is>
+      </c>
+      <c r="K57" s="17" t="n"/>
+    </row>
+    <row r="58" ht="15" customHeight="1" s="18">
+      <c r="A58" s="23" t="inlineStr">
+        <is>
           <t>cls_billman</t>
         </is>
       </c>
-      <c r="B57" s="23" t="inlineStr">
+      <c r="B58" s="23" t="inlineStr">
         <is>
           <t>Billman</t>
         </is>
       </c>
-      <c r="C57" s="23" t="inlineStr">
+      <c r="C58" s="23" t="inlineStr">
         <is>
           <t>hybrid</t>
         </is>
       </c>
-      <c r="D57" s="23" t="inlineStr">
+      <c r="D58" s="23" t="inlineStr">
         <is>
           <t>axe</t>
         </is>
       </c>
-      <c r="E57" s="23" t="inlineStr">
+      <c r="E58" s="23" t="inlineStr">
         <is>
           <t>lance</t>
         </is>
       </c>
-      <c r="F57" s="23" t="inlineStr">
+      <c r="F58" s="23" t="inlineStr">
         <is>
           <t>infantry</t>
         </is>
       </c>
-      <c r="G57" s="23" t="inlineStr">
+      <c r="G58" s="23" t="inlineStr">
         <is>
           <t>cls_tr_axe</t>
         </is>
       </c>
-      <c r="H57" s="23" t="n"/>
-      <c r="I57" s="23" t="inlineStr">
+      <c r="H58" s="23" t="n"/>
+      <c r="I58" s="23" t="inlineStr">
         <is>
           <t>setting-new</t>
         </is>
       </c>
-      <c r="J57" s="23" t="inlineStr">
+      <c r="J58" s="23" t="inlineStr">
         <is>
           <t>DRAFTED, not placed on any unit. The axe+lance pair the halberd needs (weapons.wpn_halberd req_arts) -- no existing class has it. Added 2026-10-02 so the overlap-weapon proficiency rule has a wielder; the first user is the enemy archetype ea_billman.</t>
         </is>
       </c>
-      <c r="K57" s="17" t="inlineStr">
+      <c r="K58" s="17" t="inlineStr">
         <is>
           <t>map_tp19</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="15" customHeight="1" s="18"/>
-    <row r="59">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>Deliberate permanent gaps: brawl+riding, brawl+flying. reason+flying is a founded gap (broken by paralogue into Tzitzimitl). Galeforce permanently banned. ADDENDUM (2026-10-05): added unlock_map_id -- a hybrid class is not offered at certification until the player has won that map (drafted, thematic: Billman = Throat Pass where the halberd-bearers stand; Ferryman = the Drowned March's lake; Pardoner = the mercy chapter; Ash Ascetic = the Stepped Coast's lake; Miasma Warden = the Dove Colony). Blank for every non-hybrid class. ADDENDUM (2026-10-06): the paragon tier is built. A unit that is certified, level 30+, has earned a paragon-gating epithet and can pay the fee may take a paragon class whose primary art it already knows; Tzitzimitl (the founded gap) also needs map_p_simurgh won (drafted guess: the flying paralogue). Faith has no paragon class -- a gap left for you to decide, not invented. unlock_map_id now applies to hybrid and paragon tiers.</t>
+    <row r="59"/>
+    <row r="60">
+      <c r="A60" s="25" t="inlineStr">
+        <is>
+          <t>Deliberate permanent gaps: brawl+riding, brawl+flying. reason+flying is a founded gap (broken by paralogue into Tzitzimitl). Galeforce permanently banned. ADDENDUM (2026-10-05): added unlock_map_id -- a hybrid class is not offered at certification until the player has won that map (drafted, thematic: Billman = Throat Pass where the halberd-bearers stand; Ferryman = the Drowned March's lake; Pardoner = the mercy chapter; Ash Ascetic = the Stepped Coast's lake; Miasma Warden = the Dove Colony). Blank for every non-hybrid class. ADDENDUM (2026-10-06): the paragon tier is built. A unit that is certified, level 30+, has earned a paragon-gating epithet and can pay the fee may take a paragon class whose primary art it already knows; Tzitzimitl (the founded gap) also needs map_p_simurgh won (drafted guess: the flying paralogue). Faith has no paragon class -- a gap left for you to decide, not invented. unlock_map_id now applies to hybrid and paragon tiers. ADDENDUM (2026-10-14): cls_krivis (Baltic) is a drafted faith paragon, filling the one art that had none.</t>
         </is>
       </c>
     </row>
@@ -35377,7 +35426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M42"/>
+  <dimension ref="A1:M43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="18" min="1" max="1"/>
@@ -37504,6 +37553,57 @@
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>ab_verdict</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>class:cls_krivis</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="17" t="inlineStr">
+        <is>
+          <t>Drafted signature skill for the Krivis (the judge-priest): a passive approximation of a ruling nothing gets past -- steady aim, harder to hit, softer blows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft ability table, review before treating as canon. pool is pipe-delimited tags a unit's class must match one of: 'any', 'art:&lt;art&gt;', 'move:&lt;movement&gt;', 'tier:&lt;tier&gt;', 'class:&lt;class_id&gt;'. cond: always | hp_full | hp_low (&lt;= half HP) | vs_&lt;movement&gt; (the foe's movement type) | art:&lt;art&gt; (the wielded weapon's art). Effects are flat: hit/avoid/crit/dodge points, dmg added to damage dealt, guard subtracted from damage taken, speed added to attack speed, exp_pct EXP percent. Passive combat effects only: canon's map-action skills (Shove, Steal, Refresh, Provoke...) need systems that don't exist. Slots come from promotion_rules (slots_*). Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): the six paragon signature skills (Astra, Deadeye, Fierce Iron Fist, Colossus, Stun, Corrosion) and Charge now also listed for the Bogatyr.</t>
         </is>
@@ -45087,10 +45187,10 @@
           <t>map_f00</t>
         </is>
       </c>
-      <c r="T2" t="n">
+      <c r="T2" s="17" t="n">
         <v>30</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="17" t="inlineStr">
         <is>
           <t>We were told it was a drill. ... It isn't, is it.</t>
         </is>
@@ -45164,13 +45264,13 @@
           <t>map_d02</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="S3" s="17" t="n">
         <v>50</v>
       </c>
-      <c r="T3" t="n">
+      <c r="T3" s="17" t="n">
         <v>20</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U3" s="17" t="inlineStr">
         <is>
           <t>I never wanted this spear. Tell them you never saw me.</t>
         </is>
@@ -45715,10 +45815,10 @@
           <t>map_a02</t>
         </is>
       </c>
-      <c r="T11" t="n">
+      <c r="T11" s="17" t="n">
         <v>-10</v>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U11" s="17" t="inlineStr">
         <is>
           <t>You answered the still night, and the night answers you. Go on, then.</t>
         </is>

</xml_diff>

<commit_message>
Add the Immortal (armor paragon) and make certified units move as their current class
cls_immortal (Persian, lance + bow, armor movement) fills the one movement type
that had no paragon, with the signature skill Ten Thousand (+2 dmg, +3 guard,
+2 speed). Lance-primary units see it beside the Bogatyr.

Also fixes a gap it exposed: the battle map built every unit's movement from
the class it was recruited as, so certification never changed how a unit moved
(a Paladin still walked 5 and crossed fords). Units now take their current
class's movement type and move, and are hit as that class.

test_armor_paragon (31); paragon tests updated for the extra lance option.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -22699,7 +22699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="17" min="1" max="1"/>
@@ -25511,61 +25511,110 @@
     <row r="58" ht="15" customHeight="1" s="18">
       <c r="A58" s="23" t="inlineStr">
         <is>
+          <t>cls_immortal</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>Immortal</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="inlineStr">
+        <is>
+          <t>paragon</t>
+        </is>
+      </c>
+      <c r="D58" s="23" t="inlineStr">
+        <is>
+          <t>lance</t>
+        </is>
+      </c>
+      <c r="E58" s="23" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="F58" s="23" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="G58" s="23" t="n"/>
+      <c r="H58" s="23" t="inlineStr">
+        <is>
+          <t>Ten Thousand</t>
+        </is>
+      </c>
+      <c r="I58" s="23" t="inlineStr">
+        <is>
+          <t>Persian</t>
+        </is>
+      </c>
+      <c r="J58" s="23" t="inlineStr">
+        <is>
+          <t>lv30+, deed-gated. ADDED 2026-10-16 to fill the armor gap: every paragon class moved on foot, on a horse or in the air, so the armor movement type (the General, the Housecarl, the Pavisier, the War monk, the Great shield...) had no second tier. The Immortal is the Persian heavy spearman-archer, the standing corps whose ranks were refilled the moment a man fell, so there were always ten thousand. A second lance paragon beside the Bogatyr (which rides), and it carries a bow like the Fianna. Name, culture, art pair, movement and the signature skill are all drafted; none is setting canon.</t>
+        </is>
+      </c>
+      <c r="K58" s="17" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="23" t="inlineStr">
+        <is>
           <t>cls_billman</t>
         </is>
       </c>
-      <c r="B58" s="23" t="inlineStr">
+      <c r="B59" s="23" t="inlineStr">
         <is>
           <t>Billman</t>
         </is>
       </c>
-      <c r="C58" s="23" t="inlineStr">
+      <c r="C59" s="23" t="inlineStr">
         <is>
           <t>hybrid</t>
         </is>
       </c>
-      <c r="D58" s="23" t="inlineStr">
+      <c r="D59" s="23" t="inlineStr">
         <is>
           <t>axe</t>
         </is>
       </c>
-      <c r="E58" s="23" t="inlineStr">
+      <c r="E59" s="23" t="inlineStr">
         <is>
           <t>lance</t>
         </is>
       </c>
-      <c r="F58" s="23" t="inlineStr">
+      <c r="F59" s="23" t="inlineStr">
         <is>
           <t>infantry</t>
         </is>
       </c>
-      <c r="G58" s="23" t="inlineStr">
+      <c r="G59" s="23" t="inlineStr">
         <is>
           <t>cls_tr_axe</t>
         </is>
       </c>
-      <c r="H58" s="23" t="n"/>
-      <c r="I58" s="23" t="inlineStr">
+      <c r="H59" s="23" t="n"/>
+      <c r="I59" s="23" t="inlineStr">
         <is>
           <t>setting-new</t>
         </is>
       </c>
-      <c r="J58" s="23" t="inlineStr">
+      <c r="J59" s="23" t="inlineStr">
         <is>
           <t>DRAFTED, not placed on any unit. The axe+lance pair the halberd needs (weapons.wpn_halberd req_arts) -- no existing class has it. Added 2026-10-02 so the overlap-weapon proficiency rule has a wielder; the first user is the enemy archetype ea_billman.</t>
         </is>
       </c>
-      <c r="K58" s="17" t="inlineStr">
+      <c r="K59" s="17" t="inlineStr">
         <is>
           <t>map_tp19</t>
         </is>
       </c>
     </row>
-    <row r="59"/>
-    <row r="60">
-      <c r="A60" s="25" t="inlineStr">
-        <is>
-          <t>Deliberate permanent gaps: brawl+riding, brawl+flying. reason+flying is a founded gap (broken by paralogue into Tzitzimitl). Galeforce permanently banned. ADDENDUM (2026-10-05): added unlock_map_id -- a hybrid class is not offered at certification until the player has won that map (drafted, thematic: Billman = Throat Pass where the halberd-bearers stand; Ferryman = the Drowned March's lake; Pardoner = the mercy chapter; Ash Ascetic = the Stepped Coast's lake; Miasma Warden = the Dove Colony). Blank for every non-hybrid class. ADDENDUM (2026-10-06): the paragon tier is built. A unit that is certified, level 30+, has earned a paragon-gating epithet and can pay the fee may take a paragon class whose primary art it already knows; Tzitzimitl (the founded gap) also needs map_p_simurgh won (drafted guess: the flying paralogue). Faith has no paragon class -- a gap left for you to decide, not invented. unlock_map_id now applies to hybrid and paragon tiers. ADDENDUM (2026-10-14): cls_krivis (Baltic) is a drafted faith paragon, filling the one art that had none.</t>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="25" t="inlineStr">
+        <is>
+          <t>Deliberate permanent gaps: brawl+riding, brawl+flying. reason+flying is a founded gap (broken by paralogue into Tzitzimitl). Galeforce permanently banned. ADDENDUM (2026-10-05): added unlock_map_id -- a hybrid class is not offered at certification until the player has won that map (drafted, thematic: Billman = Throat Pass where the halberd-bearers stand; Ferryman = the Drowned March's lake; Pardoner = the mercy chapter; Ash Ascetic = the Stepped Coast's lake; Miasma Warden = the Dove Colony). Blank for every non-hybrid class. ADDENDUM (2026-10-06): the paragon tier is built. A unit that is certified, level 30+, has earned a paragon-gating epithet and can pay the fee may take a paragon class whose primary art it already knows; Tzitzimitl (the founded gap) also needs map_p_simurgh won (drafted guess: the flying paralogue). Faith has no paragon class -- a gap left for you to decide, not invented. unlock_map_id now applies to hybrid and paragon tiers. ADDENDUM (2026-10-14): cls_krivis (Baltic) is a drafted faith paragon, filling the one art that had none. ADDENDUM (2026-10-16): cls_immortal (Persian) is a drafted armor-movement paragon, so no movement type is left without a second tier.</t>
         </is>
       </c>
     </row>
@@ -35426,7 +35475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M43"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" style="18" min="1" max="1"/>
@@ -37604,6 +37653,57 @@
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>ab_ten_thousand</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Ten Thousand</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>class:cls_immortal</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J43" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M43" s="17" t="inlineStr">
+        <is>
+          <t>Drafted signature skill for the Immortal: a passive approximation of ranks that close as men fall -- steady blows, harder to hurt, and enough speed back to offset the weight of the armour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft ability table, review before treating as canon. pool is pipe-delimited tags a unit's class must match one of: 'any', 'art:&lt;art&gt;', 'move:&lt;movement&gt;', 'tier:&lt;tier&gt;', 'class:&lt;class_id&gt;'. cond: always | hp_full | hp_low (&lt;= half HP) | vs_&lt;movement&gt; (the foe's movement type) | art:&lt;art&gt; (the wielded weapon's art). Effects are flat: hit/avoid/crit/dodge points, dmg added to damage dealt, guard subtracted from damage taken, speed added to attack speed, exp_pct EXP percent. Passive combat effects only: canon's map-action skills (Shove, Steal, Refresh, Provoke...) need systems that don't exist. Slots come from promotion_rules (slots_*). Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): the six paragon signature skills (Astra, Deadeye, Fierce Iron Fist, Colossus, Stun, Corrosion) and Charge now also listed for the Bogatyr.</t>
         </is>

</xml_diff>

<commit_message>
Add defections: Waldrada, Anselm, Maren and the guest Anna
Canon's defections and guest_units tabs were never read. Now winning the trigger
map makes a joined unit leave (Waldrada at the Vashti seat, Anselm at the Vetch
reunion, Maren at the Column B opener unless the Cinder Track was worked); they
leave the roster with their weapons and return as a lieutenant (never the boss)
beside a seal on a later map, listing the titles the player's play earned.
Killing one is permanent; winning the Cinder Track brings Maren back. Anna joins
once both Anselm and Maren have gone, at median level less 2, and leaves when the
reunion is won.

Canon: defections trigger/unless/return/appears maps, guest requires/depart,
guest_level_gap; validator rule c07n. test_defections (57). DEFECTIONS_DESIGN.md.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -14159,7 +14159,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="17" min="1" max="1"/>
@@ -14171,6 +14171,10 @@
     <col width="40" customWidth="1" style="17" min="7" max="7"/>
     <col width="15" customWidth="1" style="17" min="8" max="8"/>
     <col width="44" customWidth="1" style="17" min="9" max="9"/>
+    <col width="18" customWidth="1" style="18" min="10" max="10"/>
+    <col width="18" customWidth="1" style="18" min="11" max="11"/>
+    <col width="18" customWidth="1" style="18" min="12" max="12"/>
+    <col width="18" customWidth="1" style="18" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -14219,6 +14223,26 @@
           <t>signposting</t>
         </is>
       </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>trigger_map_id</t>
+        </is>
+      </c>
+      <c r="K1" s="21" t="inlineStr">
+        <is>
+          <t>trigger_unless_map_id</t>
+        </is>
+      </c>
+      <c r="L1" s="21" t="inlineStr">
+        <is>
+          <t>return_map_id</t>
+        </is>
+      </c>
+      <c r="M1" s="21" t="inlineStr">
+        <is>
+          <t>appears_map_id</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -14266,6 +14290,16 @@
           <t>signposted across Act 1 supports and her conduct on sect maps</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>map_v21</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>map_v22</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.25" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -14313,6 +14347,16 @@
           <t>a theological event, not a grievance; he says so before he goes</t>
         </is>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>map_c21</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>map_k21</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.25" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -14360,11 +14404,32 @@
           <t>caused by a supply decision several chapters earlier; reversible by a different one</t>
         </is>
       </c>
-    </row>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>map_b15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>map_ct19</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>map_ct19</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>map_tp19</t>
+        </is>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>RULES. One scripted defection per route (the story needs one thing the player cannot optimise away) and one conditional. Defection is not death: they leave the roster, appear later as a lieutenant standing near someone else's seal, and every support chain they earned stays readable. They take their epithets and pact obligations with them, so the title list on that pre-battle screen is one the player generated. Never the boss -- the anti-pact toolkit still governs the fight, so the map can be won without killing them.</t>
+          <t>RULES. One scripted defection per route (the story needs one thing the player cannot optimise away) and one conditional. Defection is not death: they leave the roster, appear later as a lieutenant standing near someone else's seal, and every support chain they earned stays readable. They take their epithets and pact obligations with them, so the title list on that pre-battle screen is one the player generated. Never the boss -- the anti-pact toolkit still governs the fight, so the map can be won without killing them. ADDENDUM (2026-10-18): the game now runs these. trigger_map_id: the defection happens when that map is first won (and the unit has joined); trigger_unless_map_id: not if this map is already won (Maren: the Ashland column was worked, so the supply decision went her way); return_map_id: winning it brings a recoverable defector back (Maren, if she has not fallen); appears_map_id: the map where she stands as a lieutenant near the seal (the boss, else the first foe). All four are drafted readings of the trigger/signposting text -- the maps are guesses. A defector who is killed as a lieutenant is gone for good (and cannot be won back).</t>
         </is>
       </c>
     </row>
@@ -14381,7 +14446,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="18" min="1" max="1"/>
@@ -14395,6 +14460,8 @@
     <col width="30" customWidth="1" style="18" min="9" max="9"/>
     <col width="40" customWidth="1" style="18" min="10" max="10"/>
     <col width="40" customWidth="1" style="18" min="11" max="11"/>
+    <col width="18" customWidth="1" style="18" min="12" max="12"/>
+    <col width="18" customWidth="1" style="18" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14453,6 +14520,16 @@
           <t>act3_payoff</t>
         </is>
       </c>
+      <c r="L1" s="26" t="inlineStr">
+        <is>
+          <t>requires_defections</t>
+        </is>
+      </c>
+      <c r="M1" s="26" t="inlineStr">
+        <is>
+          <t>depart_map_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -14510,11 +14587,21 @@
           <t>RECONSTRUCTION GAP -- not included in the changelog summary this row was built from; needs the real text from the source session (see calendar's decan-token row, which references this field directly).</t>
         </is>
       </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>def_anselm|def_maren</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>map_rf20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>PRINCIPLE -- guest units exist to cover a class niche a scripted/conditional removal could zero out, without bending the departing character's own arc to protect roster math. Modeled on FFXII's guest-character pattern: narrative weight lives almost entirely outside combat tenure, not inside it.</t>
+          <t>PRINCIPLE -- guest units exist to cover a class niche a scripted/conditional removal could zero out, without bending the departing character's own arc to protect roster math. Modeled on FFXII's guest-character pattern: narrative weight lives almost entirely outside combat tenure, not inside it. ADDENDUM (2026-10-18): requires_defections = every one of these must have happened (not merely one); depart_map_id = she leaves when that map is first won (the reunion: ch_rf20). She joins at the squad's median level less prm_guest_level_gap, fights with her class's basic art, earns no EXP and has no support chain.</t>
         </is>
       </c>
     </row>
@@ -22738,7 +22825,7 @@
       <c r="O33" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="P33" t="inlineStr">
+      <c r="P33" s="17" t="inlineStr">
         <is>
           <t>heal_allies</t>
         </is>
@@ -22792,7 +22879,7 @@
         </is>
       </c>
       <c r="M34" s="17" t="n"/>
-      <c r="N34" t="inlineStr">
+      <c r="N34" s="17" t="inlineStr">
         <is>
           <t>riding</t>
         </is>
@@ -22852,7 +22939,7 @@
       <c r="O35" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="P35" t="inlineStr">
+      <c r="P35" s="17" t="inlineStr">
         <is>
           <t>unmake</t>
         </is>
@@ -22909,7 +22996,7 @@
       <c r="O36" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P36" s="17" t="inlineStr">
         <is>
           <t>pull</t>
         </is>
@@ -26058,17 +26145,17 @@
           <t>the baseline master, always reachable if the crown is willing</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>loc_kaisareia_walls</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>always</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="L4" s="17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -26118,17 +26205,17 @@
           <t>arms lances and axes: the common soldier's tools, not the officer's. Fitting that the hardest-won master smith makes the plainest weapons</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>loc_vashti_gate</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>won:map_ct19</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="L5" s="17" t="n">
         <v>2</v>
       </c>
     </row>
@@ -26178,21 +26265,20 @@
           <t>the master smith outside the state's reach entirely, which is the point</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>loc_ostrova</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t>won:map_x11</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="L6" s="17" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -26299,12 +26385,12 @@
           <t>a blade that heals its wielder's allies on contact rather than the wielder</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="17" t="inlineStr">
         <is>
           <t>ea_simurgh</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>wpn_feather_blade</t>
         </is>
@@ -26341,12 +26427,12 @@
           <t>the Karkadann-horned lance: strong vs. mounted units, nothing special vs. infantry</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" s="17" t="inlineStr">
         <is>
           <t>ea_karkadann</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>wpn_karkadann_lance</t>
         </is>
@@ -26383,12 +26469,12 @@
           <t>an edge that unmakes weapons on contact, from something that already unmakes weapons</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>ea_anzu</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>wpn_anzu_edge</t>
         </is>
@@ -26425,12 +26511,12 @@
           <t>a bow that hums and drags the nearest enemy a tile closer -- can't be turned off</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" s="17" t="inlineStr">
         <is>
           <t>ea_shadhavar</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>wpn_shadhavar_bow</t>
         </is>
@@ -26460,7 +26546,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -34728,7 +34813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D72"/>
+  <dimension ref="A1:D73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -35852,7 +35937,23 @@
     <row r="72">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters.</t>
+          <t>prm_guest_level_gap</t>
+        </is>
+      </c>
+      <c r="B72" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" s="17" t="n"/>
+      <c r="D72" s="17" t="inlineStr">
+        <is>
+          <t>A guest unit (Anna) joins this many levels under the squad's median, from her class's trained baseline grown by her profile's expected rates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap.</t>
         </is>
       </c>
     </row>
@@ -46459,7 +46560,7 @@
           <t>map_p_shadhavar</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="V13" s="17" t="inlineStr">
         <is>
           <t>nmd_shadhavar</t>
         </is>
@@ -46533,7 +46634,7 @@
           <t>map_p_simurgh</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="V14" s="17" t="inlineStr">
         <is>
           <t>nmd_simurgh</t>
         </is>
@@ -46607,7 +46708,7 @@
           <t>map_p_karkadann</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="V15" s="17" t="inlineStr">
         <is>
           <t>nmd_karkadann</t>
         </is>
@@ -46681,7 +46782,7 @@
           <t>map_p_anzu</t>
         </is>
       </c>
-      <c r="V16" t="inlineStr">
+      <c r="V16" s="17" t="inlineStr">
         <is>
           <t>nmd_anzu</t>
         </is>

</xml_diff>

<commit_message>
Add deputy scoring: the crown's ledger and the writ scene
Canon's deputy_ledger weights are now run. On main-story chapters the crown's
surveyor (at the camp, radius 4) writes down deeds (2), delivery/hold/dispersal
(1.5), the stated objective (1), kills (0.5, 0 if unwitnessed) and a witness
bonus (1); paralogues score 0; Ricberta's revealed literacy (0.25) breaks ties.
Before the Second Writ the writ screen shows the ledger and the crown's pick;
Enter accepts, Enter twice contests (once), which withholds Column B's supply
attachment (+100 gold per Column B chapter, drafted). The deputy shows on the
overworld and in the barracks.

Canon: deputy_ledger.factor_id, supports.reveals/reveals_about/reveals_at_rank,
surveyor_radius, column_b_supply_gold; validator rule c07o. test_deputy (73).
DEPUTY_DESIGN.md.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -10109,12 +10109,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="30" customWidth="1" style="17" min="1" max="1"/>
     <col width="10" customWidth="1" style="17" min="2" max="2"/>
     <col width="46" customWidth="1" style="17" min="3" max="3"/>
+    <col width="18" customWidth="1" style="18" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -10133,6 +10134,11 @@
           <t>rationale</t>
         </is>
       </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>factor_id</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -10148,6 +10154,11 @@
           <t>main-story chapters only</t>
         </is>
       </c>
+      <c r="D2" s="17" t="inlineStr">
+        <is>
+          <t>writ_deed</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -10163,6 +10174,11 @@
           <t>unofficial work, off the books</t>
         </is>
       </c>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>paralogue_deed</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -10178,6 +10194,11 @@
           <t>counts toward the map's briefed goal</t>
         </is>
       </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>on_objective</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -10193,6 +10214,11 @@
           <t>witnessed by the auditor</t>
         </is>
       </c>
+      <c r="D5" s="17" t="inlineStr">
+        <is>
+          <t>witnessed</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -10208,6 +10234,11 @@
           <t>far-corner heroics do not appear in the report</t>
         </is>
       </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>unwitnessed_kill</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -10223,6 +10254,11 @@
           <t>legible categories outweigh kills</t>
         </is>
       </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>legible</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -10238,6 +10274,11 @@
           <t>hard to write down in a way that survives a clerk</t>
         </is>
       </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>raw_kill</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -10253,11 +10294,16 @@
           <t>Ricberta only, and only if a support revealed it</t>
         </is>
       </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>The crown picks the deputy off this. Player may contest once at the writ scene; the crown grants it and withholds Column B's supply attachment.</t>
+          <t>The crown picks the deputy off this. Player may contest once at the writ scene; the crown grants it and withholds Column B's supply attachment. ADDENDUM (2026-10-19): the game now runs this. factor_id names each row for the code. Scoring is ADDITIVE per event, on main-story (writ) chapters only: a deed earned = writ_deed (2); a delivery, solo hold or dispersal deed also = legible (1.5); a kill = raw_kill (0.5) if made within the surveyor radius, else unwitnessed_kill (0); finishing a map's stated objective (seizing, escaping, escorting, felling the boss of a defend map) = on_objective (1); ANY of those done within the surveyor radius also earns witnessed (1). The surveyor stands at the camp -- the middle of the deploy row -- since far-corner heroics 'do not appear in the report'. Paralogue deeds score paralogue_deed (0). literacy is added (not stored) once a support of Ricberta's has revealed it (supports.reveals / reveals_at_rank). The writ scene is ch_x11 (the Second Writ): the crown's pick is the highest score; the player may name another, once; the crown grants it and withholds Column B's supply attachment (drafted as gold: prm_column_b_supply_gold on each Column B chapter won). Highest score wins ties by canonical order.</t>
         </is>
       </c>
     </row>
@@ -14290,12 +14336,12 @@
           <t>signposted across Act 1 supports and her conduct on sect maps</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="17" t="inlineStr">
         <is>
           <t>map_v21</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="17" t="inlineStr">
         <is>
           <t>map_v22</t>
         </is>
@@ -14347,12 +14393,12 @@
           <t>a theological event, not a grievance; he says so before he goes</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>map_c21</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M3" s="17" t="inlineStr">
         <is>
           <t>map_k21</t>
         </is>
@@ -14404,28 +14450,27 @@
           <t>caused by a supply decision several chapters earlier; reversible by a different one</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>map_b15</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>map_ct19</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>map_ct19</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>map_tp19</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="25" t="inlineStr">
         <is>
@@ -14587,12 +14632,12 @@
           <t>RECONSTRUCTION GAP -- not included in the changelog summary this row was built from; needs the real text from the source session (see calendar's decan-token row, which references this field directly).</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="17" t="inlineStr">
         <is>
           <t>def_anselm|def_maren</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M2" s="17" t="inlineStr">
         <is>
           <t>map_rf20</t>
         </is>
@@ -27554,8 +27599,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I155"/>
+  <dimension ref="A1:L155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" style="18" min="10" max="10"/>
+    <col width="14" customWidth="1" style="18" min="11" max="11"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="17" t="inlineStr">
@@ -27603,6 +27652,21 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="J1" s="17" t="inlineStr">
+        <is>
+          <t>reveals</t>
+        </is>
+      </c>
+      <c r="K1" s="17" t="inlineStr">
+        <is>
+          <t>reveals_at_rank</t>
+        </is>
+      </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>reveals_about</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -27704,6 +27768,21 @@
           <t>Both signs reused verbatim (Avatar=Scorpion from Avatar/Maren, Ricberta=Crab from Ricberta/Sigrun). Direct tie: Ricberta's own note ('secretly literate... literacy is a deputy tiebreak') is exactly the kind of hidden-competence-as-liability the avatar's own institutional position lets them actually shield, unlike the peers who could only ever gossip about it. Platonic chain, capped at A.</t>
         </is>
       </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K4" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="17" t="inlineStr">
@@ -29208,6 +29287,21 @@
           <t>Both signs reused verbatim (Ricberta=Crab from Ricberta/Sigrun, Emmerich=Lion from Jost/Emmerich). Both diadem-route (ch_d02). Crab's loyalty to her men and Lion's showcase padding meet in a shared, quiet second ledger. Platonic chain, capped at A.</t>
         </is>
       </c>
+      <c r="J36" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K36" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
@@ -29255,6 +29349,21 @@
           <t>Signs assigned per the signs tab's own methodology (argued from behaviour, not a keyword): Ricberta=Crab off her own note ('secretly literate... literacy is a deputy tiebreak' -- guards a secret to protect her position and the people under her, the Crab's own failure mode -- loyalty to people over the cause -- is the exact shape of hiding competence to keep her sergeant's post rather than risk promotion scrutiny). Sigrun=Archer off hers ('courier rider' -- ranges out, returns with news, the Archer's failure mode 'says the true thing at the worst moment' is the literal action that breaks the support open in the B-&gt;A transition).</t>
         </is>
       </c>
+      <c r="J37" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K37" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
@@ -29302,6 +29411,21 @@
           <t>Both signs reused verbatim (Ricberta=Crab from Ricberta/Sigrun, Waldrada=Scales from Waldrada/Edda). Both diadem-route (ch_d02). Crab's loyalty-to-people failure mode and Scales' deliberation-as-delay resolve into the same answer from two directions. Platonic chain, capped at A.</t>
         </is>
       </c>
+      <c r="J38" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K38" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
@@ -29537,6 +29661,21 @@
           <t>Both signs reused verbatim (Ricberta=Crab from Ricberta/Sigrun, Gunnar=Goat from Gunnar/Edda). Cross-route (diadem/assembly), post-convergence. Gunnar's own note ('crossbow-certified') turned into a paper he cannot read; Ricberta's secret literacy finally has one safe audience. Platonic chain, capped at A.</t>
         </is>
       </c>
+      <c r="J43" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K43" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
@@ -29582,6 +29721,21 @@
       <c r="I44" s="17" t="inlineStr">
         <is>
           <t>Both signs reused verbatim (Ricberta=Crab from Ricberta/Sigrun, Edda=Maiden from Waldrada/Edda). Cross-route (diadem/assembly), post-convergence. Ricberta's secret literacy becomes a gift to a keeper of the record who can't write. Platonic chain, capped at A.</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="K44" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>u_ricberta</t>
         </is>
       </c>
     </row>
@@ -34813,7 +34967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D73"/>
+  <dimension ref="A1:D75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -35953,7 +36107,39 @@
     <row r="73">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap.</t>
+          <t>prm_surveyor_radius</t>
+        </is>
+      </c>
+      <c r="B73" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C73" s="17" t="n"/>
+      <c r="D73" s="17" t="inlineStr">
+        <is>
+          <t>Deputy scoring: an action is 'witnessed' if the unit that did it is within this many tiles of the surveyor (the camp, the middle of the deploy row).</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>prm_column_b_supply_gold</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="n">
+        <v>100</v>
+      </c>
+      <c r="C74" s="17" t="n"/>
+      <c r="D74" s="17" t="inlineStr">
+        <is>
+          <t>Deputy scoring: the Column B supply attachment, drafted as this much gold on each Column B chapter newly won -- withheld if the player contested the crown's choice of deputy at the writ scene.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add weapon names: marks from deeds, provenance names, reforging
A deed earned with a weapon in hand is written on it; the strongest mark names the
blade (Taker's Iron Axe, Iron Axe, Slayer of the Karkadann). Marks travel with the
weapon and outlive its wielder. A master smith reforges a marked convoy weapon for
150 gold, clearing the marks. The epilogue names the blade.

Canon: epithets.weapon_form/weapon_form_bare, weapon_marks_max and reforge_fee;
validator c07q.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -9704,7 +9704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9716,6 +9716,8 @@
     <col width="10" customWidth="1" style="18" min="7" max="7"/>
     <col width="14" customWidth="1" style="18" min="8" max="8"/>
     <col width="14" customWidth="1" style="18" min="9" max="9"/>
+    <col width="28" customWidth="1" style="18" min="10" max="10"/>
+    <col width="28" customWidth="1" style="18" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -9764,6 +9766,16 @@
           <t>deed_terrain</t>
         </is>
       </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>weapon_form</t>
+        </is>
+      </c>
+      <c r="K1" s="21" t="inlineStr">
+        <is>
+          <t>weapon_form_bare</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -9804,6 +9816,16 @@
       <c r="H2" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>{BASE}, Slayer of {OBJECT}</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Slayer's {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -9844,6 +9866,11 @@
       <c r="H3" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>{BASE} of the Ford</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -9884,6 +9911,11 @@
       <c r="H4" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Untouched {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -9929,6 +9961,11 @@
           <t>ter_miasma</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Ash-walker's {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -9969,6 +10006,11 @@
       <c r="H6" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Carter's {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -10009,6 +10051,11 @@
       <c r="H7" s="17" t="n">
         <v>3</v>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Merciful {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -10049,6 +10096,11 @@
       <c r="H8" s="17" t="n">
         <v>1</v>
       </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Peacemaker's {BASE}</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -10089,7 +10141,13 @@
       <c r="H9" s="17" t="n">
         <v>5</v>
       </c>
-    </row>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Taker's {BASE}</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -13233,7 +13291,7 @@
           <t>cleanses corruption; the only thing that can strip a pact without a Pardoner, and will not do it on request</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="17" t="inlineStr">
         <is>
           <t>the Simurgh's light</t>
         </is>
@@ -13280,7 +13338,7 @@
           <t>kill-taboo: whoever lands the blow dies in forty days, no reload undoes it</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>the Huma's shadow</t>
         </is>
@@ -13327,7 +13385,7 @@
           <t>COST: weapons it unmakes cannot be captured, so riding it starves your only supply line</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>the Anzu's stoop</t>
         </is>
@@ -13374,7 +13432,7 @@
           <t>the plain one on purpose -- the roster needs one straightforwardly good option</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" s="17" t="inlineStr">
         <is>
           <t>the Karkadann's charge</t>
         </is>
@@ -13421,13 +13479,12 @@
           <t>liability on escort maps, asset on defend maps</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>the Shadhavar's song</t>
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -13944,12 +14001,12 @@
           <t>triumphal</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O7" s="17" t="inlineStr">
         <is>
           <t>band</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P7" s="17" t="inlineStr">
         <is>
           <t>band</t>
         </is>
@@ -13988,12 +14045,12 @@
           <t>elegiac</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="O8" s="17" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="P8" s="17" t="inlineStr">
         <is>
           <t>hazard</t>
         </is>
@@ -16469,7 +16526,7 @@
           <t>reach -- it can feed itself from anywhere with a coast</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="17" t="inlineStr">
         <is>
           <t>Diadem</t>
         </is>
@@ -16526,7 +16583,7 @@
           <t>interior lines, timber, horses -- and credit: it HIRES fleets it cannot build</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K3" s="17" t="inlineStr">
         <is>
           <t>Assembly</t>
         </is>
@@ -16583,7 +16640,7 @@
           <t>the only gap in the mountain wall, and it charges for it</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>Toll League</t>
         </is>
@@ -16640,7 +16697,7 @@
           <t>capital, and the oldest continuous records on the map</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K5" s="17" t="inlineStr">
         <is>
           <t>River Kingdoms</t>
         </is>
@@ -16697,7 +16754,7 @@
           <t>cannot be conquered because there is nothing to seize</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K6" s="17" t="inlineStr">
         <is>
           <t>Herd Clan</t>
         </is>
@@ -16754,7 +16811,7 @@
           <t>grain, and a policy of selling it to both sides</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K7" s="17" t="inlineStr">
         <is>
           <t>Green Ports</t>
         </is>
@@ -16811,13 +16868,12 @@
           <t>pilotage -- the Isles' crews are why anyone crosses safely</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K8" s="17" t="inlineStr">
         <is>
           <t>Isles</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="15" customHeight="1" s="18">
       <c r="A10" s="25" t="inlineStr">
         <is>
@@ -21336,536 +21392,537 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>epi_head</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>{NAME}, {TITLE}, fell at {PLACE}</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>opening clause when the unit holds an epithet</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>epi_head_plain</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>{NAME} fell at {PLACE}</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>opening clause for someone plain -- the name stands alone</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>epi_tail_known</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve"> to {KILLER}</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>killer clause tail for any named or factional killer</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>epi_tail_unknown</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>, in the chaos, to no blade anyone could name</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>reserved for routs and unwitnessed deaths; bleaker than a named killer, not vaguer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>epi_tail_hazard</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve"> to {HAZARD}</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>a death with no hand in it (extension to the enum: killed_by_type hazard)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>epi_hazard_cold</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
         <is>
           <t>the cold</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>hazard names, keyed epi_hazard_&lt;id&gt;</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>epi_killer_polity</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>{A} {ADJ} {NOUN}</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>faction, not a person: a Diadem lance, an Assembly arrow</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>epi_killer_band</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>{A} {WHO}'s {NOUN}</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>an unaffiliated armed band, or a soldier whose map names no polity (extension: killed_by_type band)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>epi_killer_named</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>{PHRASE}</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>the Named creature signature verb (named.death_phrase)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>epi_killer_defector</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>{DEFECTOR}</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>a defector is named directly</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>epi_killer_boss</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>{BOSS}</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>a chapter boss is named directly</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>epi_title_slayer_of</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>{TOKEN} {OBJECT}</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>forge_vocab_token ending in "of" takes the thing slain</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>epi_title_slayer_fallback</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>the Slayer</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>when the deed was earned but the quarry was not recorded</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>epi_title_the</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="17" t="inlineStr">
         <is>
           <t>the {TOKEN}</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>a bare forge_vocab_token: the Untouched</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>epi_weapon_lost_to_enemy</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>{NAME}'s {WEAPON} passed to no one.</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} passed to no one.</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
         <is>
           <t>weapon_fate lost_to_enemy</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>epi_weapon_retrieved</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>{NAME}'s {WEAPON} came home in the convoy.</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} came home in the convoy.</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
         <is>
           <t>weapon_fate retrieved</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>epi_weapon_thrown_and_lost</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>{NAME}'s {WEAPON} was thrown, and not found again.</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} was thrown, and not found again.</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
         <is>
           <t>weapon_fate thrown_and_lost</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>epi_weapon_with_the_body</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="17" t="inlineStr">
         <is>
           <t>{NAME} was buried still holding the {WEAPON}.</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="C19" s="17" t="inlineStr">
         <is>
           <t>weapon_fate with_the_body</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>epi_support_platonic_C</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} knew {NAME} only a little, and said so.</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>platonic, tier C</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>epi_support_platonic_B</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} kept {NAME}'s watch that night.</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>platonic, tier B</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>epi_support_platonic_A</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} carried {NAME}'s name into every fight after.</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>platonic, tier A</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>epi_support_romantic_C</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} had meant to say something, and did not.</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>romantic, tier C</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>epi_support_romantic_B</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} sat with the body until morning.</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="17" t="inlineStr">
         <is>
           <t>romantic, tier B</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>epi_support_romantic_A</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} would not speak of it.</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C25" s="17" t="inlineStr">
         <is>
           <t>romantic, tier A</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>epi_support_romantic_S</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} stayed on the field until someone made them leave.</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="17" t="inlineStr">
         <is>
           <t>romantic, tier S</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>epi_support_gone</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} was gone from the company by then.</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="17" t="inlineStr">
         <is>
           <t>the partner had defected or departed</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>epi_support_fallen_before</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} had fallen already, and there was no one left to grieve.</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="C28" s="17" t="inlineStr">
         <is>
           <t>the partner died earlier</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>epi_support_fallen_after</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B29" s="17" t="inlineStr">
         <is>
           <t>{PARTNER} did not outlive the war either.</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C29" s="17" t="inlineStr">
         <is>
           <t>the partner died later</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="17" t="inlineStr">
         <is>
           <t>epi_support_alone</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="17" t="inlineStr">
         <is>
           <t>No one at the fire was close enough to grieve properly.</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C30" s="17" t="inlineStr">
         <is>
           <t>unpaired: a quiet indictment of a run that never built the relationship</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="17" t="inlineStr">
         <is>
           <t>epi_roll_title</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B31" s="17" t="inlineStr">
         <is>
           <t>The Fallen</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C31" s="17" t="inlineStr">
         <is>
           <t>heading of the fallen roll</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>epi_roll_empty</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="17" t="inlineStr">
         <is>
           <t>No one has fallen. Yet.</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="17" t="inlineStr">
         <is>
           <t>the roll when it is empty</t>
         </is>
       </c>
     </row>
+    <row r="33"/>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>IMPLEMENTATION NOTES (2026-10-09). The text of epilogue_generation, built as scripts/epilogue.gd. Wording is DRAFT; placeholders in {BRACES} are filled by the generator, and {A} becomes 'a' or 'an' by the word after it. No line uses a pronoun for the fallen or the partner -- they/them is avoided by naming. TWO EXTENSIONS to the killed_by_type enum, which the original schema did not list: 'band' (an unaffiliated armed band -- looters, relic hunters, privateers, or a soldier on a map that names no polity) and 'hazard' (a death with no hand in it: the cold on map_a03). maps.enemy_polity_id is a DRAFT: state-affiliated enemies belong to the polity opposite the chapter's route (a Diadem-route map fields Assembly soldiers); both-route maps name none, so those soldiers read as a band. Tune it map by map.</t>
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>IMPLEMENTATION NOTES (2026-10-09). The text of epilogue_generation, built as scripts/epilogue.gd. Wording is DRAFT; placeholders in {BRACES} are filled by the generator, and {A} becomes 'a' or 'an' by the word after it. No line uses a pronoun for the fallen or the partner -- they/them is avoided by naming. TWO EXTENSIONS to the killed_by_type enum, which the original schema did not list: 'band' (an unaffiliated armed band -- looters, relic hunters, privateers, or a soldier on a map that names no polity) and 'hazard' (a death with no hand in it: the cold on map_a03). maps.enemy_polity_id is a DRAFT: state-affiliated enemies belong to the polity opposite the chapter's route (a Diadem-route map fields Assembly soldiers); both-route maps name none, so those soldiers read as a band. Tune it map by map. ADDENDUM (2026-10-20): {WEAPON} is the weapon's provenance name (epithets.weapon_form), which may already read as a possessive ("Taker's Iron Axe"), so the weapon lines say 'The {WEAPON}' rather than '{NAME}'s {WEAPON}'.</t>
         </is>
       </c>
     </row>
@@ -35632,7 +35689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D75"/>
+  <dimension ref="A1:D77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -36804,7 +36861,39 @@
     <row r="75">
       <c r="A75" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters.</t>
+          <t>prm_weapon_marks_max</t>
+        </is>
+      </c>
+      <c r="B75" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C75" s="17" t="n"/>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>Weapon names: the most marks (deeds earned with it) a weapon keeps; the oldest is dropped for a new one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="17" t="inlineStr">
+        <is>
+          <t>prm_reforge_fee</t>
+        </is>
+      </c>
+      <c r="B76" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C76" s="17" t="n"/>
+      <c r="D76" s="17" t="inlineStr">
+        <is>
+          <t>Weapon names: gold a master smith charges to reforge a marked weapon from the convoy, clearing its marks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee).</t>
         </is>
       </c>
     </row>
@@ -42923,7 +43012,7 @@
           <t>dock frontage|warehouse lane</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43000,7 +43089,7 @@
           <t>hedgerow foot path|open road (riding)|the weighbridge itself</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T3" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43080,7 +43169,7 @@
       <c r="S4" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="T4" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43160,7 +43249,7 @@
       <c r="S5" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T5" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -43237,7 +43326,7 @@
           <t>wide street (riding)|narrow street (foot)|rooftops (flying)</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T6" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -43314,7 +43403,7 @@
           <t>cloister (indoors, no cold)|open ward (fast, costly)</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T7" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -43535,7 +43624,7 @@
           <t>the weather deck|below, through the hold|the rigging (flying only)</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T10" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43684,7 +43773,7 @@
           <t>ash flats (foot)|the old road (riding)</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="T12" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43761,7 +43850,7 @@
           <t>the nave (foot)|the cloister walk (flying blocked)</t>
         </is>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="T13" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -43910,7 +43999,7 @@
           <t>the causeway (foot)|open floodwater (flying only)</t>
         </is>
       </c>
-      <c r="T15" t="inlineStr">
+      <c r="T15" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -43987,7 +44076,7 @@
           <t>the reading room (foot)|the stacks (foot only)</t>
         </is>
       </c>
-      <c r="T16" t="inlineStr">
+      <c r="T16" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -45274,7 +45363,7 @@
           <t>the quay (foot, riding)|the warehouse sheds (blocks flying)|open water (flying only)</t>
         </is>
       </c>
-      <c r="T34" t="inlineStr">
+      <c r="T34" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45349,7 +45438,7 @@
           <t>the lower terrace (foot, riding)|the upper terraces (riding blocked)</t>
         </is>
       </c>
-      <c r="T35" t="inlineStr">
+      <c r="T35" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45424,7 +45513,7 @@
           <t>the ruin floor (foot, riding)|the terrace above (riding blocked)</t>
         </is>
       </c>
-      <c r="T36" t="inlineStr">
+      <c r="T36" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45499,7 +45588,7 @@
           <t>the open ground (all movement, no cover, no chokepoints)</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="T37" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45574,7 +45663,7 @@
           <t>the road (foot, riding)|the lava-fan narrows (all movement, hazard)</t>
         </is>
       </c>
-      <c r="T38" t="inlineStr">
+      <c r="T38" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45649,7 +45738,7 @@
           <t>the ash-field approach (all movement, hazard)|the gate itself (foot, riding)</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="T39" s="17" t="inlineStr">
         <is>
           <t>pol_assembly</t>
         </is>
@@ -45724,7 +45813,7 @@
           <t>the quay (foot, riding)|the warehouse sheds (blocks flying)|open water (flying only)</t>
         </is>
       </c>
-      <c r="T40" t="inlineStr">
+      <c r="T40" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -45799,7 +45888,7 @@
           <t>the old shoreline (foot, riding)|the water (flying only)</t>
         </is>
       </c>
-      <c r="T41" t="inlineStr">
+      <c r="T41" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -45874,7 +45963,7 @@
           <t>the open steppe (all movement, no cover)|the settlement edge (foot, riding)</t>
         </is>
       </c>
-      <c r="T42" t="inlineStr">
+      <c r="T42" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -45949,7 +46038,7 @@
           <t>the cliff-edge shelf (foot, riding, narrow)|the void beyond it (flying only)</t>
         </is>
       </c>
-      <c r="T43" t="inlineStr">
+      <c r="T43" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -46024,7 +46113,7 @@
           <t>the forest road (foot, riding)|the canopy (blocks flying)</t>
         </is>
       </c>
-      <c r="T44" t="inlineStr">
+      <c r="T44" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -46099,7 +46188,7 @@
           <t>the shrine yard (foot, riding)|the shrine steps (foot only)</t>
         </is>
       </c>
-      <c r="T45" t="inlineStr">
+      <c r="T45" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -46174,7 +46263,7 @@
           <t>the chapel yard (foot, riding)|the chapel walls (foot only, breach point)</t>
         </is>
       </c>
-      <c r="T46" t="inlineStr">
+      <c r="T46" s="17" t="inlineStr">
         <is>
           <t>pol_diadem</t>
         </is>
@@ -46783,12 +46872,12 @@
           <t>We were told it was a drill. ... It isn't, is it.</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="W2" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="X2" s="17" t="inlineStr">
         <is>
           <t>sword</t>
         </is>
@@ -46873,12 +46962,12 @@
           <t>I never wanted this spear. Tell them you never saw me.</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
+      <c r="W3" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="X3" s="17" t="inlineStr">
         <is>
           <t>spear</t>
         </is>
@@ -46952,12 +47041,12 @@
           <t>map_a01</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="W4" s="17" t="inlineStr">
         <is>
           <t>band</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="X4" s="17" t="inlineStr">
         <is>
           <t>axe</t>
         </is>
@@ -47031,12 +47120,12 @@
           <t>map_a03</t>
         </is>
       </c>
-      <c r="W5" t="inlineStr">
+      <c r="W5" s="17" t="inlineStr">
         <is>
           <t>band</t>
         </is>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="X5" s="17" t="inlineStr">
         <is>
           <t>arrow</t>
         </is>
@@ -47110,12 +47199,12 @@
           <t>map_d05</t>
         </is>
       </c>
-      <c r="W6" t="inlineStr">
+      <c r="W6" s="17" t="inlineStr">
         <is>
           <t>band</t>
         </is>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="X6" s="17" t="inlineStr">
         <is>
           <t>cutlass</t>
         </is>
@@ -47189,12 +47278,12 @@
           <t>map_f00</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
+      <c r="W7" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="X7" s="17" t="inlineStr">
         <is>
           <t>lance</t>
         </is>
@@ -47264,12 +47353,12 @@
         </is>
       </c>
       <c r="Q8" s="17" t="n"/>
-      <c r="W8" t="inlineStr">
+      <c r="W8" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="X8" s="17" t="inlineStr">
         <is>
           <t>sword</t>
         </is>
@@ -47339,12 +47428,12 @@
         </is>
       </c>
       <c r="Q9" s="17" t="n"/>
-      <c r="W9" t="inlineStr">
+      <c r="W9" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="X9" s="17" t="inlineStr">
         <is>
           <t>lance</t>
         </is>
@@ -47414,12 +47503,12 @@
         </is>
       </c>
       <c r="Q10" s="17" t="n"/>
-      <c r="W10" t="inlineStr">
+      <c r="W10" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="X10" s="17" t="inlineStr">
         <is>
           <t>axe</t>
         </is>
@@ -47501,7 +47590,7 @@
           <t>You answered the still night, and the night answers you. Go on, then.</t>
         </is>
       </c>
-      <c r="W11" t="inlineStr">
+      <c r="W11" s="17" t="inlineStr">
         <is>
           <t>individual</t>
         </is>
@@ -47575,7 +47664,7 @@
           <t>map_a03</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
+      <c r="W12" s="17" t="inlineStr">
         <is>
           <t>individual</t>
         </is>
@@ -47654,7 +47743,7 @@
           <t>nmd_shadhavar</t>
         </is>
       </c>
-      <c r="W13" t="inlineStr">
+      <c r="W13" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
@@ -47733,7 +47822,7 @@
           <t>nmd_simurgh</t>
         </is>
       </c>
-      <c r="W14" t="inlineStr">
+      <c r="W14" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
@@ -47812,7 +47901,7 @@
           <t>nmd_karkadann</t>
         </is>
       </c>
-      <c r="W15" t="inlineStr">
+      <c r="W15" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
@@ -47891,7 +47980,7 @@
           <t>nmd_anzu</t>
         </is>
       </c>
-      <c r="W16" t="inlineStr">
+      <c r="W16" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
@@ -47970,12 +48059,12 @@
           <t>wpn_halberd</t>
         </is>
       </c>
-      <c r="W17" t="inlineStr">
+      <c r="W17" s="17" t="inlineStr">
         <is>
           <t>state</t>
         </is>
       </c>
-      <c r="X17" t="inlineStr">
+      <c r="X17" s="17" t="inlineStr">
         <is>
           <t>halberd</t>
         </is>

</xml_diff>

<commit_message>
Add the Sapper: Rinsa's Breach and Mine
cls_sapper placed on Rinsa (brawl, personal). Breach (D) brings an adjacent wall
or building down into a breach tile everyone can cross; Mine (M) lays a charge
for the first enemy to end a move on it. Three charges a map; suspensions keep
them. Per-map breach_symbols, ter_breach terrain, validator c07r.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -5318,7 +5318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="1" max="1"/>
@@ -6360,6 +6360,43 @@
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>ter_breach</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>v</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>breach (a broken wall)</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G28" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-21: what a wall or building becomes once a Sapper has brought it down -- rubble to climb over, slower for armor and riders, nothing to a flier. No hazard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft, review before treating as canon. 99 = impassable (genre convention: any integer exceeding every unit's move stat). Two real gaps this table exposes rather than solves: (1) prologue_roster has no movement_type column, so nothing can actually look up 'Tasme is riding' to apply these costs yet; (2) ter_wall/ter_statue costs are static but should really key off prologue_structures' HP/destroyed state instead of a fixed lookup. Grounded in map_f00.txt, map_f00_reference.png, maps.terrain for map_f00, and prologue_roster's per-unit notes; g/t/./a/* costs have no textual basis anywhere and are placeholder 1s pending your call. Drafted by a Claude Code session, 2026-09-14. ADDENDUM: hazard_dmg column + 11 new symbols added for map_a02/map_a03 (D and E -- defend point, escape tile -- also added as their own rows, matching whatever base terrain they sit on, since every grid symbol needs a cost/hazard entry or map_grid treats it as impassable). hazard_dmg is flat HP lost for ending a turn on that tile -- only map_a03's outdoor tiles (o/u/R) use it, grounded directly in map_a03's own terrain text ('cold drains 2 HP/turn outdoors'). Drafted by a Claude Code session, 2026-09-23. ADDENDUM 2: ter_ford (map_d03) and ter_covered_market (map_b15) added. d01/x11 reuse entirely existing symbols (./s/b/*/a/c/E) rather than adding new ones -- 'dock frontage'/'warehouse lane'/'muster field'/'river crossing' all matched an existing cost profile closely enough not to warrant a new row. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 3: ter_hedgerow (map_d02), ter_miasma/ter_ice (map_a01) added. map_d05 reuses ter_channel entirely for its open water ('riding impossible, armor sinks' already matches ter_channel's existing cost profile exactly) and ter_span for its gangways -- no new symbols needed there. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 4 (2026-09-25): hazard_dmg calibration pass. Checked every hazard-bearing row's own grounding before testing rather than assuming they were unsourced placeholders like the movement-cost columns were: ter_open_ward/ter_reliquary's hazard=2 is a DIRECT quote (map_a03.terrain: 'cold drains 2 HP/turn outdoors'), ter_rubble's reuses it ('still outdoors' on the same map), and ter_miasma's reuses it too ('rather than inventing a different number') -- only ter_ice's hazard=1 was ever flagged as a genuine approximation ('a stand-in for a real slip mechanic'). Simulated realistic crossing exposure (turn-by-turn shortest-path movement, damage applied only at turn end per _apply_hazard_damage's own real behavior) for an infantry unit across every map that uses a hazard symbol (map_a01/a03/ct19/d09/d10/k22/p_buried_works/p_karkadann): a full crossing costs 0-2 total hazard HP in every case (often just one turn-end tick), 7-12% of typical early-game HP -- felt, not punishing, and on map_d09 the pathfinder found the ford/span route built specifically to avoid the miasma entirely, taking 0 damage, exactly as that map intended. None of the 8 maps using hazard terrain are defend/survive objectives, so sustained multi-turn dwelling (the only way these values could become dangerous) is never structurally forced. No values changed -- both the sourced 2s and ice's approximate 1 (already half of miasma's severity, matching its own 'minor'/'risky' framing relative to miasma's 'toxic gas') held up against real content rather than staying untested assumptions. Drafted by a Claude Code session, 2026-09-25.</t>
         </is>
@@ -9816,12 +9853,12 @@
       <c r="H2" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="17" t="inlineStr">
         <is>
           <t>{BASE}, Slayer of {OBJECT}</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="17" t="inlineStr">
         <is>
           <t>Slayer's {BASE}</t>
         </is>
@@ -9866,7 +9903,7 @@
       <c r="H3" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>{BASE} of the Ford</t>
         </is>
@@ -9911,7 +9948,7 @@
       <c r="H4" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>Untouched {BASE}</t>
         </is>
@@ -9961,7 +9998,7 @@
           <t>ter_miasma</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J5" s="17" t="inlineStr">
         <is>
           <t>Ash-walker's {BASE}</t>
         </is>
@@ -10006,7 +10043,7 @@
       <c r="H6" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J6" s="17" t="inlineStr">
         <is>
           <t>Carter's {BASE}</t>
         </is>
@@ -10051,7 +10088,7 @@
       <c r="H7" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J7" s="17" t="inlineStr">
         <is>
           <t>Merciful {BASE}</t>
         </is>
@@ -10096,7 +10133,7 @@
       <c r="H8" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J8" s="17" t="inlineStr">
         <is>
           <t>Peacemaker's {BASE}</t>
         </is>
@@ -10141,13 +10178,12 @@
       <c r="H9" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J9" s="17" t="inlineStr">
         <is>
           <t>Taker's {BASE}</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -21918,7 +21954,6 @@
         </is>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
@@ -24330,7 +24365,7 @@
       </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>brawl</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
@@ -24352,7 +24387,12 @@
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>IN DRAWER, not yet placed</t>
+          <t>Rinsa (PLACED 2026-10-21: the descender who leads people down into the dark, so she knows how to get under a thing). Brawl, so she still fights; Breach (bring a wall down into a way through) and Mine (a charge laid on a tile for the first enemy to step on), three charges a map between them.</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>breach|mine</t>
         </is>
       </c>
     </row>
@@ -35689,7 +35729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -36893,7 +36933,39 @@
     <row r="77">
       <c r="A77" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee).</t>
+          <t>prm_sapper_charges</t>
+        </is>
+      </c>
+      <c r="B77" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C77" s="17" t="n"/>
+      <c r="D77" s="17" t="inlineStr">
+        <is>
+          <t>Sapper: charges a Sapper has on one map, shared between Breach and Mine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="inlineStr">
+        <is>
+          <t>prm_mine_damage</t>
+        </is>
+      </c>
+      <c r="B78" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C78" s="17" t="n"/>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>Sapper: flat damage a mine does to the first enemy that ends a move on it (a bit under a steel sword hit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage).</t>
         </is>
       </c>
     </row>
@@ -41929,7 +42001,7 @@
       </c>
       <c r="G18" s="23" t="inlineStr">
         <is>
-          <t>cls_tr_brawl</t>
+          <t>cls_sapper</t>
         </is>
       </c>
       <c r="H18" s="23" t="inlineStr">
@@ -42731,7 +42803,7 @@
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>trained</t>
+          <t>personal</t>
         </is>
       </c>
       <c r="D18" s="17" t="n">
@@ -42816,7 +42888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T53"/>
+  <dimension ref="A1:U53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="17" min="1" max="1"/>
@@ -42837,6 +42909,7 @@
     <col width="28" customWidth="1" style="17" min="18" max="18"/>
     <col width="14" customWidth="1" style="18" min="19" max="19"/>
     <col width="16" customWidth="1" style="18" min="20" max="20"/>
+    <col width="16" customWidth="1" style="18" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -42940,6 +43013,11 @@
           <t>enemy_polity_id</t>
         </is>
       </c>
+      <c r="U1" s="21" t="inlineStr">
+        <is>
+          <t>breach_symbols</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -43017,6 +43095,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -43331,6 +43414,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -45293,6 +45381,11 @@
           <t>the south corridor (all movement, clear)|straight through the rubble (foot favored, hazardous)</t>
         </is>
       </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
@@ -45443,6 +45536,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
@@ -45518,6 +45616,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
@@ -45743,6 +45846,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
@@ -45968,6 +46076,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -46193,6 +46306,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
@@ -46268,6 +46386,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
@@ -46336,6 +46459,11 @@
       <c r="R47" s="17" t="inlineStr">
         <is>
           <t>the plaza (foot, riding)|the covered market (blocks flying)|the silo blocks (impassable, all types)</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add eight weapons: Perun's Brand, Morningstar, two legendary bows, sacred texts and grimoires
A lightning sword (reach 2, strikes at RES), a two-range axe flail, Vila's Moonbow
(reach 3, effective vs fliers), Neith's Bow, the Miroslav Gospel (renew), the
Zographos Codex, the Goetia of Astaroth (drain) and The Lemegeton (recoil). Boss
drops, four new weapon effects, validator and flipbook updated.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -1019,6 +1019,11 @@
           <t>Stands on the defend-point tile (D) -- literally where the crowd/townsfolk are.</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>wpn_zographos_codex</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
@@ -1609,6 +1614,11 @@
           <t>Same template, east crossing. Two instances of the same archetype, not two distinct characters -- consistent with nothing being named in the source text.</t>
         </is>
       </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>wpn_perun_brand</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
@@ -4053,7 +4063,7 @@
       </c>
       <c r="K79" s="17" t="inlineStr">
         <is>
-          <t>wpn_sword_mid</t>
+          <t>wpn_lemegeton</t>
         </is>
       </c>
     </row>
@@ -4128,6 +4138,11 @@
           <t>The looter ringleader exploiting the dockside unrest -- see chapters.ch_d04's own note on why the protesters themselves aren't combatants.</t>
         </is>
       </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>wpn_morningstar</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="17" t="inlineStr">
@@ -4236,6 +4251,11 @@
           <t>Scavengers picking through the ruin -- the renunciants who live here are not combatants, see chapters.ch_d07.</t>
         </is>
       </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>wpn_neith_bow</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="17" t="inlineStr">
@@ -4498,6 +4518,11 @@
           <t>Opportunists working the medicine trade, same framing as ch_d04's harbour.</t>
         </is>
       </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>wpn_morningstar</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="17" t="inlineStr">
@@ -4724,6 +4749,11 @@
           <t>Bandits using the treeline for cover, not an organized force.</t>
         </is>
       </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>wpn_vila_moonbow</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="17" t="inlineStr">
@@ -4760,6 +4790,11 @@
           <t>sect_march's own 'Prophecy NPCs convert green levies' -- levies mid-conversion.</t>
         </is>
       </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>wpn_miroslav_gospel</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="17" t="inlineStr">
@@ -4952,7 +4987,7 @@
       </c>
       <c r="K103" s="17" t="inlineStr">
         <is>
-          <t>wpn_axe_high</t>
+          <t>wpn_astaroth_goetia</t>
         </is>
       </c>
     </row>
@@ -24390,7 +24425,7 @@
           <t>Rinsa (PLACED 2026-10-21: the descender who leads people down into the dark, so she knows how to get under a thing). Brawl, so she still fights; Breach (bring a wall down into a way through) and Mine (a charge laid on a tile for the first enemy to step on), three charges a map between them.</t>
         </is>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L49" s="17" t="inlineStr">
         <is>
           <t>breach|mine</t>
         </is>
@@ -24908,7 +24943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P37"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="1" max="1"/>
@@ -26742,6 +26777,451 @@
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>wpn_perun_brand</t>
+        </is>
+      </c>
+      <c r="B37" s="17" t="inlineStr">
+        <is>
+          <t>Perun's Brand</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>sword</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E37" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="G37" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H37" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="I37" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J37" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22 (the Levin Sword's heir). Perun is the Slavic thunder god, whose lightning splits the oak; the thunderbolt is the god's own 'brand'. Reaches two tiles and strikes at the foe's RES instead of its DEF: armor is no shelter from lightning. Dropped by the second captain of the Second Writ.</t>
+        </is>
+      </c>
+      <c r="M37" s="17" t="n"/>
+      <c r="O37" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="17" t="inlineStr">
+        <is>
+          <t>res_strike</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>wpn_morningstar</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>Morningstar</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>mid</t>
+        </is>
+      </c>
+      <c r="E38" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F38" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="G38" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I38" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="J38" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. A spiked flail on a haft: an axe weapon that reaches only two tiles, like a bow, so it cannot answer a blow from an adjacent foe. Dropped by the harbour bosses of Act 1.</t>
+        </is>
+      </c>
+      <c r="M38" s="17" t="n"/>
+      <c r="O38" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P38" s="17" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>wpn_vila_moonbow</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>Vila's Moonbow</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F39" s="17" t="n">
+        <v>90</v>
+      </c>
+      <c r="G39" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H39" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K39" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L39" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22 (the Balkan Artemis). The vila (Serbian) or samodiva (Bulgarian) is the wild woman of mountain and forest, an archer who answers a hunter's insolence with an arrow. A crescent bow that reaches three tiles and brings fliers down (effective against flying). Dropped on the Timber Road.</t>
+        </is>
+      </c>
+      <c r="M39" s="17" t="n"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>flying</t>
+        </is>
+      </c>
+      <c r="O39" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P39" s="17" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>wpn_neith_bow</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>Neith's Bow</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F40" s="17" t="n">
+        <v>95</v>
+      </c>
+      <c r="G40" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="H40" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I40" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J40" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L40" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. Neith, the Libyan-born huntress and weaver goddess of Sais, carried a bow and two arrows. Almost weightless, so it follows up easily, and it crits often. Dropped at the Stranded Harbour.</t>
+        </is>
+      </c>
+      <c r="M40" s="17" t="n"/>
+      <c r="O40" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P40" s="17" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="17" t="inlineStr">
+        <is>
+          <t>wpn_miroslav_gospel</t>
+        </is>
+      </c>
+      <c r="B41" s="17" t="inlineStr">
+        <is>
+          <t>Miroslav Gospel</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E41" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F41" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="G41" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="I41" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. The Miroslav Gospel is a real Serbian illuminated manuscript of the 12th century. The wielder recovers strength with every blow that lands. Dropped at the March Shrine.</t>
+        </is>
+      </c>
+      <c r="M41" s="17" t="n"/>
+      <c r="O41" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="17" t="inlineStr">
+        <is>
+          <t>renew</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="17" t="inlineStr">
+        <is>
+          <t>wpn_zographos_codex</t>
+        </is>
+      </c>
+      <c r="B42" s="17" t="inlineStr">
+        <is>
+          <t>Zographos Codex</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E42" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F42" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="G42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I42" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J42" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L42" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. The Codex Zographensis is among the oldest Glagolitic gospel books, the script made for people who had never had scripture in their own tongue. The plain one on purpose: the hardest-hitting sacred text and nothing else. Carried by the preacher of the still night.</t>
+        </is>
+      </c>
+      <c r="M42" s="17" t="n"/>
+      <c r="O42" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="17" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>wpn_astaroth_goetia</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="inlineStr">
+        <is>
+          <t>Goetia of Astaroth</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E43" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F43" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="G43" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="I43" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J43" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. Astaroth is the Lesser Key's duke of the knowledge of the past, a grandee of the underworld. An evil grimoire that feeds the reader: half the damage it deals comes back as health. Taken at the feeding of the Colossus.</t>
+        </is>
+      </c>
+      <c r="M43" s="17" t="n"/>
+      <c r="O43" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P43" s="17" t="inlineStr">
+        <is>
+          <t>drain</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="17" t="inlineStr">
+        <is>
+          <t>wpn_lemegeton</t>
+        </is>
+      </c>
+      <c r="B44" s="17" t="inlineStr">
+        <is>
+          <t>The Lemegeton</t>
+        </is>
+      </c>
+      <c r="C44" s="17" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>legendary</t>
+        </is>
+      </c>
+      <c r="E44" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F44" s="17" t="n">
+        <v>75</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H44" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="I44" s="17" t="n">
+        <v>30</v>
+      </c>
+      <c r="J44" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-22. The Lemegeton Clavicula Salomonis, the Lesser Key itself, holds the seventy-two spirits. The most powerful book in the game and it charges for it: the reader pays a little blood each time they open it (never enough to kill). Found in the Buried Works.</t>
+        </is>
+      </c>
+      <c r="M44" s="17" t="n"/>
+      <c r="O44" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="17" t="inlineStr">
+        <is>
+          <t>recoil</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft weapons table, review before treating as canon. Covers ordinary equipment only -- forges/materials' 5 legendary drops (3-of-5 cap) are a separate system above this tier, per forges' own note that the common smith 'arms lances and axes: the common soldier's tools, not the officer's.' Three tiers per art (basic/mid/high, flavor-named Iron/Steel/Silver) x 7 arts = 21 weapons. Might/hit/crit/weight/uses follow the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises) -- this design's own stated lineage per PROJECT_HANDOFF.md, not sourced from anything in canon.xlsx. Range: melee arts (sword/lance/axe/brawl) = 1, bow = 2, reason/faith = 1-2 (standard FE magic range). Names are placeholder and mechanical on purpose (e.g. 'Iron Tome', 'Iron Rite') -- real flavor-naming consistent with the setting's Byzantine/Near-East register is a writing pass for later, not attempted here. No weapon-rank/proficiency gating system exists yet (who can use which tier) -- units' single art_primary/secondary per class implicitly limits which art a unit fights with, but nothing yet gates basic vs. mid vs. high within that art. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: 'worn' tier added below basic -- might 1, hit 55, one art each. Built for the prologue's conquered-army soldiers (enemy_archetypes.ea_conquered_soldier): veteran-level troops equipped with whatever's left after a siege, not a new balance tier anyone is meant to fight through progression. Numbers are a judgment call (roughly basic tier's might/hit at a fifth to two-thirds), not derived from anything in canon.xlsx. Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-09-25): crit calibration pass. This row's own text already said crit 'follows the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises)' but every weapon actually shipped with crit=0, flat across all 4 tiers -- never filled in despite the stated intent. Extended the same tier-scaling might/hit/weight/uses already use: worn=0, basic=0 (unchanged -- starter/scavenged gear staying crit-free matches genre convention), mid=5, high=10. Simulated the resulting crit_chance() output (weapon_crit + attacker.dex - defender.lck, this session's own 2026-09-25 formula calibration) against all 1,056 ordered unit/enemy attacker-defender combos per tier: basic/worn stays at the formula's own baseline (57.5% nonzero, mean 3.4%, max 21%); mid roughly doubles presence (86.8% nonzero, mean 7.1%, max 26%); high makes crit a real threat without ever approaching a coinflip (97.3% nonzero, mean 11.9%, max 31%, only 2 of 1,056 combos clear 30%). Kept the crit value uniform across all 7 arts, matching every other column on this table already being purely tier-based, not art-based -- nothing here or in canon.xlsx supports giving e.g. bows a crit edge over axes. ADDENDUM (2026-10-02): added req_arts (pipe-delimited arts a wielder must ALL be proficient in; blank = just the weapon's own art) and effective_vs (pipe-delimited movement types the weapon deals x2 might to), plus 3 overlap weapons (halberd, maul, censer). A weapon with 2+ req_arts is triangle-neutral. Attack speed = spd - max(0, weight - str) (mag for magic arts); a unit doubles at +4 speed. See combat.gd. ADDENDUM 2 (2026-10-03): added convoy_qty -- how many of each weapon the shared convoy holds at the start of a playthrough (one mid-tier weapon per art; the overlap weapons start at 0 and arrive as drops). Every unit also starts with the basic weapon of its art (Equipment.ensure_loadout). `uses` is now spent: 1 per strike made, the weapon breaks at 0, no repair (map_f00's design note). ADDENDUM (2026-10-17): the 'legendary' tier is the master smiths' work (forges/materials tabs): four weapons, one per usable Named material, never found or bought. effect = a special on-hit rule (heal_allies / unmake / pull); blank = none. Legendary weapons need a certified class like high-tier ones.</t>
         </is>
@@ -35729,7 +36209,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -36965,7 +37445,55 @@
     <row r="79">
       <c r="A79" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage).</t>
+          <t>prm_renew_heal</t>
+        </is>
+      </c>
+      <c r="B79" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C79" s="17" t="n"/>
+      <c r="D79" s="17" t="inlineStr">
+        <is>
+          <t>Weapons: HP the Miroslav Gospel's wielder recovers after every blow that lands.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t>prm_drain_pct</t>
+        </is>
+      </c>
+      <c r="B80" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C80" s="17" t="n"/>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>Weapons: percent of the damage dealt that the Goetia of Astaroth returns to its reader as health (rounded down).</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="17" t="inlineStr">
+        <is>
+          <t>prm_recoil_damage</t>
+        </is>
+      </c>
+      <c r="B81" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C81" s="17" t="n"/>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>Weapons: HP The Lemegeton costs its reader each time they fight with it (never lethal: it stops at 1).</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage).</t>
         </is>
       </c>
     </row>
@@ -43095,7 +43623,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -43414,7 +43942,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U6" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -45381,7 +45909,7 @@
           <t>the south corridor (all movement, clear)|straight through the rubble (foot favored, hazardous)</t>
         </is>
       </c>
-      <c r="U33" t="inlineStr">
+      <c r="U33" s="17" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -45536,7 +46064,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="U35" t="inlineStr">
+      <c r="U35" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -45616,7 +46144,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="U36" t="inlineStr">
+      <c r="U36" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -45846,7 +46374,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="U39" s="17" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -46076,7 +46604,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U42" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>
@@ -46306,7 +46834,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="U45" s="17" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -46386,7 +46914,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U46" s="17" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -46461,7 +46989,7 @@
           <t>the plaza (foot, riding)|the covered market (blocks flying)|the silo blocks (impassable, all types)</t>
         </is>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="U47" s="17" t="inlineStr">
         <is>
           <t>b</t>
         </is>

</xml_diff>

<commit_message>
Add the mythic weapon tier and raise legendary above Silver
Legendary weapons now sit at 15-17 might (Silver is 13); a new mythic tier at
18-21, paragon wielders only, has one weapon per art: Marko's Claymore, Saint
George's Spear, Svarog's Cleaver, Rostam's Tamarisk Bow, Svyatogor's Grip, the
Lemegeton (moved up) and Slavonic Enoch. A boss may drop several weapons.
Validator checks the might ladder (c07s).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -1019,7 +1019,7 @@
           <t>Stands on the defend-point tile (D) -- literally where the crowd/townsfolk are.</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="17" t="inlineStr">
         <is>
           <t>wpn_zographos_codex</t>
         </is>
@@ -1614,7 +1614,7 @@
           <t>Same template, east crossing. Two instances of the same archetype, not two distinct characters -- consistent with nothing being named in the source text.</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
+      <c r="K17" s="17" t="inlineStr">
         <is>
           <t>wpn_perun_brand</t>
         </is>
@@ -3658,7 +3658,7 @@
       </c>
       <c r="K69" s="17" t="inlineStr">
         <is>
-          <t>wpn_axe_high</t>
+          <t>wpn_axe_high|wpn_stgeorge_spear</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="K71" s="17" t="inlineStr">
         <is>
-          <t>wpn_axe_high</t>
+          <t>wpn_axe_high|wpn_rostam_bow</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3786,7 @@
       </c>
       <c r="K72" s="17" t="inlineStr">
         <is>
-          <t>wpn_axe_high</t>
+          <t>wpn_axe_high|wpn_svyatogor_grip</t>
         </is>
       </c>
     </row>
@@ -4063,7 +4063,7 @@
       </c>
       <c r="K79" s="17" t="inlineStr">
         <is>
-          <t>wpn_lemegeton</t>
+          <t>wpn_astaroth_goetia</t>
         </is>
       </c>
     </row>
@@ -4138,7 +4138,7 @@
           <t>The looter ringleader exploiting the dockside unrest -- see chapters.ch_d04's own note on why the protesters themselves aren't combatants.</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
+      <c r="K81" s="17" t="inlineStr">
         <is>
           <t>wpn_morningstar</t>
         </is>
@@ -4251,7 +4251,7 @@
           <t>Scavengers picking through the ruin -- the renunciants who live here are not combatants, see chapters.ch_d07.</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
+      <c r="K84" s="17" t="inlineStr">
         <is>
           <t>wpn_neith_bow</t>
         </is>
@@ -4518,7 +4518,7 @@
           <t>Opportunists working the medicine trade, same framing as ch_d04's harbour.</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
+      <c r="K91" s="17" t="inlineStr">
         <is>
           <t>wpn_morningstar</t>
         </is>
@@ -4749,7 +4749,7 @@
           <t>Bandits using the treeline for cover, not an organized force.</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
+      <c r="K97" s="17" t="inlineStr">
         <is>
           <t>wpn_vila_moonbow</t>
         </is>
@@ -4790,7 +4790,7 @@
           <t>sect_march's own 'Prophecy NPCs convert green levies' -- levies mid-conversion.</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
+      <c r="K98" s="17" t="inlineStr">
         <is>
           <t>wpn_miroslav_gospel</t>
         </is>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="K101" s="17" t="inlineStr">
         <is>
-          <t>wpn_axe_high</t>
+          <t>wpn_axe_high|wpn_svarog_cleaver</t>
         </is>
       </c>
     </row>
@@ -4987,7 +4987,7 @@
       </c>
       <c r="K103" s="17" t="inlineStr">
         <is>
-          <t>wpn_astaroth_goetia</t>
+          <t>wpn_lemegeton</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="K107" s="17" t="inlineStr">
         <is>
-          <t>wpn_lance_high</t>
+          <t>wpn_lance_high|wpn_slavonic_enoch</t>
         </is>
       </c>
     </row>
@@ -5177,7 +5177,7 @@
       </c>
       <c r="K108" s="17" t="inlineStr">
         <is>
-          <t>wpn_sword_high</t>
+          <t>wpn_sword_high|wpn_marko_claymore</t>
         </is>
       </c>
     </row>
@@ -24943,7 +24943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="1" max="1"/>
@@ -26569,7 +26569,7 @@
         </is>
       </c>
       <c r="E33" s="17" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F33" s="17" t="n">
         <v>85</v>
@@ -26626,7 +26626,7 @@
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F34" s="17" t="n">
         <v>75</v>
@@ -26683,7 +26683,7 @@
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F35" s="17" t="n">
         <v>80</v>
@@ -26740,7 +26740,7 @@
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F36" s="17" t="n">
         <v>85</v>
@@ -26797,7 +26797,7 @@
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F37" s="17" t="n">
         <v>85</v>
@@ -26907,7 +26907,7 @@
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F39" s="17" t="n">
         <v>90</v>
@@ -26933,7 +26933,7 @@
         </is>
       </c>
       <c r="M39" s="17" t="n"/>
-      <c r="N39" t="inlineStr">
+      <c r="N39" s="17" t="inlineStr">
         <is>
           <t>flying</t>
         </is>
@@ -26965,7 +26965,7 @@
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F40" s="17" t="n">
         <v>95</v>
@@ -27018,7 +27018,7 @@
         </is>
       </c>
       <c r="E41" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F41" s="17" t="n">
         <v>85</v>
@@ -27075,7 +27075,7 @@
         </is>
       </c>
       <c r="E42" s="17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F42" s="17" t="n">
         <v>80</v>
@@ -27128,7 +27128,7 @@
         </is>
       </c>
       <c r="E43" s="17" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F43" s="17" t="n">
         <v>80</v>
@@ -27150,7 +27150,7 @@
       </c>
       <c r="L43" s="17" t="inlineStr">
         <is>
-          <t>DRAFTED 2026-10-22. Astaroth is the Lesser Key's duke of the knowledge of the past, a grandee of the underworld. An evil grimoire that feeds the reader: half the damage it deals comes back as health. Taken at the feeding of the Colossus.</t>
+          <t>DRAFTED 2026-10-22. Astaroth is the Lesser Key's duke of the knowledge of the past, a grandee of the underworld. An evil grimoire that feeds the reader: half the damage it deals comes back as health. Found in the Buried Works.</t>
         </is>
       </c>
       <c r="M43" s="17" t="n"/>
@@ -27181,11 +27181,11 @@
       </c>
       <c r="D44" s="17" t="inlineStr">
         <is>
-          <t>legendary</t>
+          <t>mythic</t>
         </is>
       </c>
       <c r="E44" s="17" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F44" s="17" t="n">
         <v>75</v>
@@ -27197,7 +27197,7 @@
         <v>9</v>
       </c>
       <c r="I44" s="17" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J44" s="17" t="n">
         <v>1</v>
@@ -27207,7 +27207,7 @@
       </c>
       <c r="L44" s="17" t="inlineStr">
         <is>
-          <t>DRAFTED 2026-10-22. The Lemegeton Clavicula Salomonis, the Lesser Key itself, holds the seventy-two spirits. The most powerful book in the game and it charges for it: the reader pays a little blood each time they open it (never enough to kill). Found in the Buried Works.</t>
+          <t>DRAFTED 2026-10-22, made MYTHIC 2026-10-23. The Lemegeton Clavicula Salomonis, the Lesser Key itself, holds the seventy-two spirits. The most dangerous book in the game and it charges for it: the reader pays a little blood each time they open it (never enough to kill). Taken at the feeding of the Colossus.</t>
         </is>
       </c>
       <c r="M44" s="17" t="n"/>
@@ -27222,6 +27222,333 @@
     </row>
     <row r="45">
       <c r="A45" s="17" t="inlineStr">
+        <is>
+          <t>wpn_marko_claymore</t>
+        </is>
+      </c>
+      <c r="B45" s="17" t="inlineStr">
+        <is>
+          <t>Marko's Claymore</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>sword</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E45" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="F45" s="17" t="n">
+        <v>70</v>
+      </c>
+      <c r="G45" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H45" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="I45" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J45" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L45" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. Kraljevic Marko is the Serbian folk hero of the Ottoman centuries, a giant of a man with a giant's sword who outlives every master. A great two-handed blade, too heavy for most hands: the biggest sword in the game and nothing else. Taken at the end of Act 2.</t>
+        </is>
+      </c>
+      <c r="M45" s="17" t="n"/>
+      <c r="O45" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" s="17" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>wpn_stgeorge_spear</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="inlineStr">
+        <is>
+          <t>Saint George's Spear</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>lance</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E46" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="F46" s="17" t="n">
+        <v>75</v>
+      </c>
+      <c r="G46" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="I46" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J46" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L46" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. Saint George is the dragon-slayer, patron of half the Balkans (Djurdjevdan, the spring feast). A spear that brings down what flies. Taken at the Reckoning.</t>
+        </is>
+      </c>
+      <c r="M46" s="17" t="n"/>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>flying</t>
+        </is>
+      </c>
+      <c r="O46" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P46" s="17" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="17" t="inlineStr">
+        <is>
+          <t>wpn_svarog_cleaver</t>
+        </is>
+      </c>
+      <c r="B47" s="17" t="inlineStr">
+        <is>
+          <t>Svarog's Cleaver</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E47" s="17" t="n">
+        <v>21</v>
+      </c>
+      <c r="F47" s="17" t="n">
+        <v>65</v>
+      </c>
+      <c r="G47" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="I47" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J47" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. Svarog is the Slavic smith and sky god, who forged the plough and the sword. The heaviest and hardest-hitting weapon in the game; few can swing it often. Taken in the Granary District of Kaisareia.</t>
+        </is>
+      </c>
+      <c r="M47" s="17" t="n"/>
+      <c r="O47" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" s="17" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>wpn_rostam_bow</t>
+        </is>
+      </c>
+      <c r="B48" s="17" t="inlineStr">
+        <is>
+          <t>Rostam's Tamarisk Bow</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E48" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F48" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="G48" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H48" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I48" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J48" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="K48" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="L48" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. Rostam, the hero of the Shahnameh, killed the invulnerable Esfandiyar with a tamarisk arrow shown him by the Simurgh. A bow that reaches three tiles with the power of a champion. Taken in the North Wind Winds.</t>
+        </is>
+      </c>
+      <c r="M48" s="17" t="n"/>
+      <c r="O48" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="17" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="17" t="inlineStr">
+        <is>
+          <t>wpn_svyatogor_grip</t>
+        </is>
+      </c>
+      <c r="B49" s="17" t="inlineStr">
+        <is>
+          <t>Svyatogor's Grip</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>brawl</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E49" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <v>80</v>
+      </c>
+      <c r="G49" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="H49" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="I49" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J49" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. Svyatogor is the Russian bylina giant so large the earth could not bear him, the elder of the bogatyrs. Gauntlets of a giant's strength. Taken at His Lake.</t>
+        </is>
+      </c>
+      <c r="M49" s="17" t="n"/>
+      <c r="O49" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" s="17" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>wpn_slavonic_enoch</t>
+        </is>
+      </c>
+      <c r="B50" s="17" t="inlineStr">
+        <is>
+          <t>Slavonic Enoch</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
+        <is>
+          <t>mythic</t>
+        </is>
+      </c>
+      <c r="E50" s="17" t="n">
+        <v>18</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <v>85</v>
+      </c>
+      <c r="G50" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="I50" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="J50" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L50" s="17" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-23. 2 Enoch survives only in Old Church Slavonic: a book of the heavens that the Balkans kept when no one else did. Every blow heals the allies beside its reader. Taken at the Throat Pass.</t>
+        </is>
+      </c>
+      <c r="M50" s="17" t="n"/>
+      <c r="O50" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P50" s="17" t="inlineStr">
+        <is>
+          <t>heal_allies</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft weapons table, review before treating as canon. Covers ordinary equipment only -- forges/materials' 5 legendary drops (3-of-5 cap) are a separate system above this tier, per forges' own note that the common smith 'arms lances and axes: the common soldier's tools, not the officer's.' Three tiers per art (basic/mid/high, flavor-named Iron/Steel/Silver) x 7 arts = 21 weapons. Might/hit/crit/weight/uses follow the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises) -- this design's own stated lineage per PROJECT_HANDOFF.md, not sourced from anything in canon.xlsx. Range: melee arts (sword/lance/axe/brawl) = 1, bow = 2, reason/faith = 1-2 (standard FE magic range). Names are placeholder and mechanical on purpose (e.g. 'Iron Tome', 'Iron Rite') -- real flavor-naming consistent with the setting's Byzantine/Near-East register is a writing pass for later, not attempted here. No weapon-rank/proficiency gating system exists yet (who can use which tier) -- units' single art_primary/secondary per class implicitly limits which art a unit fights with, but nothing yet gates basic vs. mid vs. high within that art. Drafted by a Claude Code session, 2026-09-16. ADDENDUM: 'worn' tier added below basic -- might 1, hit 55, one art each. Built for the prologue's conquered-army soldiers (enemy_archetypes.ea_conquered_soldier): veteran-level troops equipped with whatever's left after a siege, not a new balance tier anyone is meant to fight through progression. Numbers are a judgment call (roughly basic tier's might/hit at a fifth to two-thirds), not derived from anything in canon.xlsx. Drafted by a Claude Code session, 2026-09-16. ADDENDUM (2026-09-25): crit calibration pass. This row's own text already said crit 'follows the classic Fire Emblem Iron-Steel-Silver progression (might up, hit and durability down as tier rises)' but every weapon actually shipped with crit=0, flat across all 4 tiers -- never filled in despite the stated intent. Extended the same tier-scaling might/hit/weight/uses already use: worn=0, basic=0 (unchanged -- starter/scavenged gear staying crit-free matches genre convention), mid=5, high=10. Simulated the resulting crit_chance() output (weapon_crit + attacker.dex - defender.lck, this session's own 2026-09-25 formula calibration) against all 1,056 ordered unit/enemy attacker-defender combos per tier: basic/worn stays at the formula's own baseline (57.5% nonzero, mean 3.4%, max 21%); mid roughly doubles presence (86.8% nonzero, mean 7.1%, max 26%); high makes crit a real threat without ever approaching a coinflip (97.3% nonzero, mean 11.9%, max 31%, only 2 of 1,056 combos clear 30%). Kept the crit value uniform across all 7 arts, matching every other column on this table already being purely tier-based, not art-based -- nothing here or in canon.xlsx supports giving e.g. bows a crit edge over axes. ADDENDUM (2026-10-02): added req_arts (pipe-delimited arts a wielder must ALL be proficient in; blank = just the weapon's own art) and effective_vs (pipe-delimited movement types the weapon deals x2 might to), plus 3 overlap weapons (halberd, maul, censer). A weapon with 2+ req_arts is triangle-neutral. Attack speed = spd - max(0, weight - str) (mag for magic arts); a unit doubles at +4 speed. See combat.gd. ADDENDUM 2 (2026-10-03): added convoy_qty -- how many of each weapon the shared convoy holds at the start of a playthrough (one mid-tier weapon per art; the overlap weapons start at 0 and arrive as drops). Every unit also starts with the basic weapon of its art (Equipment.ensure_loadout). `uses` is now spent: 1 per strike made, the weapon breaks at 0, no repair (map_f00's design note). ADDENDUM (2026-10-17): the 'legendary' tier is the master smiths' work (forges/materials tabs): four weapons, one per usable Named material, never found or bought. effect = a special on-hit rule (heal_allies / unmake / pull); blank = none. Legendary weapons need a certified class like high-tier ones.</t>
         </is>

</xml_diff>

<commit_message>
Build the Skald: Edda's Refresh, Steal and Epithet Aura
Refresh (R) lets an adjacent ally who has acted act again; Steal (X) lifts an
adjacent non-boss enemy's weapon into the convoy and leaves it unarmed; the
Epithet Aura gives allies within two tiles +3 hit and avoid per earned deed, to
+9. Canon parameters, validator c07t, tests with a mutation pass.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -24370,7 +24370,11 @@
         </is>
       </c>
       <c r="G48" s="23" t="n"/>
-      <c r="H48" s="23" t="n"/>
+      <c r="H48" s="23" t="inlineStr">
+        <is>
+          <t>Epithet Aura</t>
+        </is>
+      </c>
       <c r="I48" s="23" t="inlineStr">
         <is>
           <t>no paperwork exists</t>
@@ -24378,7 +24382,12 @@
       </c>
       <c r="J48" s="23" t="inlineStr">
         <is>
-          <t>Edda; Refresh + Steal + epithet aura</t>
+          <t>Edda; Refresh + Steal + epithet aura. BUILT 2026-10-24 (SKALD_DESIGN.md): Refresh gives an adjacent ally who has acted another turn; Steal lifts an adjacent enemy's weapon (never a boss's) and leaves it unarmed; the Epithet Aura gives every ally near her a little hit and avoid for each deed they have earned.</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>refresh|steal</t>
         </is>
       </c>
     </row>
@@ -27321,7 +27330,7 @@
         </is>
       </c>
       <c r="M46" s="17" t="n"/>
-      <c r="N46" t="inlineStr">
+      <c r="N46" s="17" t="inlineStr">
         <is>
           <t>flying</t>
         </is>
@@ -36536,7 +36545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D82"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -37820,7 +37829,87 @@
     <row r="82">
       <c r="A82" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage).</t>
+          <t>prm_steal_base</t>
+        </is>
+      </c>
+      <c r="B82" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C82" s="17" t="n"/>
+      <c r="D82" s="17" t="inlineStr">
+        <is>
+          <t>Skald: percent chance a Steal succeeds against an enemy of equal speed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="17" t="inlineStr">
+        <is>
+          <t>prm_steal_per_spd</t>
+        </is>
+      </c>
+      <c r="B83" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C83" s="17" t="n"/>
+      <c r="D83" s="17" t="inlineStr">
+        <is>
+          <t>Skald: percentage points of Steal chance for each point of the Skald's speed over the enemy's (and minus for each under). Never below 5% or above 95%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>prm_aura_radius</t>
+        </is>
+      </c>
+      <c r="B84" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" s="17" t="n"/>
+      <c r="D84" s="17" t="inlineStr">
+        <is>
+          <t>Skald: tiles around her (Manhattan) in which the Epithet Aura reaches, herself included.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>prm_aura_per_deed</t>
+        </is>
+      </c>
+      <c r="B85" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C85" s="17" t="n"/>
+      <c r="D85" s="17" t="inlineStr">
+        <is>
+          <t>Skald: hit and avoid each ally in the aura gains for every deed (epithet) it has earned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>prm_aura_cap</t>
+        </is>
+      </c>
+      <c r="B86" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="C86" s="17" t="n"/>
+      <c r="D86" s="17" t="inlineStr">
+        <is>
+          <t>Skald: the most hit and avoid the aura can give one ally (three deeds' worth).</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap).</t>
         </is>
       </c>
     </row>
@@ -39497,7 +39586,7 @@
       </c>
       <c r="M32" s="17" t="inlineStr">
         <is>
-          <t>Canon note on Skald: 'epithet aura'.</t>
+          <t>Edda's own verse, a small extra on top of the real Epithet Aura she carries as a Skald (the class's aura, which lifts every ally near her by their deeds). Canon note on Skald: 'epithet aura'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the Martyr and the Quartermaster
Martyr (Anselm): Provoke (V) pulls every enemy that can reach him for one enemy
phase; Miracle leaves him at 1 HP once a map. Quartermaster: two column guests,
Wolfram and Hildegund (one per column), whose Supply (Q) hands an adjacent ally
the best convoy weapon it can wield. Guest machinery gains joins_after_map_id,
column and stats_like_unit_id; validator c07u.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -14672,7 +14672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="18" min="1" max="1"/>
@@ -14688,6 +14688,9 @@
     <col width="40" customWidth="1" style="18" min="11" max="11"/>
     <col width="18" customWidth="1" style="18" min="12" max="12"/>
     <col width="18" customWidth="1" style="18" min="13" max="13"/>
+    <col width="18" customWidth="1" style="18" min="14" max="14"/>
+    <col width="18" customWidth="1" style="18" min="15" max="15"/>
+    <col width="18" customWidth="1" style="18" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -14756,6 +14759,21 @@
           <t>depart_map_id</t>
         </is>
       </c>
+      <c r="N1" s="26" t="inlineStr">
+        <is>
+          <t>joins_after_map_id</t>
+        </is>
+      </c>
+      <c r="O1" s="26" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="P1" s="26" t="inlineStr">
+        <is>
+          <t>stats_like_unit_id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -14827,12 +14845,136 @@
     <row r="3">
       <c r="A3" s="17" t="inlineStr">
         <is>
-          <t>PRINCIPLE -- guest units exist to cover a class niche a scripted/conditional removal could zero out, without bending the departing character's own arc to protect roster math. Modeled on FFXII's guest-character pattern: narrative weight lives almost entirely outside combat tenure, not inside it. ADDENDUM (2026-10-18): requires_defections = every one of these must have happened (not merely one); depart_map_id = she leaves when that map is first won (the reunion: ch_rf20). She joins at the squad's median level less prm_guest_level_gap, fights with her class's basic art, earns no EXP and has no support chain.</t>
+          <t>gst_qm_a</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>Wolfram</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="17" t="inlineStr">
+        <is>
+          <t>cls_quartermaster</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>gp_frail_lucky</t>
+        </is>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>Joins once the company has won its first Act 1 map on either route (the supply train catches up). With the main column on every map except Column B's.</t>
+        </is>
+      </c>
+      <c r="G3" s="17" t="inlineStr">
+        <is>
+          <t>After map_d01 or map_a01 is won.</t>
+        </is>
+      </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>Never.</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>None: a non-combatant.</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17" t="n"/>
+      <c r="L3" s="17" t="n"/>
+      <c r="M3" s="17" t="n"/>
+      <c r="N3" s="17" t="inlineStr">
+        <is>
+          <t>map_d01|map_a01</t>
+        </is>
+      </c>
+      <c r="O3" s="17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="P3" s="17" t="inlineStr">
+        <is>
+          <t>u_kheldar</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>gst_qm_b</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Hildegund</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="n"/>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>cls_quartermaster</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>gp_frail_lucky</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Joins at the same time as Wolfram, but keeps the convoy for Column B: on a Column B map she is the quartermaster and Wolfram is not.</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>After map_d01 or map_a01 is won.</t>
+        </is>
+      </c>
+      <c r="H4" s="17" t="inlineStr">
+        <is>
+          <t>Never.</t>
+        </is>
+      </c>
+      <c r="I4" s="17" t="inlineStr">
+        <is>
+          <t>None: a non-combatant.</t>
+        </is>
+      </c>
+      <c r="J4" s="17" t="n"/>
+      <c r="K4" s="17" t="n"/>
+      <c r="L4" s="17" t="n"/>
+      <c r="M4" s="17" t="n"/>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>map_d01|map_a01</t>
+        </is>
+      </c>
+      <c r="O4" s="17" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="P4" s="17" t="inlineStr">
+        <is>
+          <t>u_kheldar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>PRINCIPLE -- guest units exist to cover a class niche a scripted/conditional removal could zero out, without bending the departing character's own arc to protect roster math. Modeled on FFXII's guest-character pattern: narrative weight lives almost entirely outside combat tenure, not inside it. ADDENDUM (2026-10-18): requires_defections = every one of these must have happened (not merely one); depart_map_id = she leaves when that map is first won (the reunion: ch_rf20). She joins at the squad's median level less prm_guest_level_gap, fights with her class's basic art, earns no EXP and has no support chain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>RECONSTRUCTED 2026-09-15 by a Claude Code session from a changelog summary of edits made in a separate Claude.ai session on this same workbook -- not copied verbatim from that session's actual file. Field text for trigger_condition/joins/departs/support_shape/off_screen_purpose_on_exit is a faithful reconstruction of what the changelog described; act3_payoff is a known gap (see that column's note). Verify against the source session if exact wording matters.</t>
         </is>
@@ -24282,7 +24424,11 @@
         </is>
       </c>
       <c r="G46" s="23" t="n"/>
-      <c r="H46" s="23" t="n"/>
+      <c r="H46" s="23" t="inlineStr">
+        <is>
+          <t>Convoy Keeper</t>
+        </is>
+      </c>
       <c r="I46" s="23" t="inlineStr">
         <is>
           <t>no paperwork exists</t>
@@ -24290,7 +24436,12 @@
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>Merlinus revival; one per column</t>
+          <t>Merlinus revival; one per column. BUILT 2026-10-25 as two GUESTS (Wolfram for the main column, Hildegund for Column B), not as roster units: a non-combatant who keeps the convoy. Supply hands an adjacent ally the best weapon in the convoy it can wield, and takes its old one back.</t>
+        </is>
+      </c>
+      <c r="L46" s="17" t="inlineStr">
+        <is>
+          <t>supply</t>
         </is>
       </c>
     </row>
@@ -24326,7 +24477,11 @@
         </is>
       </c>
       <c r="G47" s="23" t="n"/>
-      <c r="H47" s="23" t="n"/>
+      <c r="H47" s="23" t="inlineStr">
+        <is>
+          <t>Miracle</t>
+        </is>
+      </c>
       <c r="I47" s="23" t="inlineStr">
         <is>
           <t>no paperwork exists</t>
@@ -24334,7 +24489,12 @@
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>Provoke + Miracle + Resolve</t>
+          <t>Provoke + Miracle + Resolve. PLACED 2026-10-25 on Anselm (MARTYR_QUARTERMASTER_DESIGN.md). Provoke: for one enemy phase every enemy that can reach the Martyr must attack the Martyr. Miracle: once a map, a blow that would kill the Martyr leaves them at 1 HP. Resolve: stands firmer when hurt (the ability row).</t>
+        </is>
+      </c>
+      <c r="L47" s="17" t="inlineStr">
+        <is>
+          <t>provoke</t>
         </is>
       </c>
     </row>
@@ -24385,7 +24545,7 @@
           <t>Edda; Refresh + Steal + epithet aura. BUILT 2026-10-24 (SKALD_DESIGN.md): Refresh gives an adjacent ally who has acted another turn; Steal lifts an adjacent enemy's weapon (never a boss's) and leaves it unarmed; the Epithet Aura gives every ally near her a little hit and avoid for each deed they have earned.</t>
         </is>
       </c>
-      <c r="L48" t="inlineStr">
+      <c r="L48" s="17" t="inlineStr">
         <is>
           <t>refresh|steal</t>
         </is>
@@ -36545,7 +36705,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D87"/>
+  <dimension ref="A1:D88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -37909,7 +38069,23 @@
     <row r="87">
       <c r="A87" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap).</t>
+          <t>prm_miracle_per_map</t>
+        </is>
+      </c>
+      <c r="B87" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C87" s="17" t="n"/>
+      <c r="D87" s="17" t="inlineStr">
+        <is>
+          <t>Martyr: how many times on one map a blow that would kill a Martyr leaves them at 1 HP instead.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map.</t>
         </is>
       </c>
     </row>
@@ -42717,7 +42893,7 @@
       </c>
       <c r="G14" s="23" t="inlineStr">
         <is>
-          <t>cls_tr_faith</t>
+          <t>cls_martyr</t>
         </is>
       </c>
       <c r="H14" s="23" t="inlineStr">
@@ -43591,7 +43767,7 @@
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>trained</t>
+          <t>personal</t>
         </is>
       </c>
       <c r="D14" s="17" t="n">

</xml_diff>

<commit_message>
Build the standard forges and the requisition tier
Requisition tier 1-3 (tier 2 after the Second Writ, tier 3 after the Reunion) sets
how many standard orders may be open. The Diadem's and the Assembly's forges make
ordinary weapons for gold, ready after one newly won chapter, with 20% off their
house arts; silver is for tier 3. O on the overworld opens the requisitions
screen. Validator c07v.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -27734,7 +27734,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="17" min="1" max="1"/>
@@ -27748,6 +27748,7 @@
     <col width="16" customWidth="1" style="18" min="10" max="10"/>
     <col width="18" customWidth="1" style="18" min="11" max="11"/>
     <col width="10" customWidth="1" style="18" min="12" max="12"/>
+    <col width="26" customWidth="1" style="18" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1" s="18">
@@ -27811,6 +27812,11 @@
           <t>cycle_n</t>
         </is>
       </c>
+      <c r="M1" s="21" t="inlineStr">
+        <is>
+          <t>house_arts</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -27843,7 +27849,20 @@
       </c>
       <c r="I2" s="23" t="inlineStr">
         <is>
-          <t>the ordinary spine sidequest; no master required</t>
+          <t>the ordinary spine sidequest; no master required. BUILT 2026-10-26 (STANDARD_FORGES_DESIGN.md): orders of ordinary weapons for gold, one chapter, up to your requisition tier open at once, anywhere. The Diadem's house arts (cheaper here): sword, lance, reason, faith -- the capital's library and armories.</t>
+        </is>
+      </c>
+      <c r="K2" s="17" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="L2" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="17" t="inlineStr">
+        <is>
+          <t>sword|lance|reason|faith</t>
         </is>
       </c>
     </row>
@@ -27878,7 +27897,20 @@
       </c>
       <c r="I3" s="23" t="inlineStr">
         <is>
-          <t>the ordinary spine sidequest; no master required</t>
+          <t>the ordinary spine sidequest; no master required. BUILT 2026-10-26 (STANDARD_FORGES_DESIGN.md): the same orders at the Assembly's forge. Its house arts (cheaper here): axe, bow, brawl -- timber, horse-country and the lake towns.</t>
+        </is>
+      </c>
+      <c r="K3" s="17" t="inlineStr">
+        <is>
+          <t>always</t>
+        </is>
+      </c>
+      <c r="L3" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="17" t="inlineStr">
+        <is>
+          <t>axe|bow|brawl</t>
         </is>
       </c>
     </row>
@@ -36705,7 +36737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D88"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38085,7 +38117,111 @@
     <row r="88">
       <c r="A88" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map.</t>
+          <t>prm_requisition_tier_2</t>
+        </is>
+      </c>
+      <c r="B88" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C88" s="17" t="inlineStr">
+        <is>
+          <t>map_x11</t>
+        </is>
+      </c>
+      <c r="D88" s="17" t="inlineStr">
+        <is>
+          <t>Requisition tier 2 (two open orders) once this map is won: the Second Writ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="17" t="inlineStr">
+        <is>
+          <t>prm_requisition_tier_3</t>
+        </is>
+      </c>
+      <c r="B89" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C89" s="17" t="inlineStr">
+        <is>
+          <t>map_rf20</t>
+        </is>
+      </c>
+      <c r="D89" s="17" t="inlineStr">
+        <is>
+          <t>Requisition tier 3 (three open orders, and silver weapons) once this map is won: the Reunion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t>prm_standard_cost_basic</t>
+        </is>
+      </c>
+      <c r="B90" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C90" s="17" t="n"/>
+      <c r="D90" s="17" t="inlineStr">
+        <is>
+          <t>Standard forge: gold for a basic (iron) weapon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="17" t="inlineStr">
+        <is>
+          <t>prm_standard_cost_mid</t>
+        </is>
+      </c>
+      <c r="B91" s="17" t="n">
+        <v>300</v>
+      </c>
+      <c r="C91" s="17" t="n"/>
+      <c r="D91" s="17" t="inlineStr">
+        <is>
+          <t>Standard forge: gold for a mid (steel) weapon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="17" t="inlineStr">
+        <is>
+          <t>prm_standard_cost_high</t>
+        </is>
+      </c>
+      <c r="B92" s="17" t="n">
+        <v>800</v>
+      </c>
+      <c r="C92" s="17" t="n"/>
+      <c r="D92" s="17" t="inlineStr">
+        <is>
+          <t>Standard forge: gold for a high (silver) weapon, which needs requisition tier 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="17" t="inlineStr">
+        <is>
+          <t>prm_standard_house_discount_pct</t>
+        </is>
+      </c>
+      <c r="B93" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="C93" s="17" t="n"/>
+      <c r="D93" s="17" t="inlineStr">
+        <is>
+          <t>Standard forge: percent off the weapons of that forge's house arts (forges.house_arts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build mounts and Named riding
Canon-first mounts tab (Warhorse plus the Simurgh, Shadhavar, Karkadann, Anzu), a Mounts
autoload, barracks Mount mode, intact capture of a Named, Warhorse requisition and capture,
rider-fell fate, and map effects for each Named mount.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -26,38 +26,39 @@
     <sheet name="validation" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="regions" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="named" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="states" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="defections" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="guest_units" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="locations" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="polities" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="settlements" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="eras" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="flashbacks" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="prologue_roster" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="prologue_structures" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="prologue_tuning" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="signs" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="calendar" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="practices" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="the_claimant" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="the_hierophant" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="roster_gaps" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="canon_flags" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="epilogue_generation" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="epilogue_text" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="weapons" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="forges" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="materials" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="christian_allegory" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="ascension_signals" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="endings" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="naming_reference" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="supports" sheetId="47" state="visible" r:id="rId47"/>
-    <sheet name="promotion_rules" sheetId="48" state="visible" r:id="rId48"/>
-    <sheet name="abilities" sheetId="49" state="visible" r:id="rId49"/>
-    <sheet name="world_paths" sheetId="50" state="visible" r:id="rId50"/>
-    <sheet name="cargo_units" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="mounts" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="states" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="defections" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="guest_units" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="locations" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="polities" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="settlements" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="eras" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="flashbacks" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="prologue_roster" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="prologue_structures" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="prologue_tuning" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet name="signs" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="calendar" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet name="practices" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="the_claimant" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="the_hierophant" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="roster_gaps" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="canon_flags" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="epilogue_generation" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="epilogue_text" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="weapons" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="forges" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="materials" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="christian_allegory" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="ascension_signals" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="endings" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="naming_reference" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="supports" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="promotion_rules" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="abilities" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="world_paths" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="cargo_units" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -14240,6 +14241,252 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="18" min="1" max="1"/>
+    <col width="16" customWidth="1" style="18" min="2" max="2"/>
+    <col width="80" customWidth="1" style="18" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>mount_id</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>kind</t>
+        </is>
+      </c>
+      <c r="D1" s="26" t="inlineStr">
+        <is>
+          <t>named_id</t>
+        </is>
+      </c>
+      <c r="E1" s="26" t="inlineStr">
+        <is>
+          <t>movement</t>
+        </is>
+      </c>
+      <c r="F1" s="26" t="inlineStr">
+        <is>
+          <t>effect</t>
+        </is>
+      </c>
+      <c r="G1" s="26" t="inlineStr">
+        <is>
+          <t>requisition_cost</t>
+        </is>
+      </c>
+      <c r="H1" s="26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>mnt_warhorse</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Warhorse</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>horse</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>riding</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>400</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>DRAFTED 2026-10-27. The ordinary mount: acquired by requisition (the standard forges' orders), by capturing a mounted enemy, or by inheritance (a fallen rider's, if it is recovered). Grants riding movement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>mnt_simurgh</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>the Simurgh</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>named</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nmd_simurgh</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>flying</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>rider_heal</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Canon: 5 HP/turn to rider and adjacent allies (flat, not percentage). Taken intact from the Simurgh's paralogue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mnt_shadhavar</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>the Shadhavar</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>named</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nmd_shadhavar</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>riding</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>pull_foe</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Canon: every turn, pulls the nearest enemy one tile toward the rider; CANNOT be turned off. A liability on escort maps, an asset on defend maps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>mnt_karkadann</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>the Karkadann</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>named</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nmd_karkadann</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>riding</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>charge</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Canon: strong against mounted units; a devastating charge that leaves it stuck one turn. The plain one on purpose.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>mnt_anzu</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>the Anzu</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>named</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nmd_anzu</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>flying</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>unmake_touch</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Canon: contact degrades enemy weapons; only bites what is already worn; broken means unarmed, not dead. COST: an enemy it has left unarmed drops nothing, so riding it starves your only supply line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MOUNTS (drafted 2026-10-27, MOUNTS_DESIGN.md). Canon (roster_gaps): mounts are acquirable equipment (capture / inheritance / requisition), not a class trait -- any of the 18 can end up mounted. A mount gives its rider its movement type (riding or flying) and, for a Named, its signature mechanic. The Huma is a map hazard, not a mount, and has no row. Declared gaps hold: brawl cannot ride or fly, reason cannot fly (see canon_validate DECLARED_GAPS); a unit that already moves as riding, flying or armor takes no mount. The three-way capture of a Named: killed (a prime material), captured at or below capture_hp_pct (a diminished material, a harvest), captured at or below capture_intact_hp_pct (the Named itself, INTACT, as a mount).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
@@ -14380,7 +14627,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14666,7 +14913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14985,7 +15232,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -16609,7 +16856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17101,7 +17348,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17804,7 +18051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18102,7 +18349,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18364,7 +18611,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19176,190 +19423,6 @@
       <c r="A14" s="17" t="inlineStr">
         <is>
           <t>NOTE -- weapon_art/str/mag/dex/spd/lck/def/res added. weapon_art is read straight off each unit's own 'role' text (e.g. pu_kadar's role is literally 'axe'); pu_nashar is null, matching his existing 'cannot attack' / dmg_vs_statue=0. The 7 numeric stats are NOT newly invented numbers -- all 7 combat-capable units reuse the exact 'trained' tier baseline already established in unit_base_stats/enemy_archetypes generation (identical to ea_relic_hunter's own stats, since enemies get baseline alone with no growth bonus), with str/mag swapped for the two magic-art units (Enmet, Ilat) the same way trained-tier player mages already skew mag over str (see u_emmerich/u_anselm in unit_base_stats). hp and dmg_vs_statue are untouched. This exists to let real unit-vs-unit combat run on this roster at all -- previously only move/hp/dmg_vs_statue existed, nothing Combat.gd could use. Added for the F0 garrison-soldier fight; review/replace freely if named per-unit stats are ever written. Drafted by a Claude Code session, 2026-09-16.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="15" customWidth="1" style="17" min="1" max="1"/>
-    <col width="22" customWidth="1" style="17" min="2" max="2"/>
-    <col width="17" customWidth="1" style="17" min="3" max="3"/>
-    <col width="8" customWidth="1" style="17" min="4" max="4"/>
-    <col width="9" customWidth="1" style="17" min="5" max="5"/>
-    <col width="12" customWidth="1" style="17" min="6" max="6"/>
-    <col width="22" customWidth="1" style="17" min="7" max="7"/>
-    <col width="62" customWidth="1" style="17" min="8" max="8"/>
-    <col width="46" customWidth="1" style="17" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1" s="18">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>structure_id</t>
-        </is>
-      </c>
-      <c r="B1" s="21" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="21" t="inlineStr">
-        <is>
-          <t>turns_to_destroy</t>
-        </is>
-      </c>
-      <c r="D1" s="21" t="inlineStr">
-        <is>
-          <t>hp</t>
-        </is>
-      </c>
-      <c r="E1" s="21" t="inlineStr">
-        <is>
-          <t>defence</t>
-        </is>
-      </c>
-      <c r="F1" s="21" t="inlineStr">
-        <is>
-          <t>retaliates</t>
-        </is>
-      </c>
-      <c r="G1" s="21" t="inlineStr">
-        <is>
-          <t>requires_multiple_units</t>
-        </is>
-      </c>
-      <c r="H1" s="21" t="inlineStr">
-        <is>
-          <t>behaviour</t>
-        </is>
-      </c>
-      <c r="I1" s="21" t="inlineStr">
-        <is>
-          <t>what_it_argues</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="23.85" customHeight="1" s="18">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>str_wall</t>
-        </is>
-      </c>
-      <c r="B2" s="23" t="inlineStr">
-        <is>
-          <t>The river wall</t>
-        </is>
-      </c>
-      <c r="C2" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D2" s="23" t="n">
-        <v>400</v>
-      </c>
-      <c r="E2" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G2" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="H2" s="23" t="inlineStr">
-        <is>
-          <t>Enmet removes it in one cast on turn 1; 40 tiles of masonry, a generation to build</t>
-        </is>
-      </c>
-      <c r="I2" s="23" t="inlineStr">
-        <is>
-          <t>SPECTACLE: instant, and it takes one gifted person</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="23.85" customHeight="1" s="18">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>str_statue</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="inlineStr">
-        <is>
-          <t>The patron's image</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="23" t="n">
-        <v>340</v>
-      </c>
-      <c r="E3" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" s="23" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="G3" s="23" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="H3" s="23" t="inlineStr">
-        <is>
-          <t>no defence, no retaliation, cannot be one-shot by anyone; every unit must walk up and hit it</t>
-        </is>
-      </c>
-      <c r="I3" s="23" t="inlineStr">
-        <is>
-          <t>EROSION: slow, communal, boring, and it needs everybody's hands on it</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="18">
-      <c r="A5" s="25" t="inlineStr">
-        <is>
-          <t>The inversion IS the prologue. Military conquest is instant and spectacular. Cultural erasure is slow and takes the whole warband. No cutscene explains this; the numbers do. Do not let one unit finish the statue.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="18">
-      <c r="A8" s="25" t="inlineStr">
-        <is>
-          <t>The image is broken before the name is written, and the name is never shown. Order matters: you</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="18">
-      <c r="A9" s="25" t="inlineStr">
-        <is>
-          <t>cannot write down a god that people can still see, and the player cannot be told what a god is</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="18">
-      <c r="A10" s="25" t="inlineStr">
-        <is>
-          <t>called and still share the world's ignorance.</t>
         </is>
       </c>
     </row>
@@ -19713,6 +19776,190 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="15" customWidth="1" style="17" min="1" max="1"/>
+    <col width="22" customWidth="1" style="17" min="2" max="2"/>
+    <col width="17" customWidth="1" style="17" min="3" max="3"/>
+    <col width="8" customWidth="1" style="17" min="4" max="4"/>
+    <col width="9" customWidth="1" style="17" min="5" max="5"/>
+    <col width="12" customWidth="1" style="17" min="6" max="6"/>
+    <col width="22" customWidth="1" style="17" min="7" max="7"/>
+    <col width="62" customWidth="1" style="17" min="8" max="8"/>
+    <col width="46" customWidth="1" style="17" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="18">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>structure_id</t>
+        </is>
+      </c>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>turns_to_destroy</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>defence</t>
+        </is>
+      </c>
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>retaliates</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
+        <is>
+          <t>requires_multiple_units</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>behaviour</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>what_it_argues</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="23.85" customHeight="1" s="18">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>str_wall</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>The river wall</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="23" t="n">
+        <v>400</v>
+      </c>
+      <c r="E2" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G2" s="23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H2" s="23" t="inlineStr">
+        <is>
+          <t>Enmet removes it in one cast on turn 1; 40 tiles of masonry, a generation to build</t>
+        </is>
+      </c>
+      <c r="I2" s="23" t="inlineStr">
+        <is>
+          <t>SPECTACLE: instant, and it takes one gifted person</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="23.85" customHeight="1" s="18">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>str_statue</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="inlineStr">
+        <is>
+          <t>The patron's image</t>
+        </is>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" s="23" t="n">
+        <v>340</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="23" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G3" s="23" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H3" s="23" t="inlineStr">
+        <is>
+          <t>no defence, no retaliation, cannot be one-shot by anyone; every unit must walk up and hit it</t>
+        </is>
+      </c>
+      <c r="I3" s="23" t="inlineStr">
+        <is>
+          <t>EROSION: slow, communal, boring, and it needs everybody's hands on it</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="18">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>The inversion IS the prologue. Military conquest is instant and spectacular. Cultural erasure is slow and takes the whole warband. No cutscene explains this; the numbers do. Do not let one unit finish the statue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="18">
+      <c r="A8" s="25" t="inlineStr">
+        <is>
+          <t>The image is broken before the name is written, and the name is never shown. Order matters: you</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="18">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
+          <t>cannot write down a god that people can still see, and the player cannot be told what a god is</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="18">
+      <c r="A10" s="25" t="inlineStr">
+        <is>
+          <t>called and still share the world's ignorance.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
@@ -19876,7 +20123,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20448,7 +20695,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20645,7 +20892,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20888,7 +21135,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21032,7 +21279,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21119,7 +21366,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21225,7 +21472,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21336,7 +21583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21570,576 +21817,6 @@
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="30" customWidth="1" style="18" min="1" max="1"/>
-    <col width="60" customWidth="1" style="18" min="2" max="2"/>
-    <col width="70" customWidth="1" style="18" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>phrase_id</t>
-        </is>
-      </c>
-      <c r="B1" s="26" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="C1" s="26" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="17" t="inlineStr">
-        <is>
-          <t>epi_head</t>
-        </is>
-      </c>
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>{NAME}, {TITLE}, fell at {PLACE}</t>
-        </is>
-      </c>
-      <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>opening clause when the unit holds an epithet</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>epi_head_plain</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>{NAME} fell at {PLACE}</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
-        <is>
-          <t>opening clause for someone plain -- the name stands alone</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
-        <is>
-          <t>epi_tail_known</t>
-        </is>
-      </c>
-      <c r="B4" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> to {KILLER}</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="inlineStr">
-        <is>
-          <t>killer clause tail for any named or factional killer</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="17" t="inlineStr">
-        <is>
-          <t>epi_tail_unknown</t>
-        </is>
-      </c>
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>, in the chaos, to no blade anyone could name</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="inlineStr">
-        <is>
-          <t>reserved for routs and unwitnessed deaths; bleaker than a named killer, not vaguer</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="17" t="inlineStr">
-        <is>
-          <t>epi_tail_hazard</t>
-        </is>
-      </c>
-      <c r="B6" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"> to {HAZARD}</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>a death with no hand in it (extension to the enum: killed_by_type hazard)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>epi_hazard_cold</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>the cold</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
-        <is>
-          <t>hazard names, keyed epi_hazard_&lt;id&gt;</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
-        <is>
-          <t>epi_killer_polity</t>
-        </is>
-      </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>{A} {ADJ} {NOUN}</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
-        <is>
-          <t>faction, not a person: a Diadem lance, an Assembly arrow</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
-        <is>
-          <t>epi_killer_band</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>{A} {WHO}'s {NOUN}</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="inlineStr">
-        <is>
-          <t>an unaffiliated armed band, or a soldier whose map names no polity (extension: killed_by_type band)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
-        <is>
-          <t>epi_killer_named</t>
-        </is>
-      </c>
-      <c r="B10" s="17" t="inlineStr">
-        <is>
-          <t>{PHRASE}</t>
-        </is>
-      </c>
-      <c r="C10" s="17" t="inlineStr">
-        <is>
-          <t>the Named creature signature verb (named.death_phrase)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
-        <is>
-          <t>epi_killer_defector</t>
-        </is>
-      </c>
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>{DEFECTOR}</t>
-        </is>
-      </c>
-      <c r="C11" s="17" t="inlineStr">
-        <is>
-          <t>a defector is named directly</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
-        <is>
-          <t>epi_killer_boss</t>
-        </is>
-      </c>
-      <c r="B12" s="17" t="inlineStr">
-        <is>
-          <t>{BOSS}</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>a chapter boss is named directly</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>epi_title_slayer_of</t>
-        </is>
-      </c>
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>{TOKEN} {OBJECT}</t>
-        </is>
-      </c>
-      <c r="C13" s="17" t="inlineStr">
-        <is>
-          <t>forge_vocab_token ending in "of" takes the thing slain</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
-        <is>
-          <t>epi_title_slayer_fallback</t>
-        </is>
-      </c>
-      <c r="B14" s="17" t="inlineStr">
-        <is>
-          <t>the Slayer</t>
-        </is>
-      </c>
-      <c r="C14" s="17" t="inlineStr">
-        <is>
-          <t>when the deed was earned but the quarry was not recorded</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
-        <is>
-          <t>epi_title_the</t>
-        </is>
-      </c>
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>the {TOKEN}</t>
-        </is>
-      </c>
-      <c r="C15" s="17" t="inlineStr">
-        <is>
-          <t>a bare forge_vocab_token: the Untouched</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="17" t="inlineStr">
-        <is>
-          <t>epi_weapon_lost_to_enemy</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="inlineStr">
-        <is>
-          <t>The {WEAPON} passed to no one.</t>
-        </is>
-      </c>
-      <c r="C16" s="17" t="inlineStr">
-        <is>
-          <t>weapon_fate lost_to_enemy</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>epi_weapon_retrieved</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>The {WEAPON} came home in the convoy.</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>weapon_fate retrieved</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>epi_weapon_thrown_and_lost</t>
-        </is>
-      </c>
-      <c r="B18" s="17" t="inlineStr">
-        <is>
-          <t>The {WEAPON} was thrown, and not found again.</t>
-        </is>
-      </c>
-      <c r="C18" s="17" t="inlineStr">
-        <is>
-          <t>weapon_fate thrown_and_lost</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="17" t="inlineStr">
-        <is>
-          <t>epi_weapon_with_the_body</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>{NAME} was buried still holding the {WEAPON}.</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>weapon_fate with_the_body</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_platonic_C</t>
-        </is>
-      </c>
-      <c r="B20" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} knew {NAME} only a little, and said so.</t>
-        </is>
-      </c>
-      <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>platonic, tier C</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_platonic_B</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} kept {NAME}'s watch that night.</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
-        <is>
-          <t>platonic, tier B</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_platonic_A</t>
-        </is>
-      </c>
-      <c r="B22" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} carried {NAME}'s name into every fight after.</t>
-        </is>
-      </c>
-      <c r="C22" s="17" t="inlineStr">
-        <is>
-          <t>platonic, tier A</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_romantic_C</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} had meant to say something, and did not.</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>romantic, tier C</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_romantic_B</t>
-        </is>
-      </c>
-      <c r="B24" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} sat with the body until morning.</t>
-        </is>
-      </c>
-      <c r="C24" s="17" t="inlineStr">
-        <is>
-          <t>romantic, tier B</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_romantic_A</t>
-        </is>
-      </c>
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} would not speak of it.</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>romantic, tier A</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_romantic_S</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} stayed on the field until someone made them leave.</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>romantic, tier S</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_gone</t>
-        </is>
-      </c>
-      <c r="B27" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} was gone from the company by then.</t>
-        </is>
-      </c>
-      <c r="C27" s="17" t="inlineStr">
-        <is>
-          <t>the partner had defected or departed</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_fallen_before</t>
-        </is>
-      </c>
-      <c r="B28" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} had fallen already, and there was no one left to grieve.</t>
-        </is>
-      </c>
-      <c r="C28" s="17" t="inlineStr">
-        <is>
-          <t>the partner died earlier</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_fallen_after</t>
-        </is>
-      </c>
-      <c r="B29" s="17" t="inlineStr">
-        <is>
-          <t>{PARTNER} did not outlive the war either.</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="inlineStr">
-        <is>
-          <t>the partner died later</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>epi_support_alone</t>
-        </is>
-      </c>
-      <c r="B30" s="17" t="inlineStr">
-        <is>
-          <t>No one at the fire was close enough to grieve properly.</t>
-        </is>
-      </c>
-      <c r="C30" s="17" t="inlineStr">
-        <is>
-          <t>unpaired: a quiet indictment of a run that never built the relationship</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="17" t="inlineStr">
-        <is>
-          <t>epi_roll_title</t>
-        </is>
-      </c>
-      <c r="B31" s="17" t="inlineStr">
-        <is>
-          <t>The Fallen</t>
-        </is>
-      </c>
-      <c r="C31" s="17" t="inlineStr">
-        <is>
-          <t>heading of the fallen roll</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>epi_roll_empty</t>
-        </is>
-      </c>
-      <c r="B32" s="17" t="inlineStr">
-        <is>
-          <t>No one has fallen. Yet.</t>
-        </is>
-      </c>
-      <c r="C32" s="17" t="inlineStr">
-        <is>
-          <t>the roll when it is empty</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="17" t="inlineStr">
-        <is>
-          <t>IMPLEMENTATION NOTES (2026-10-09). The text of epilogue_generation, built as scripts/epilogue.gd. Wording is DRAFT; placeholders in {BRACES} are filled by the generator, and {A} becomes 'a' or 'an' by the word after it. No line uses a pronoun for the fallen or the partner -- they/them is avoided by naming. TWO EXTENSIONS to the killed_by_type enum, which the original schema did not list: 'band' (an unaffiliated armed band -- looters, relic hunters, privateers, or a soldier on a map that names no polity) and 'hazard' (a death with no hand in it: the cold on map_a03). maps.enemy_polity_id is a DRAFT: state-affiliated enemies belong to the polity opposite the chapter's route (a Diadem-route map fields Assembly soldiers); both-route maps name none, so those soldiers read as a band. Tune it map by map. ADDENDUM (2026-10-20): {WEAPON} is the weapon's provenance name (epithets.weapon_form), which may already read as a possessive ("Taker's Iron Axe"), so the weapon lines say 'The {WEAPON}' rather than '{NAME}'s {WEAPON}'.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -25112,6 +24789,576 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" style="18" min="1" max="1"/>
+    <col width="60" customWidth="1" style="18" min="2" max="2"/>
+    <col width="70" customWidth="1" style="18" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="26" t="inlineStr">
+        <is>
+          <t>phrase_id</t>
+        </is>
+      </c>
+      <c r="B1" s="26" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="C1" s="26" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>epi_head</t>
+        </is>
+      </c>
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>{NAME}, {TITLE}, fell at {PLACE}</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="inlineStr">
+        <is>
+          <t>opening clause when the unit holds an epithet</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
+        <is>
+          <t>epi_head_plain</t>
+        </is>
+      </c>
+      <c r="B3" s="17" t="inlineStr">
+        <is>
+          <t>{NAME} fell at {PLACE}</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>opening clause for someone plain -- the name stands alone</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>epi_tail_known</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> to {KILLER}</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>killer clause tail for any named or factional killer</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>epi_tail_unknown</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>, in the chaos, to no blade anyone could name</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>reserved for routs and unwitnessed deaths; bleaker than a named killer, not vaguer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>epi_tail_hazard</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> to {HAZARD}</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>a death with no hand in it (extension to the enum: killed_by_type hazard)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>epi_hazard_cold</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>the cold</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>hazard names, keyed epi_hazard_&lt;id&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>epi_killer_polity</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>{A} {ADJ} {NOUN}</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>faction, not a person: a Diadem lance, an Assembly arrow</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>epi_killer_band</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>{A} {WHO}'s {NOUN}</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>an unaffiliated armed band, or a soldier whose map names no polity (extension: killed_by_type band)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
+        <is>
+          <t>epi_killer_named</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>{PHRASE}</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>the Named creature signature verb (named.death_phrase)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
+        <is>
+          <t>epi_killer_defector</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>{DEFECTOR}</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>a defector is named directly</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
+        <is>
+          <t>epi_killer_boss</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>{BOSS}</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>a chapter boss is named directly</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t>epi_title_slayer_of</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>{TOKEN} {OBJECT}</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>forge_vocab_token ending in "of" takes the thing slain</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
+        <is>
+          <t>epi_title_slayer_fallback</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>the Slayer</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>when the deed was earned but the quarry was not recorded</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>epi_title_the</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>the {TOKEN}</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>a bare forge_vocab_token: the Untouched</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>epi_weapon_lost_to_enemy</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} passed to no one.</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>weapon_fate lost_to_enemy</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="17" t="inlineStr">
+        <is>
+          <t>epi_weapon_retrieved</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} came home in the convoy.</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>weapon_fate retrieved</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="17" t="inlineStr">
+        <is>
+          <t>epi_weapon_thrown_and_lost</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>The {WEAPON} was thrown, and not found again.</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>weapon_fate thrown_and_lost</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>epi_weapon_with_the_body</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>{NAME} was buried still holding the {WEAPON}.</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>weapon_fate with_the_body</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_platonic_C</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} knew {NAME} only a little, and said so.</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>platonic, tier C</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_platonic_B</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} kept {NAME}'s watch that night.</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>platonic, tier B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_platonic_A</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} carried {NAME}'s name into every fight after.</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>platonic, tier A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_romantic_C</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} had meant to say something, and did not.</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>romantic, tier C</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_romantic_B</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} sat with the body until morning.</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>romantic, tier B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_romantic_A</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} would not speak of it.</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>romantic, tier A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_romantic_S</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} stayed on the field until someone made them leave.</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>romantic, tier S</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_gone</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} was gone from the company by then.</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>the partner had defected or departed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_fallen_before</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} had fallen already, and there was no one left to grieve.</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>the partner died earlier</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_fallen_after</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="inlineStr">
+        <is>
+          <t>{PARTNER} did not outlive the war either.</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>the partner died later</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="inlineStr">
+        <is>
+          <t>epi_support_alone</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>No one at the fire was close enough to grieve properly.</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>unpaired: a quiet indictment of a run that never built the relationship</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>epi_roll_title</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>The Fallen</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>heading of the fallen roll</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>epi_roll_empty</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>No one has fallen. Yet.</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>the roll when it is empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>IMPLEMENTATION NOTES (2026-10-09). The text of epilogue_generation, built as scripts/epilogue.gd. Wording is DRAFT; placeholders in {BRACES} are filled by the generator, and {A} becomes 'a' or 'an' by the word after it. No line uses a pronoun for the fallen or the partner -- they/them is avoided by naming. TWO EXTENSIONS to the killed_by_type enum, which the original schema did not list: 'band' (an unaffiliated armed band -- looters, relic hunters, privateers, or a soldier on a map that names no polity) and 'hazard' (a death with no hand in it: the cold on map_a03). maps.enemy_polity_id is a DRAFT: state-affiliated enemies belong to the polity opposite the chapter's route (a Diadem-route map fields Assembly soldiers); both-route maps name none, so those soldiers read as a band. Tune it map by map. ADDENDUM (2026-10-20): {WEAPON} is the weapon's provenance name (epithets.weapon_form), which may already read as a possessive ("Taker's Iron Axe"), so the weapon lines say 'The {WEAPON}' rather than '{NAME}'s {WEAPON}'.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:P51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -27728,7 +27975,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28108,7 +28355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28375,7 +28622,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28628,7 +28875,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28789,7 +29036,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29012,7 +29259,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -29363,7 +29610,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -36731,13 +36978,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D94"/>
+  <dimension ref="A1:D99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38221,7 +38468,87 @@
     <row r="94">
       <c r="A94" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters.</t>
+          <t>prm_capture_intact_hp_pct</t>
+        </is>
+      </c>
+      <c r="B94" s="17" t="n">
+        <v>25</v>
+      </c>
+      <c r="C94" s="17" t="n"/>
+      <c r="D94" s="17" t="inlineStr">
+        <is>
+          <t>Mounts: a Named creature captured at or below this percent of its max HP is taken INTACT (a mount); between this and capture_hp_pct it is harvested for a diminished material.</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="17" t="inlineStr">
+        <is>
+          <t>prm_mount_heal</t>
+        </is>
+      </c>
+      <c r="B95" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C95" s="17" t="n"/>
+      <c r="D95" s="17" t="inlineStr">
+        <is>
+          <t>Mounts: HP the Simurgh restores at the start of each of your turns to its rider and every ally beside them (canon: 5 flat).</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t>prm_charge_distance</t>
+        </is>
+      </c>
+      <c r="B96" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C96" s="17" t="n"/>
+      <c r="D96" s="17" t="inlineStr">
+        <is>
+          <t>Mounts: tiles the Karkadann's rider must have moved this turn for the charge to count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="inlineStr">
+        <is>
+          <t>prm_charge_bonus</t>
+        </is>
+      </c>
+      <c r="B97" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C97" s="17" t="n"/>
+      <c r="D97" s="17" t="inlineStr">
+        <is>
+          <t>Mounts: damage added to the Karkadann rider's attack after a charge; the rider is then stuck (cannot move) on their next turn.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="17" t="inlineStr">
+        <is>
+          <t>prm_mount_capture_per_map</t>
+        </is>
+      </c>
+      <c r="B98" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" s="17" t="n"/>
+      <c r="D98" s="17" t="inlineStr">
+        <is>
+          <t>Mounts: the most Warhorses one map's captures of mounted enemies can bring in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map).</t>
         </is>
       </c>
     </row>
@@ -38230,7 +38557,427 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A1:J13"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="16" customWidth="1" style="17" min="1" max="1"/>
+    <col width="8" customWidth="1" style="17" min="2" max="9"/>
+    <col width="13" customWidth="1" style="17" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="18">
+      <c r="A1" s="21" t="inlineStr">
+        <is>
+          <t>profile_id</t>
+        </is>
+      </c>
+      <c r="B1" s="21" t="inlineStr">
+        <is>
+          <t>hp</t>
+        </is>
+      </c>
+      <c r="C1" s="21" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="D1" s="21" t="inlineStr">
+        <is>
+          <t>mag</t>
+        </is>
+      </c>
+      <c r="E1" s="21" t="inlineStr">
+        <is>
+          <t>dex</t>
+        </is>
+      </c>
+      <c r="F1" s="21" t="inlineStr">
+        <is>
+          <t>spd</t>
+        </is>
+      </c>
+      <c r="G1" s="21" t="inlineStr">
+        <is>
+          <t>lck</t>
+        </is>
+      </c>
+      <c r="H1" s="21" t="inlineStr">
+        <is>
+          <t>def</t>
+        </is>
+      </c>
+      <c r="I1" s="21" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>total_check</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" s="18">
+      <c r="A2" s="23" t="inlineStr">
+        <is>
+          <t>gp_bruiser</t>
+        </is>
+      </c>
+      <c r="B2" s="23" t="n">
+        <v>65</v>
+      </c>
+      <c r="C2" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="D2" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="F2" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="G2" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H2" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="I2" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="J2" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="18">
+      <c r="A3" s="23" t="inlineStr">
+        <is>
+          <t>gp_armor</t>
+        </is>
+      </c>
+      <c r="B3" s="23" t="n">
+        <v>70</v>
+      </c>
+      <c r="C3" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="F3" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="G3" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="H3" s="23" t="n">
+        <v>70</v>
+      </c>
+      <c r="I3" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J3" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="18">
+      <c r="A4" s="23" t="inlineStr">
+        <is>
+          <t>gp_cavalry</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="D4" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E4" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F4" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="G4" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H4" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="I4" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J4" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="5" ht="15" customHeight="1" s="18">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>gp_flier</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="D5" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="F5" s="23" t="n">
+        <v>60</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H5" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="I5" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J5" s="23" t="n">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1" s="18">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>gp_archer</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="D6" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="F6" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="J6" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1" s="18">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>gp_mage</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>55</v>
+      </c>
+      <c r="E7" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="I7" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="J7" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1" s="18">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>gp_healer</t>
+        </is>
+      </c>
+      <c r="B8" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="E8" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1" s="18">
+      <c r="A9" s="23" t="inlineStr">
+        <is>
+          <t>gp_frail_lucky</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E9" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>75</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1" s="18">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>gp_jagen</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="F10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>15</v>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1" s="18">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>gp_avatar</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>45</v>
+      </c>
+      <c r="F11" s="23" t="n">
+        <v>50</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <v>40</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="J11" s="23" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1" s="18">
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>Archetype profiles, not per-unit growths. Target band 305-325 for recruits; Jagens 150 by design. ADDENDUM (2026-09-25): calibration pass, first ruleset-calibration work after this session's content-generation phase closed out. Six profiles were out of the 305-325 band per this row's own target (and the validation tab's own v10 check): gp_bruiser/gp_armor/gp_cavalry/gp_archer/gp_mage all sat at 290-300, gp_avatar sat at 330. Adjusted each to exactly 315 (the band midpoint) by raising or lowering stats that preserve each archetype's own shape rather than flattening it -- e.g. gp_mage gained HP/def (a fragile caster getting slightly less fragile) while str stayed its deliberate dump stat; gp_armor gained HP/def/res while spd stayed deliberately low; gp_avatar (over band, a generalist) was trimmed evenly across spd/dex/lck rather than gutting one stat. gp_flier(305)/gp_healer(310)/gp_frail_lucky(315) were already in band and left untouched; gp_jagen(150) is exempt by this row's own design note.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -40475,427 +41222,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="0">
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="0"/>
-  </sheetPr>
-  <dimension ref="A1:J13"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
-  <cols>
-    <col width="16" customWidth="1" style="17" min="1" max="1"/>
-    <col width="8" customWidth="1" style="17" min="2" max="9"/>
-    <col width="13" customWidth="1" style="17" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1" s="18">
-      <c r="A1" s="21" t="inlineStr">
-        <is>
-          <t>profile_id</t>
-        </is>
-      </c>
-      <c r="B1" s="21" t="inlineStr">
-        <is>
-          <t>hp</t>
-        </is>
-      </c>
-      <c r="C1" s="21" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="D1" s="21" t="inlineStr">
-        <is>
-          <t>mag</t>
-        </is>
-      </c>
-      <c r="E1" s="21" t="inlineStr">
-        <is>
-          <t>dex</t>
-        </is>
-      </c>
-      <c r="F1" s="21" t="inlineStr">
-        <is>
-          <t>spd</t>
-        </is>
-      </c>
-      <c r="G1" s="21" t="inlineStr">
-        <is>
-          <t>lck</t>
-        </is>
-      </c>
-      <c r="H1" s="21" t="inlineStr">
-        <is>
-          <t>def</t>
-        </is>
-      </c>
-      <c r="I1" s="21" t="inlineStr">
-        <is>
-          <t>res</t>
-        </is>
-      </c>
-      <c r="J1" s="21" t="inlineStr">
-        <is>
-          <t>total_check</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="15" customHeight="1" s="18">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>gp_bruiser</t>
-        </is>
-      </c>
-      <c r="B2" s="23" t="n">
-        <v>65</v>
-      </c>
-      <c r="C2" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="D2" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="F2" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="G2" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H2" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="I2" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="J2" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="18">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>gp_armor</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="n">
-        <v>70</v>
-      </c>
-      <c r="C3" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="D3" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E3" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="F3" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="G3" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="H3" s="23" t="n">
-        <v>70</v>
-      </c>
-      <c r="I3" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="J3" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="18">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>gp_cavalry</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="C4" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="D4" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="F4" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="G4" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H4" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="I4" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="J4" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="18">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>gp_flier</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="C5" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="D5" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="E5" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="F5" s="23" t="n">
-        <v>60</v>
-      </c>
-      <c r="G5" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H5" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="I5" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="J5" s="23" t="n">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="18">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>gp_archer</t>
-        </is>
-      </c>
-      <c r="B6" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="C6" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="D6" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="E6" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="F6" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="G6" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H6" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="I6" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="J6" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="18">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>gp_mage</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="C7" s="23" t="n">
-        <v>10</v>
-      </c>
-      <c r="D7" s="23" t="n">
-        <v>55</v>
-      </c>
-      <c r="E7" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="F7" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="H7" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="I7" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="J7" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="18">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>gp_healer</t>
-        </is>
-      </c>
-      <c r="B8" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="C8" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="D8" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="E8" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="F8" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="G8" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="H8" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="I8" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="J8" s="23" t="n">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="18">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>gp_frail_lucky</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="C9" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="D9" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="E9" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="F9" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>75</v>
-      </c>
-      <c r="H9" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="I9" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="J9" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="18">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>gp_jagen</t>
-        </is>
-      </c>
-      <c r="B10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="C10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="D10" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="E10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="H10" s="23" t="n">
-        <v>20</v>
-      </c>
-      <c r="I10" s="23" t="n">
-        <v>15</v>
-      </c>
-      <c r="J10" s="23" t="n">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="18">
-      <c r="A11" s="23" t="inlineStr">
-        <is>
-          <t>gp_avatar</t>
-        </is>
-      </c>
-      <c r="B11" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="C11" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="D11" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="E11" s="23" t="n">
-        <v>45</v>
-      </c>
-      <c r="F11" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <v>40</v>
-      </c>
-      <c r="H11" s="23" t="n">
-        <v>30</v>
-      </c>
-      <c r="I11" s="23" t="n">
-        <v>35</v>
-      </c>
-      <c r="J11" s="23" t="n">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="18">
-      <c r="A13" s="25" t="inlineStr">
-        <is>
-          <t>Archetype profiles, not per-unit growths. Target band 305-325 for recruits; Jagens 150 by design. ADDENDUM (2026-09-25): calibration pass, first ruleset-calibration work after this session's content-generation phase closed out. Six profiles were out of the 305-325 band per this row's own target (and the validation tab's own v10 check): gp_bruiser/gp_armor/gp_cavalry/gp_archer/gp_mage all sat at 290-300, gp_avatar sat at 330. Adjusted each to exactly 315 (the band midpoint) by raising or lowering stats that preserve each archetype's own shape rather than flattening it -- e.g. gp_mage gained HP/def (a fragile caster getting slightly less fragile) while str stayed its deliberate dump stat; gp_armor gained HP/def/res while spd stayed deliberately low; gp_avatar (over band, a generalist) was trimmed evenly across spd/dex/lck rather than gutting one stat. gp_flier(305)/gp_healer(310)/gp_frail_lucky(315) were already in band and left untouched; gp_jagen(150) is exempt by this row's own design note.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -41993,7 +42320,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Build the Huma's shadow
Canon-first huma parameters, a Huma autoload, a drifting shadow on the open road that marks
units for stats and draws every enemy, the epilogue credit for a fall in the shadow, the
validator rule c07x and tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -13407,7 +13407,7 @@
       </c>
       <c r="H3" s="23" t="inlineStr">
         <is>
-          <t>kill-taboo: whoever lands the blow dies in forty days, no reload undoes it</t>
+          <t>kill-taboo: whoever lands the blow dies in forty days, no reload undoes it ADDENDUM (2026-10-28, HUMA_DESIGN.md): the shadow is built as a drifting patch on its paralogue (promotion_rules prm_huma_*); marked units gain stats and every enemy prefers them; the Huma is never a unit, so the taboo is kept by making the blow impossible; a unit who falls while marked is credited to 'the Huma's shadow' in the epilogue.</t>
         </is>
       </c>
       <c r="I3" s="17" t="inlineStr">
@@ -13557,6 +13557,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -14296,185 +14297,185 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>mnt_warhorse</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>Warhorse</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="17" t="inlineStr">
         <is>
           <t>horse</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>riding</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="17" t="n">
         <v>400</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="17" t="inlineStr">
         <is>
           <t>DRAFTED 2026-10-27. The ordinary mount: acquired by requisition (the standard forges' orders), by capturing a mounted enemy, or by inheritance (a fallen rider's, if it is recovered). Grants riding movement.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>mnt_simurgh</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>the Simurgh</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>nmd_simurgh</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>flying</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>rider_heal</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H3" s="17" t="inlineStr">
         <is>
           <t>Canon: 5 HP/turn to rider and adjacent allies (flat, not percentage). Taken intact from the Simurgh's paralogue.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>mnt_shadhavar</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>the Shadhavar</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>nmd_shadhavar</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>riding</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>pull_foe</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>Canon: every turn, pulls the nearest enemy one tile toward the rider; CANNOT be turned off. A liability on escort maps, an asset on defend maps.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>mnt_karkadann</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>the Karkadann</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>nmd_karkadann</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>riding</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>charge</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H5" s="17" t="inlineStr">
         <is>
           <t>Canon: strong against mounted units; a devastating charge that leaves it stuck one turn. The plain one on purpose.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>mnt_anzu</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="17" t="inlineStr">
         <is>
           <t>the Anzu</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>named</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>nmd_anzu</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>flying</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>unmake_touch</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H6" s="17" t="inlineStr">
         <is>
           <t>Canon: contact degrades enemy weapons; only bites what is already worn; broken means unarmed, not dead. COST: an enemy it has left unarmed drops nothing, so riding it starves your only supply line.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>MOUNTS (drafted 2026-10-27, MOUNTS_DESIGN.md). Canon (roster_gaps): mounts are acquirable equipment (capture / inheritance / requisition), not a class trait -- any of the 18 can end up mounted. A mount gives its rider its movement type (riding or flying) and, for a Named, its signature mechanic. The Huma is a map hazard, not a mount, and has no row. Declared gaps hold: brawl cannot ride or fly, reason cannot fly (see canon_validate DECLARED_GAPS); a unit that already moves as riding, flying or armor takes no mount. The three-way capture of a Named: killed (a prime material), captured at or below capture_hp_pct (a diminished material, a harvest), captured at or below capture_intact_hp_pct (the Named itself, INTACT, as a mount).</t>
         </is>
@@ -36984,7 +36985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38548,7 +38549,91 @@
     <row r="99">
       <c r="A99" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map).</t>
+          <t>prm_huma_maps</t>
+        </is>
+      </c>
+      <c r="B99" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C99" s="17" t="inlineStr">
+        <is>
+          <t>map_p_huma</t>
+        </is>
+      </c>
+      <c r="D99" s="17" t="inlineStr">
+        <is>
+          <t>The Huma: the maps its shadow drifts over (pipe-delimited ids in the text column). Canon: a map hazard, not a mount -- it never lands, so it belongs to the open road.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="17" t="inlineStr">
+        <is>
+          <t>prm_huma_radius</t>
+        </is>
+      </c>
+      <c r="B100" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" s="17" t="n"/>
+      <c r="D100" s="17" t="inlineStr">
+        <is>
+          <t>The Huma: the shadow covers every tile within this many tiles of its centre, in both directions (2 = a 5 x 5 patch).</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="17" t="inlineStr">
+        <is>
+          <t>prm_huma_drift</t>
+        </is>
+      </c>
+      <c r="B101" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C101" s="17" t="n"/>
+      <c r="D101" s="17" t="inlineStr">
+        <is>
+          <t>The Huma: columns the shadow's centre drifts east each turn; it wraps to the west edge at the far end. Its row is the middle of the map.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="17" t="inlineStr">
+        <is>
+          <t>prm_huma_start_col</t>
+        </is>
+      </c>
+      <c r="B102" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="C102" s="17" t="n"/>
+      <c r="D102" s="17" t="inlineStr">
+        <is>
+          <t>The Huma: the column the shadow's centre lies over on turn 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t>prm_huma_bonus</t>
+        </is>
+      </c>
+      <c r="B103" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" s="17" t="n"/>
+      <c r="D103" s="17" t="inlineStr">
+        <is>
+          <t>The Huma: every unit standing in the shadow (yours or theirs) gains this much str, mag, def, res and spd -- 'marked units gain stats'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the Named's mutual knowledge
Killing a Named stand-in is remembered for the run (named_wary_kills, canon 1); after that no
Named can be captured, for a mount or a harvest, and the capture line says why. Canon
parameter, Forge record, saved state, capture gate, validator parameter and tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -13557,11 +13557,10 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>Four of five pact with an OBJECT (feather, shadow, text, nest, song) -- obligations attach to things in this world. Three-way capture: intact (marked weapon, keeps its ability) / harvest (diminished, permanent grudge) / kill (two materials, better weapon). The Named know each other: kill one and the next will not be captured.</t>
+          <t>Four of five pact with an OBJECT (feather, shadow, text, nest, song) -- obligations attach to things in this world. Three-way capture: intact (marked weapon, keeps its ability) / harvest (diminished, permanent grudge) / kill (two materials, better weapon). The Named know each other: kill one and the next will not be captured. ADDENDUM (2026-10-29, NAMED_RULES_DESIGN.md): 'kill one and the next will not be captured' is built as a run-long count of Named stand-ins killed (promotion_rules prm_named_wary_kills = 1): from then on no Named is captured, for a mount or a harvest, and the capture line says why. Killing is therefore the irreversible choice; the Anzu's cost (an unarmed enemy drops nothing) was built with the mounts.</t>
         </is>
       </c>
     </row>
@@ -36985,7 +36984,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38633,7 +38632,23 @@
     <row r="104">
       <c r="A104" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus).</t>
+          <t>prm_named_wary_kills</t>
+        </is>
+      </c>
+      <c r="B104" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C104" s="17" t="n"/>
+      <c r="D104" s="17" t="inlineStr">
+        <is>
+          <t>The Named know each other (named.notes): once this many Named stand-ins have been KILLED (a run-long count, one per creature), no Named will be captured -- no intact mount, no harvest. Canon is 'kill one and the next will not be captured', so 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the Named mounts' defection triggers
The Simurgh leaves when the feather changes hands, the Karkadann when the Ashland is written
off or the writ is decided, the Anzu when Ricberta's literacy is revealed and she is not its
rider; the Shadhavar never. Data-driven mounts columns, Mounts.check_departures, win-screen
and barracks lines, validator checks and tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -14245,7 +14245,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="1" max="1"/>
@@ -14294,6 +14294,26 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="I1" s="26" t="inlineStr">
+        <is>
+          <t>leaves_when</t>
+        </is>
+      </c>
+      <c r="J1" s="26" t="inlineStr">
+        <is>
+          <t>leaves_map_id</t>
+        </is>
+      </c>
+      <c r="K1" s="26" t="inlineStr">
+        <is>
+          <t>leaves_unless_map_id</t>
+        </is>
+      </c>
+      <c r="L1" s="26" t="inlineStr">
+        <is>
+          <t>leaves_line</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
@@ -14361,6 +14381,18 @@
           <t>Canon: 5 HP/turn to rider and adjacent allies (flat, not percentage). Taken intact from the Simurgh's paralogue.</t>
         </is>
       </c>
+      <c r="I3" s="17" t="inlineStr">
+        <is>
+          <t>handed_on</t>
+        </is>
+      </c>
+      <c r="J3" s="17" t="n"/>
+      <c r="K3" s="17" t="n"/>
+      <c r="L3" s="17" t="inlineStr">
+        <is>
+          <t>She arrives green and stops being green: the feather has changed hands, and the Simurgh is gone from the stable.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="17" t="inlineStr">
@@ -14435,6 +14467,26 @@
           <t>Canon: strong against mounted units; a devastating charge that leaves it stuck one turn. The plain one on purpose.</t>
         </is>
       </c>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>map_won|writ</t>
+        </is>
+      </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>map_b15</t>
+        </is>
+      </c>
+      <c r="K5" s="17" t="inlineStr">
+        <is>
+          <t>map_ct19</t>
+        </is>
+      </c>
+      <c r="L5" s="17" t="inlineStr">
+        <is>
+          <t>The Karkadann turns: it guards the doves, and a company that writes the Ashland off, or takes the crown's orders, is not one whose terms it can keep.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
@@ -14472,11 +14524,24 @@
           <t>Canon: contact degrades enemy weapons; only bites what is already worn; broken means unarmed, not dead. COST: an enemy it has left unarmed drops nothing, so riding it starves your only supply line.</t>
         </is>
       </c>
-    </row>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>literacy</t>
+        </is>
+      </c>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="17" t="n"/>
+      <c r="L6" s="17" t="inlineStr">
+        <is>
+          <t>Someone has shown a literacy its rider lacks, and the Anzu turns to the one who can read the register.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>MOUNTS (drafted 2026-10-27, MOUNTS_DESIGN.md). Canon (roster_gaps): mounts are acquirable equipment (capture / inheritance / requisition), not a class trait -- any of the 18 can end up mounted. A mount gives its rider its movement type (riding or flying) and, for a Named, its signature mechanic. The Huma is a map hazard, not a mount, and has no row. Declared gaps hold: brawl cannot ride or fly, reason cannot fly (see canon_validate DECLARED_GAPS); a unit that already moves as riding, flying or armor takes no mount. The three-way capture of a Named: killed (a prime material), captured at or below capture_hp_pct (a diminished material, a harvest), captured at or below capture_intact_hp_pct (the Named itself, INTACT, as a mount).</t>
+          <t>MOUNTS (drafted 2026-10-27, MOUNTS_DESIGN.md). Canon (roster_gaps): mounts are acquirable equipment (capture / inheritance / requisition), not a class trait -- any of the 18 can end up mounted. A mount gives its rider its movement type (riding or flying) and, for a Named, its signature mechanic. The Huma is a map hazard, not a mount, and has no row. Declared gaps hold: brawl cannot ride or fly, reason cannot fly (see canon_validate DECLARED_GAPS); a unit that already moves as riding, flying or armor takes no mount. The three-way capture of a Named: killed (a prime material), captured at or below capture_hp_pct (a diminished material, a harvest), captured at or below capture_intact_hp_pct (the Named itself, INTACT, as a mount). ADDENDUM (2026-10-30, NAMED_DEFECTIONS_DESIGN.md): a Named mount can LEAVE the company, on the creature's own defection trigger (named.defection_trigger): leaves_when is a pipe list of handed_on (the Simurgh: the feather changes hands -- she is given to a different rider than the living one who first held it), map_won (leaves_map_id is won and leaves_unless_map_id never was: the Karkadann, 'the moment you threaten the doves' -- the same Ashland write-off that sends Maren away), writ (the crown's deputy is decided: 'state orders and its terms are simply incompatible') and literacy (Ricberta's literacy is revealed and she is not its rider: the Anzu, 'someone demonstrates literacy you lack'). The Shadhavar has none ('uncontrolled by design': it was never yours to lose) and the Huma never defects. A mount that leaves goes back to the wild and can be won again; leaves_line is what the player is told.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the Kaisareia Trial as the crown's ledger machine
The trial reads out the company's docket of mercies and kills; the avatar recommends in person, or
the commission (the deputy) recommends off its holder's own record. The sentence is final and kept
in the saved run. Canon trial_reading column and mercy weight, Deputy functions, a trial screen,
validator rule c07y and tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -9777,7 +9777,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -9849,6 +9849,11 @@
           <t>weapon_form_bare</t>
         </is>
       </c>
+      <c r="L1" s="21" t="inlineStr">
+        <is>
+          <t>trial_reading</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -10129,6 +10134,11 @@
           <t>Merciful {BASE}</t>
         </is>
       </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>mercy</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -10174,6 +10184,11 @@
           <t>Peacemaker's {BASE}</t>
         </is>
       </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>mercy</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -10219,7 +10234,13 @@
           <t>Taker's {BASE}</t>
         </is>
       </c>
-    </row>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>mercy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -11134,7 +11155,7 @@
       <c r="F7" s="23" t="n"/>
       <c r="G7" s="23" t="inlineStr">
         <is>
-          <t>the Diadem convenes at Kaisareia; the avatar (or whoever holds the relevant commission) recommends sentence; SETS flag_hierophant_verdict (mercy | execution), forking to ch_h33_mercy or ch_h34_war1</t>
+          <t>the Diadem convenes at Kaisareia; the avatar (or whoever holds the relevant commission) recommends sentence; SETS flag_hierophant_verdict (mercy | execution), forking to ch_h33_mercy or ch_h34_war1 ADDENDUM (2026-10-31, TRIAL_DESIGN.md): built as the crown's ledger machine -- the commission holder (the deputy, else the avatar) is read out with the company's docket of mercies and kills; the avatar may recommend in person, or let the commission recommend off the holder's own record; the sentence is final and recorded.</t>
         </is>
       </c>
       <c r="H7" s="23" t="inlineStr">
@@ -14537,7 +14558,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" s="17" t="inlineStr">
         <is>
@@ -37049,7 +37069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38713,7 +38733,23 @@
     <row r="105">
       <c r="A105" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills.</t>
+          <t>prm_trial_mercy_weight</t>
+        </is>
+      </c>
+      <c r="B105" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C105" s="17" t="n"/>
+      <c r="D105" s="17" t="inlineStr">
+        <is>
+          <t>The Kaisareia Trial (ch_h32): the commission holder's own docket -- each recorded mercy (a deed whose epithets.trial_reading is 'mercy': capture, talk, dispersal) counts this many kills; the commission recommends MERCY when mercies x weight &gt;= kills, otherwise EXECUTION.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the calendar's soft footprint
Each sect keeps a calendar from its Venerated-birth sign; a chapter's governing sign advances one a
chapter; units and Named of that sign gain +5 hit and avoid, and the briefing says whose day it is.
Canon columns and parameter, an Almanac autoload, map and overworld lines, validator rule c07z and tests.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -10134,7 +10134,7 @@
           <t>Merciful {BASE}</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" s="17" t="inlineStr">
         <is>
           <t>mercy</t>
         </is>
@@ -10184,7 +10184,7 @@
           <t>Peacemaker's {BASE}</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" s="17" t="inlineStr">
         <is>
           <t>mercy</t>
         </is>
@@ -10234,13 +10234,12 @@
           <t>Taker's {BASE}</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="17" t="inlineStr">
         <is>
           <t>mercy</t>
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -13285,7 +13284,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="17" min="1" max="1"/>
@@ -13342,6 +13341,11 @@
           <t>death_phrase</t>
         </is>
       </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>sign_id</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -13389,6 +13393,11 @@
           <t>the Simurgh's light</t>
         </is>
       </c>
+      <c r="J2" s="17" t="inlineStr">
+        <is>
+          <t>sgn_crab</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="34.5" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -13436,6 +13445,11 @@
           <t>the Huma's shadow</t>
         </is>
       </c>
+      <c r="J3" s="17" t="inlineStr">
+        <is>
+          <t>sgn_lion</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.25" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -13483,6 +13497,11 @@
           <t>the Anzu's stoop</t>
         </is>
       </c>
+      <c r="J4" s="17" t="inlineStr">
+        <is>
+          <t>sgn_maiden</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.25" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -13530,6 +13549,11 @@
           <t>the Karkadann's charge</t>
         </is>
       </c>
+      <c r="J5" s="17" t="inlineStr">
+        <is>
+          <t>sgn_bull</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -13577,7 +13601,13 @@
           <t>the Shadhavar's song</t>
         </is>
       </c>
-    </row>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>sgn_fishes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -19524,7 +19554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:K8"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -19590,6 +19620,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="K1" s="21" t="inlineStr">
+        <is>
+          <t>calendar_sign_id</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -19690,6 +19725,11 @@
           <t>WILD COSMOLOGY, strange rather than spooky: the heavens are populated and the dead are busy; the stars are inhabited; the Venerated is one of many in a succession that continues, and the faithful are not going to a reward but to a POST. New scripture is still arriving, dictated, in progress -- chapters can be added between the player's Act 2 visits. The deposed patrons of the Hundred Cities are the planets: not destroyed by Sargath but ELEVATED, and the register is a misreading of a promotion (spectacularly wrong, and unfalsifiable). Translation runs through a physical instrument -- a stone, a bowl, a hat -- something ordinary the seer uses to read what is not there. They are rebaptising the dead by name off the parish lists, which puts the prophets and the crown's clerks in the same archive for opposite reasons. Prophecy NPCs convert green levies ADDENDUM: this is the sect the_hierophant tab resolves as the Hierophant movement's consolidation point (RESOLVED 2026-09-23) -- see that tab and endings.end_hierophant. ADDENDUM 2 (2026-09-24): ch_p_macuil / map_p_macuil is this sect's paralogue -- reassigned from an earlier, wrong sect_coast attribution; confirmed via locations.loc_north_wind (region_id=rgn_drowned_march, 'the second hermit; likewise refuses') matching the chapter's own title and that region's own 'north' direction. See ch_p_macuil's own corrected note for the full reasoning. ADDENDUM 3 (2026-09-24): ch_p_simurgh / map_p_simurgh is this sect's second paralogue -- locations.loc_simurgh_nest and named.nmd_simurgh, both region_id=rgn_drowned_march. This sect's declared paralogue set is now complete: every locations row tagged chapters='P' with region_id=rgn_drowned_march or rgn_the_shoulder (loc_north_wind, loc_simurgh_nest) has a built chapter.</t>
         </is>
       </c>
+      <c r="K3" s="23" t="inlineStr">
+        <is>
+          <t>sgn_vessel</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.25" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -19740,6 +19780,11 @@
           <t>GROWS THE ENLIGHTENED ONE (canon). A CONFESSION, NOT A PEOPLE: you join it, anyone can, nobody is born a factor, and they recruit loudly in the open. They hold a sovereign state (the Toll League) with a seat and a treaty. Lending is universal in this world -- the Diadem crown lends, the Assembly borrows, the nobility is leveraged through pacts -- so credit is the water everyone swims in, not a marked group's trait. The historical analogue is Christian: the faith spread along trade routes carried by merchants, and Paul worked the port cities as a tentmaker. THE SECT THAT MARKETS TO THE SUFFERING: not 'endure now, reward later' but 'the payment has already been made, on your behalf, and you were not consulted' ADDENDUM (2026-09-24): ch_p_anzu / map_p_anzu is this sect's paralogue -- locations.loc_flats_interior and named.nmd_anzu, both region_id=rgn_glass_flats, already confirmed claimed_by_sect_id=sect_road. rgn_the_throat, this sect's other claimed region (seat of sect_road itself), has its own paralogue-tagged location (loc_open_road, the Huma) not yet built -- this sect's declared paralogue set is not yet complete. ADDENDUM 2 (2026-09-24): ch_p_huma / map_p_huma is this sect's second paralogue --locations.loc_open_road and named.nmd_huma, region_id=rgn_the_throat. This sect's declared paralogue set is now complete: Anzu and the Huma.</t>
         </is>
       </c>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>sgn_scales</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.25" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -19790,6 +19835,11 @@
           <t>grows the Grand Inquisitor; home-front thread, ambushes at reunion ADDENDUM (2026-09-25): ch_k21/ch_k22 (map_k21/map_k22) are this sect's own Act3 content -- locations.loc_kaisareia_walls, region_id=rgn_center (already confirmed claimed_by_sect_id=sect_court), 'the capital as a battlefield'. This is the home-front thread's own climax, the same way ch_e31/e32 belong to sect_road and ch_h31-h34 belong to sect_march -- see ch_k21/ch_k22's own notes for the full reasoning, including an unresolved cross-reference to the 'colossus' motif ch_e32_perverse and the_hierophant also use. The Grand Inquisitor this sect 'grows' per its own notes is not confirmed anywhere to be embodied by, or even present at, this chapter's fight -- that identification is not made here.</t>
         </is>
       </c>
+      <c r="K5" s="23" t="inlineStr">
+        <is>
+          <t>sgn_ram</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -19841,6 +19891,7 @@
         </is>
       </c>
     </row>
+    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -20928,13 +20979,18 @@
           <t>MECHANICAL FOOTPRINT -- keep it light</t>
         </is>
       </c>
-      <c r="B9" s="23" t="n"/>
+      <c r="B9" s="23" t="inlineStr">
+        <is>
+          <t>None ADDENDUM (2026-11-01, CALENDAR_DESIGN.md): built as follows. Each sect keeps a calendar that starts at its Venerated-birth sign (sects.calendar_sign_id: the court/Diadem keeps the Ram, the Continuing Word the Vessel, the Company of the Road the Scales; the Unstained observe nothing and the silent refuse to say, so on their chapters no day is favoured). A chapter belongs to its sect_id's calendar (a chapter with no sect keeps the court's, the state's own). The governing sign of a chapter is the calendar's sign advanced by the chapter's number (one sign a chapter, twelve to the wheel). Units whose sign (from the supports tab, where every roster unit has one) is the governing sign, and Named whose named.sign_id is, gain promotion_rules calendar_bonus hit and avoid. The briefing says whose day it is; there is no menu.</t>
+        </is>
+      </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
           <t>Each Named and each pact-holder is governed by a decan. The calendar tells you which, so certain chapters carry a soft advantage, legible from the briefing, with no new menu. The sect you side with changes which days favour you -- which is astrology doing what people actually used it for. Do not let this become a second stat system.</t>
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -20942,6 +20998,8 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
+    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="18">
       <c r="A14" s="25" t="inlineStr">
         <is>
@@ -37069,7 +37127,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38749,7 +38807,23 @@
     <row r="106">
       <c r="A106" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight.</t>
+          <t>prm_calendar_bonus</t>
+        </is>
+      </c>
+      <c r="B106" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C106" s="17" t="n"/>
+      <c r="D106" s="17" t="inlineStr">
+        <is>
+          <t>The calendar's soft advantage (calendar tab, MECHANICAL FOOTPRINT): on a chapter whose governing sign is a unit's own (or a Named's), that unit gains this much hit and avoid. Light on purpose -- 'do not let this become a second stat system'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build flashbacks F1 and F2
The prologue's map laws become a flashback concept; F1 (the scribes' quarter: copyists, a clerk's
ledger, a page lost silently) and F2 (the last court: a free pact, and the court falls whatever you
do) get chapters, maps, rosters and canon rows; the party is taken into a memory when one falls
due. Flashback autoload, validator updates, tests, a design note and an authorship note.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -920,7 +920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K113"/>
+  <dimension ref="A1:K135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" style="18" min="11" max="11"/>
@@ -5338,6 +5338,696 @@
     </row>
     <row r="113">
       <c r="A113" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_01</t>
+        </is>
+      </c>
+      <c r="B113" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D113" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E113" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I113" s="17" t="n"/>
+      <c r="J113" s="17" t="inlineStr">
+        <is>
+          <t>FLASHBACK F1: the quarter's raiders (reused archetypes) -- zealots of the deposed patrons' cults come for the copy; no names</t>
+        </is>
+      </c>
+      <c r="K113" s="17" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_02</t>
+        </is>
+      </c>
+      <c r="B114" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C114" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D114" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E114" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F114" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="I114" s="17" t="n"/>
+      <c r="J114" s="17" t="n"/>
+      <c r="K114" s="17" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_03</t>
+        </is>
+      </c>
+      <c r="B115" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C115" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D115" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E115" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F115" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I115" s="17" t="n"/>
+      <c r="J115" s="17" t="n"/>
+      <c r="K115" s="17" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_04</t>
+        </is>
+      </c>
+      <c r="B116" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C116" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D116" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E116" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="F116" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="I116" s="17" t="n"/>
+      <c r="J116" s="17" t="n"/>
+      <c r="K116" s="17" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_05</t>
+        </is>
+      </c>
+      <c r="B117" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C117" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D117" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E117" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I117" s="17" t="n"/>
+      <c r="J117" s="17" t="n"/>
+      <c r="K117" s="17" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_06</t>
+        </is>
+      </c>
+      <c r="B118" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C118" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D118" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E118" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I118" s="17" t="n"/>
+      <c r="J118" s="17" t="n"/>
+      <c r="K118" s="17" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_07</t>
+        </is>
+      </c>
+      <c r="B119" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C119" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D119" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E119" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F119" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I119" s="17" t="n"/>
+      <c r="J119" s="17" t="n"/>
+      <c r="K119" s="17" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="17" t="inlineStr">
+        <is>
+          <t>spn_f01_08</t>
+        </is>
+      </c>
+      <c r="B120" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C120" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D120" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E120" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F120" s="17" t="n">
+        <v>13</v>
+      </c>
+      <c r="I120" s="17" t="n"/>
+      <c r="J120" s="17" t="n"/>
+      <c r="K120" s="17" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_01</t>
+        </is>
+      </c>
+      <c r="B121" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C121" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D121" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E121" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F121" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I121" s="17" t="n"/>
+      <c r="J121" s="17" t="inlineStr">
+        <is>
+          <t>FLASHBACK F2: the unbelieving provinces' levies, all on the field at the start; nothing reinforces</t>
+        </is>
+      </c>
+      <c r="K121" s="17" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_02</t>
+        </is>
+      </c>
+      <c r="B122" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C122" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D122" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E122" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F122" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I122" s="17" t="n"/>
+      <c r="J122" s="17" t="n"/>
+      <c r="K122" s="17" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_03</t>
+        </is>
+      </c>
+      <c r="B123" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C123" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D123" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E123" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F123" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="I123" s="17" t="n"/>
+      <c r="J123" s="17" t="n"/>
+      <c r="K123" s="17" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_04</t>
+        </is>
+      </c>
+      <c r="B124" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C124" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D124" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E124" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F124" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="I124" s="17" t="n"/>
+      <c r="J124" s="17" t="n"/>
+      <c r="K124" s="17" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_05</t>
+        </is>
+      </c>
+      <c r="B125" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C125" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D125" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E125" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F125" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="I125" s="17" t="n"/>
+      <c r="J125" s="17" t="n"/>
+      <c r="K125" s="17" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_06</t>
+        </is>
+      </c>
+      <c r="B126" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C126" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D126" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E126" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="F126" s="17" t="n">
+        <v>17</v>
+      </c>
+      <c r="I126" s="17" t="n"/>
+      <c r="J126" s="17" t="n"/>
+      <c r="K126" s="17" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_07</t>
+        </is>
+      </c>
+      <c r="B127" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C127" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D127" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E127" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F127" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I127" s="17" t="n"/>
+      <c r="J127" s="17" t="n"/>
+      <c r="K127" s="17" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_08</t>
+        </is>
+      </c>
+      <c r="B128" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C128" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D128" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E128" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F128" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="I128" s="17" t="n"/>
+      <c r="J128" s="17" t="n"/>
+      <c r="K128" s="17" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_09</t>
+        </is>
+      </c>
+      <c r="B129" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C129" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D129" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E129" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F129" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="I129" s="17" t="n"/>
+      <c r="J129" s="17" t="n"/>
+      <c r="K129" s="17" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_10</t>
+        </is>
+      </c>
+      <c r="B130" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C130" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D130" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E130" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="F130" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="I130" s="17" t="n"/>
+      <c r="J130" s="17" t="n"/>
+      <c r="K130" s="17" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_11</t>
+        </is>
+      </c>
+      <c r="B131" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C131" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D131" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E131" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F131" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="I131" s="17" t="n"/>
+      <c r="J131" s="17" t="n"/>
+      <c r="K131" s="17" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_12</t>
+        </is>
+      </c>
+      <c r="B132" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C132" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D132" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E132" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F132" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="I132" s="17" t="n"/>
+      <c r="J132" s="17" t="n"/>
+      <c r="K132" s="17" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_13</t>
+        </is>
+      </c>
+      <c r="B133" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C133" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D133" s="17" t="inlineStr">
+        <is>
+          <t>ea_looter</t>
+        </is>
+      </c>
+      <c r="E133" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F133" s="17" t="n">
+        <v>15</v>
+      </c>
+      <c r="I133" s="17" t="n"/>
+      <c r="J133" s="17" t="n"/>
+      <c r="K133" s="17" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="17" t="inlineStr">
+        <is>
+          <t>spn_f02_14</t>
+        </is>
+      </c>
+      <c r="B134" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="C134" s="17" t="inlineStr">
+        <is>
+          <t>mook</t>
+        </is>
+      </c>
+      <c r="D134" s="17" t="inlineStr">
+        <is>
+          <t>ea_conscript_levy</t>
+        </is>
+      </c>
+      <c r="E134" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="F134" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="I134" s="17" t="n"/>
+      <c r="J134" s="17" t="n"/>
+      <c r="K134" s="17" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft, review before treating as canon. row/col are grid coordinates in the corresponding map_*.txt file (0-indexed, row0=top). kind: 'boss'/'mook' spawn once at map load; 'den' spawns wave_size new enemy_id units every spawn_interval turns, up to max_waves (null = forever). Positions are placement choices grounded in each map's own text where possible (Boyan on the defend point, Vitomir/the relic hunter den by the reliquary) but the exact tile coordinates themselves are invented, not sourced. Drafted by a Claude Code session, 2026-09-23. ADDENDUM: 12 rows added for map_d01/d03/x11/b15. None of these four maps name a specific antagonist the way map_a02/a03 do -- every row here reuses an existing grounded archetype (ea_looter, ea_conscript_levy, ea_privateer, ea_war_captain) rather than inventing new named characters, per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 2: 9 rows added for map_d02/a01/d05 -- the last three maps in the maps tab without a scene. All three reuse archetypes whose own first_seen_map_id already points at these exact maps (ea_conscript_levy/d02, ea_looter/a01, ea_privateer/d05), the closest grounding this tab gets short of a named individual. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 3: 17 rows added fleshing out the 6 Act2 skeleton maps (v21/v22/c21/m21/m22/r16) into playable content. All reuse existing archetypes -- none of these six name a specific individual antagonist the way map_a02/a03 do -- per each row's own notes. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 4: 22 rows added fleshing out the 10 Act3/paralogue skeleton maps into playable content. Act3's tougher tier is reflected by reusing ea_war_captain/ea_warlord (the miniboss/boss templates) throughout rather than Act1/2's commoner-tier mooks -- no new archetypes invented, same discipline as every prior addendum. Drafted by a Claude Code session, 2026-09-23. ADDENDUM 5 (2026-10-03): added drop_weapon_id -- the weapon this enemy adds to the player's convoy when defeated, once per spawn_id per playthrough. Drafted: Act 1 non-trivial bosses drop a mid-tier weapon, Act 2+ bosses and the paralogues the high tier, and the two Billmen the halberd (the only way to get an overlap weapon). Nobody in the roster can wield a halberd yet (it needs cls_billman) -- it just waits in the convoy.</t>
         </is>
@@ -6449,7 +7139,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="17" min="1" max="1"/>
@@ -9761,6 +10451,126 @@
       <c r="N52" s="17" t="inlineStr">
         <is>
           <t>ch_tp19|ch_ct19</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>ch_f01</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>flashback</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
+        <is>
+          <t>unified</t>
+        </is>
+      </c>
+      <c r="E53" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>The scribes' quarter</t>
+        </is>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
+          <t>fb_f1 (flashbacks tab), act 1 -&gt; 2: the First Register is copied for the first time, under deadline. Protect the copyists; a page is lost and the game does not tell you which; a clerk records deeds as they happen (teaches the epithet ledger). The missing name enters the world here, as an accident nobody notices. Opens after the Act 1 finale (ch_d10|ch_a10) and takes the party into the memory.</t>
+        </is>
+      </c>
+      <c r="K53" s="17" t="inlineStr">
+        <is>
+          <t>eerie</t>
+        </is>
+      </c>
+      <c r="L53" s="17" t="inlineStr">
+        <is>
+          <t>the epithet ledger, by watching a clerk write</t>
+        </is>
+      </c>
+      <c r="M53" s="17" t="inlineStr">
+        <is>
+          <t>loc_scribes_quarter</t>
+        </is>
+      </c>
+      <c r="N53" s="17" t="inlineStr">
+        <is>
+          <t>ch_d10|ch_a10</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>ch_f02</t>
+        </is>
+      </c>
+      <c r="B54" s="17" t="inlineStr">
+        <is>
+          <t>flashback</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
+        <is>
+          <t>unified</t>
+        </is>
+      </c>
+      <c r="E54" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
+        <is>
+          <t>The last court of the Long Reign</t>
+        </is>
+      </c>
+      <c r="G54" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="J54" s="17" t="inlineStr">
+        <is>
+          <t>fb_f2, act 2 -&gt; 3: the church that held the realm together, on the day it stopped being believed. A defence with no reinforcements and no supply; the state simply runs out. The only flashback the player can lose without a restart: losing is the ending of the memory. Teaches what the pact layer costs by letting you spend it freely and lose anyway. Opens after the Reunion (ch_rf20).</t>
+        </is>
+      </c>
+      <c r="K54" s="17" t="inlineStr">
+        <is>
+          <t>elegiac</t>
+        </is>
+      </c>
+      <c r="L54" s="17" t="inlineStr">
+        <is>
+          <t>what the pact layer costs</t>
+        </is>
+      </c>
+      <c r="M54" s="17" t="inlineStr">
+        <is>
+          <t>loc_last_court</t>
+        </is>
+      </c>
+      <c r="N54" s="17" t="inlineStr">
+        <is>
+          <t>ch_rf20</t>
         </is>
       </c>
     </row>
@@ -13607,7 +14417,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -14093,7 +14902,11 @@
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="n"/>
-      <c r="B7" s="23" t="n"/>
+      <c r="B7" s="23" t="inlineStr">
+        <is>
+          <t>flashback</t>
+        </is>
+      </c>
       <c r="C7" s="23" t="n"/>
       <c r="D7" s="23" t="inlineStr">
         <is>
@@ -15353,7 +16166,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="22" customWidth="1" style="17" min="1" max="1"/>
@@ -16958,7 +17771,83 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="25" t="inlineStr">
+      <c r="A39" s="17" t="inlineStr">
+        <is>
+          <t>loc_scribes_quarter</t>
+        </is>
+      </c>
+      <c r="B39" s="17" t="inlineStr">
+        <is>
+          <t>The scribes' quarter (a memory)</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F39" s="17" t="inlineStr">
+        <is>
+          <t>flashback</t>
+        </is>
+      </c>
+      <c r="G39" s="17" t="inlineStr">
+        <is>
+          <t>a flashback ~780 years early, the first copy of the First Register under deadline: not on the world map; the overworld draws it as a memory in the corner, and the party is taken there when it falls due</t>
+        </is>
+      </c>
+      <c r="H39" s="17" t="n">
+        <v>200</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="17" t="inlineStr">
+        <is>
+          <t>loc_last_court</t>
+        </is>
+      </c>
+      <c r="B40" s="17" t="inlineStr">
+        <is>
+          <t>The last court of the Long Reign (a memory)</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
+        <is>
+          <t>both</t>
+        </is>
+      </c>
+      <c r="E40" s="17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>flashback</t>
+        </is>
+      </c>
+      <c r="G40" s="17" t="inlineStr">
+        <is>
+          <t>a flashback, the day the church that held the realm together stopped being believed: not on the world map; a memory in the corner, taken at the end of Act 2</t>
+        </is>
+      </c>
+      <c r="H40" s="17" t="n">
+        <v>320</v>
+      </c>
+      <c r="I40" s="17" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>Comma-separated chapter numbers mean the ground is re-staged. Act 3 fights over Act 1's own fords and roads at army scale, so the player recognises the terrain they escorted a grain wagon across in chapter 3. 'P' = paralogue, unlocked through the supply network rather than the writ, so some stay dark in any given run. 34 locations against 30 chapters plus paralogues -- the world has the capacity, with room to cut. ADDENDUM (2026-10-11): map_x/map_y are overworld screen coordinates (a 1152x540 canvas, drafted: regions follow regions.direction, nothing is to scale); loc_ur_nashet is a flashback, not a place on the map.</t>
         </is>
@@ -18470,7 +19359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="14" customWidth="1" style="17" min="1" max="1"/>
@@ -18528,6 +19417,16 @@
           <t>the_turn</t>
         </is>
       </c>
+      <c r="J1" s="21" t="inlineStr">
+        <is>
+          <t>chapter_id</t>
+        </is>
+      </c>
+      <c r="K1" s="21" t="inlineStr">
+        <is>
+          <t>engine_rule</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.25" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -18575,6 +19474,16 @@
           <t>ends with the city taken and its patron written into a book; the player did that. THE NAME IS NEVER SHOWN: the scribe's hand covers the page, the angle is wrong, the rain is on it. The player performs the founding crime without learning what was written.</t>
         </is>
       </c>
+      <c r="J2" s="23" t="inlineStr">
+        <is>
+          <t>ch_f00</t>
+        </is>
+      </c>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>prologue</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.25" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -18622,6 +19531,16 @@
           <t>the missing name enters the world here, as an accident nobody notices</t>
         </is>
       </c>
+      <c r="J3" s="23" t="inlineStr">
+        <is>
+          <t>ch_f01</t>
+        </is>
+      </c>
+      <c r="K3" s="23" t="inlineStr">
+        <is>
+          <t>copyists|clerk_ledger|lost_page</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="23.25" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -18669,11 +19588,21 @@
           <t>the only flashback the player can lose without a restart; losing is the ending</t>
         </is>
       </c>
+      <c r="J4" s="23" t="inlineStr">
+        <is>
+          <t>ch_f02</t>
+        </is>
+      </c>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>free_pact|falls</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="25" t="inlineStr">
         <is>
-          <t>A flashback may legally break the map laws: it is a memory and it is teaching, not testing. F0 as prologue means the player's first act in the game is the founding crime, performed before they know it is one. Different roster each time; nobody in a flashback is recruitable.</t>
+          <t>A flashback may legally break the map laws: it is a memory and it is teaching, not testing. F0 as prologue means the player's first act in the game is the founding crime, performed before they know it is one. Different roster each time; nobody in a flashback is recruitable. ADDENDUM (2026-11-02, FLASHBACKS_DESIGN.md): F1 and F2 are built as chapters ch_f01 / ch_f02 (act 'flashback'), each with its own roster in prologue_roster (flashback_id) and the prologue's map laws (no permadeath, no forge, no requisition, one weapon each, no repair). engine_rule names the mechanics: F1 copyists (cargo units the quarter must keep), clerk_ledger (a clerk writes deeds down as they happen), lost_page (a page of the copy is lost and no text ever says which); F2 free_pact (every pact answers once, free, and weapons never wear) and falls (the court falls whatever you do; the chapter is complete either way, and which way is remembered). The party is taken to a memory when one falls due.</t>
         </is>
       </c>
     </row>
@@ -18732,7 +19661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U14"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="15" customWidth="1" style="17" min="1" max="1"/>
@@ -18853,6 +19782,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="V1" s="21" t="inlineStr">
+        <is>
+          <t>flashback_id</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="23.85" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -18936,6 +19870,11 @@
           <t>the one time in the whole game the player commands a head of state in person</t>
         </is>
       </c>
+      <c r="V2" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="23.85" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -19019,6 +19958,11 @@
           <t>young, rain-soaked, unbothered, the most destructive thing on the continent; the modern doctrinal bans exist because of people like her</t>
         </is>
       </c>
+      <c r="V3" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -19102,6 +20046,11 @@
           <t>shows the player what mobility buys and what it costs</t>
         </is>
       </c>
+      <c r="V4" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="23.85" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -19185,6 +20134,11 @@
           <t>the span is one tile wide; he simply does not move</t>
         </is>
       </c>
+      <c r="V5" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -19268,6 +20222,11 @@
           <t>the channels teach that water stops feet and not arrows</t>
         </is>
       </c>
+      <c r="V6" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -19351,6 +20310,11 @@
           <t>the highest damage against the statue, which is the point</t>
         </is>
       </c>
+      <c r="V7" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="23" t="inlineStr">
@@ -19434,6 +20398,11 @@
           <t>she can hit the statue too, badly, and the game does not stop her</t>
         </is>
       </c>
+      <c r="V8" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="23.85" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -19512,30 +20481,915 @@
           <t>the player spends the map vaguely protecting him without knowing why</t>
         </is>
       </c>
+      <c r="V9" s="23" t="inlineStr">
+        <is>
+          <t>fb_f0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>pu_f1_hadda</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="inlineStr">
+        <is>
+          <t>Hadda</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="inlineStr">
+        <is>
+          <t>reed-captain of the quarter's watch</t>
+        </is>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>reed-captain of the quarter's watch</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="n"/>
+      <c r="K10" s="23" t="n"/>
+      <c r="L10" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="17" t="inlineStr">
+        <is>
+          <t>sword</t>
+        </is>
+      </c>
+      <c r="N10" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="R10" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S10" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="T10" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U10" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V10" s="23" t="inlineStr">
+        <is>
+          <t>fb_f1</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
-      <c r="A11" s="25" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>pu_f1_zimri</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="inlineStr">
+        <is>
+          <t>Zimri</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="inlineStr">
+        <is>
+          <t>door-warden of the scriptorium</t>
+        </is>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>door-warden of the scriptorium</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="23" t="n"/>
+      <c r="L11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t>lance</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q11" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R11" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S11" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="T11" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U11" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V11" s="23" t="inlineStr">
+        <is>
+          <t>fb_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>pu_f1_nuru</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Nuru</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>a roof-watcher with a short bow</t>
+        </is>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>a roof-watcher with a short bow</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="n"/>
+      <c r="K12" s="23" t="n"/>
+      <c r="L12" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="17" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="N12" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O12" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q12" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R12" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S12" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="T12" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U12" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V12" s="23" t="inlineStr">
+        <is>
+          <t>fb_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="inlineStr">
+        <is>
+          <t>pu_f1_abil</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>Abil</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>a porter who carries the reed bundles</t>
+        </is>
+      </c>
+      <c r="D13" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>a porter who carries the reed bundles</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="n"/>
+      <c r="K13" s="23" t="n"/>
+      <c r="L13" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="17" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="O13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="T13" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V13" s="23" t="inlineStr">
+        <is>
+          <t>fb_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>pu_f1_sinna</t>
+        </is>
+      </c>
+      <c r="B14" s="23" t="inlineStr">
+        <is>
+          <t>Sinna</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="inlineStr">
+        <is>
+          <t>a temple singer who sat with the copyists</t>
+        </is>
+      </c>
+      <c r="D14" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G14" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>a temple singer who sat with the copyists</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="23" t="n"/>
+      <c r="L14" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="17" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="P14" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q14" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R14" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S14" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T14" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="U14" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V14" s="23" t="inlineStr">
+        <is>
+          <t>fb_f1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_valeria</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="inlineStr">
+        <is>
+          <t>Valeria</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="inlineStr">
+        <is>
+          <t>the last bishop of the court</t>
+        </is>
+      </c>
+      <c r="D15" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G15" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" s="23" t="n">
+        <v>22</v>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>the last bishop of the court</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="n"/>
+      <c r="K15" s="23" t="n"/>
+      <c r="L15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" s="17" t="inlineStr">
+        <is>
+          <t>faith</t>
+        </is>
+      </c>
+      <c r="N15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="P15" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R15" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S15" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="U15" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V15" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_corvin</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="inlineStr">
+        <is>
+          <t>Corvin</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="inlineStr">
+        <is>
+          <t>captain of the court's guard</t>
+        </is>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F16" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="H16" s="23" t="n">
+        <v>26</v>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>captain of the court's guard</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="n"/>
+      <c r="K16" s="23" t="n"/>
+      <c r="L16" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="17" t="inlineStr">
+        <is>
+          <t>sword</t>
+        </is>
+      </c>
+      <c r="N16" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O16" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q16" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="R16" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S16" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="T16" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="U16" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V16" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_decimus</t>
+        </is>
+      </c>
+      <c r="B17" s="23" t="inlineStr">
+        <is>
+          <t>Decimus</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="inlineStr">
+        <is>
+          <t>a veteran of the legions' last levy</t>
+        </is>
+      </c>
+      <c r="D17" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H17" s="23" t="n">
+        <v>30</v>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>a veteran of the legions' last levy</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="n"/>
+      <c r="K17" s="23" t="n"/>
+      <c r="L17" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" s="17" t="inlineStr">
+        <is>
+          <t>axe</t>
+        </is>
+      </c>
+      <c r="N17" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="O17" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q17" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S17" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="T17" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U17" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V17" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_lucan</t>
+        </is>
+      </c>
+      <c r="B18" s="23" t="inlineStr">
+        <is>
+          <t>Lucan</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="inlineStr">
+        <is>
+          <t>an archer of the dais</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F18" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="H18" s="23" t="n">
+        <v>21</v>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>an archer of the dais</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="n"/>
+      <c r="K18" s="23" t="n"/>
+      <c r="L18" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="17" t="inlineStr">
+        <is>
+          <t>bow</t>
+        </is>
+      </c>
+      <c r="N18" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="O18" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q18" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R18" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S18" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="T18" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U18" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V18" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_ianthe</t>
+        </is>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
+        <is>
+          <t>Ianthe</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="inlineStr">
+        <is>
+          <t>the court's archivist, who can read the old rites</t>
+        </is>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H19" s="23" t="n">
+        <v>18</v>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>the court's archivist, who can read the old rites</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="n"/>
+      <c r="K19" s="23" t="n"/>
+      <c r="L19" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="17" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="P19" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q19" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="R19" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S19" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="T19" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="U19" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V19" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>pu_f2_sabinus</t>
+        </is>
+      </c>
+      <c r="B20" s="23" t="inlineStr">
+        <is>
+          <t>Sabinus</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="inlineStr">
+        <is>
+          <t>a doorward</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>infantry</t>
+        </is>
+      </c>
+      <c r="F20" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G20" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H20" s="23" t="n">
+        <v>27</v>
+      </c>
+      <c r="I20" s="23" t="inlineStr">
+        <is>
+          <t>a doorward</t>
+        </is>
+      </c>
+      <c r="J20" s="23" t="n"/>
+      <c r="K20" s="23" t="n"/>
+      <c r="L20" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
+        <is>
+          <t>lance</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="O20" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q20" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="S20" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="T20" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="U20" s="23" t="inlineStr">
+        <is>
+          <t>flashback roster: nobody here is recruitable</t>
+        </is>
+      </c>
+      <c r="V20" s="23" t="inlineStr">
+        <is>
+          <t>fb_f2</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="25" t="inlineStr">
         <is>
           <t>Eight ancestors, each a preview of a class the player will spend 30 chapters earning. Nobody here is recruitable and nobody here appears again. The roster is a PROMISE, and the campaign is the bill.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>NOTE -- movement_type sourcing. For each unit, ancestor_of was cross-referenced against classes.movement. pu_sargath/cls_strategist, pu_enmet/cls_warlock, pu_bel_iddin/cls_general+cls_great_shield (both armor), and pu_ilat/cls_bishop are unambiguous single- or agreeing-class matches. pu_tasme=riding is stated outright ('the riding column') and matches her own note. pu_sirru and pu_kadar are each ancestor_of TWO classes with DIFFERENT movement types (Sniper=infantry vs Pavisier=armor; Warrior=infantry vs Housecarl=armor) -- infantry was picked as the first-listed lineage in both cases, not because the prose settles it either way. pu_nashar has no matching class at all ('surveyor'/'clerk thread' aren't class names in the classes tab) and was defaulted to infantry from his non-combat foot-follower role. Review pu_sirru, pu_kadar, and pu_nashar in particular. Drafted by a Claude Code session, 2026-09-14.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>NOTE -- deploy_row/deploy_col added. deploy_row=15 for all 8 (the court, behind the unbroken wall) is stated outright in map_f00_reference.png's caption. deploy_col is only textually grounded for two units: Sargath at col 9 lines up under his seize objective (also col 9, row 2); Bel-Iddin at col 11 lines up under the aqueduct span, explicitly '(11,12)' in the same caption. Enmet/Sirru/Kadar/Ilat/Nashar's columns are my placement choices (roughly: Enmet beside Sargath since she acts on the wall turn 1; Sirru beside Bel-Iddin near the channel she shoots across; Kadar off to the col-14-16 side where the lower terrace gap is; Ilat/Nashar central with the main group) -- not sourced from anything written, review and correct freely. Drafted by a Claude Code session, 2026-09-14.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>NOTE -- weapon_art/str/mag/dex/spd/lck/def/res added. weapon_art is read straight off each unit's own 'role' text (e.g. pu_kadar's role is literally 'axe'); pu_nashar is null, matching his existing 'cannot attack' / dmg_vs_statue=0. The 7 numeric stats are NOT newly invented numbers -- all 7 combat-capable units reuse the exact 'trained' tier baseline already established in unit_base_stats/enemy_archetypes generation (identical to ea_relic_hunter's own stats, since enemies get baseline alone with no growth bonus), with str/mag swapped for the two magic-art units (Enmet, Ilat) the same way trained-tier player mages already skew mag over str (see u_emmerich/u_anselm in unit_base_stats). hp and dmg_vs_statue are untouched. This exists to let real unit-vs-unit combat run on this roster at all -- previously only move/hp/dmg_vs_statue existed, nothing Combat.gd could use. Added for the F0 garrison-soldier fight; review/replace freely if named per-unit stats are ever written. Drafted by a Claude Code session, 2026-09-16.</t>
         </is>
@@ -19891,7 +21745,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="15" customHeight="1" s="18">
       <c r="A8" s="25" t="inlineStr">
         <is>
@@ -20990,7 +22843,6 @@
         </is>
       </c>
     </row>
-    <row r="10"/>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="25" t="inlineStr">
         <is>
@@ -20998,8 +22850,6 @@
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="18">
       <c r="A14" s="25" t="inlineStr">
         <is>
@@ -37127,7 +38977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D107"/>
+  <dimension ref="A1:D108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -38823,7 +40673,23 @@
     <row r="107">
       <c r="A107" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus.</t>
+          <t>prm_flashback_register_pages</t>
+        </is>
+      </c>
+      <c r="B107" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C107" s="17" t="n"/>
+      <c r="D107" s="17" t="inlineStr">
+        <is>
+          <t>Flashback F1: how many pages the First Register's first copy has; one is lost when the copy is finished, and the game never says which (the number is only kept as a hidden flag).</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus. ADDENDUM (2026-11-02): flashback_register_pages.</t>
         </is>
       </c>
     </row>
@@ -42601,7 +44467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" style="18" min="1" max="1"/>
@@ -42826,8 +44692,164 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>cargo_f01_copyist1</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Copyist (first desk)</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I6" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" s="17" t="inlineStr">
+        <is>
+          <t>map_f01: a copyist at a desk (cargo_needed 3 of 4 must live to the eighth turn)</t>
+        </is>
+      </c>
+    </row>
     <row r="7">
       <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>cargo_f01_copyist2</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Copyist (second desk)</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="17" t="n">
+        <v>7</v>
+      </c>
+      <c r="J7" s="17" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
+        <is>
+          <t>cargo_f01_copyist3</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Copyist (third desk)</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I8" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="J8" s="17" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
+        <is>
+          <t>cargo_f01_copyist4</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Copyist (fourth desk)</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
+        <is>
+          <t>armor</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="I9" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="J9" s="17" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>NOTE -- draft cargo units (2026-10-12). A cargo unit is a player-side unit that cannot fight and must be walked to its map's escort tile (the 'E' symbol); delivering one is what the escort objective now means on a map with cargo (maps.cargo_needed delivered to win; if too few remain alive the map is lost) and what ep_delivery counts. Wagon and cart stats are first-pass guesses. d03's 'escort 2 of 3' is canon; the cart's hp and the wagons' defence are mine.</t>
         </is>
@@ -44746,7 +46768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U53"/>
+  <dimension ref="A1:U55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="17" min="1" max="1"/>
@@ -48606,14 +50628,157 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>map_f01</t>
+        </is>
+      </c>
+      <c r="B52" s="17" t="inlineStr">
+        <is>
+          <t>The scribes' quarter</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="n">
+        <v>16</v>
+      </c>
+      <c r="D52" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>defend</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G52" s="17" t="inlineStr">
+        <is>
+          <t>a walled quarter of reed-roofed workshops round one scriptorium; the gate streets run straight in</t>
+        </is>
+      </c>
+      <c r="H52" s="17" t="inlineStr">
+        <is>
+          <t>ch_f01</t>
+        </is>
+      </c>
+      <c r="I52" s="17" t="inlineStr">
+        <is>
+          <t>FLASHBACK F1 (DRAFTED 2026-11-02). Breaks the map laws like the prologue: no permadeath, no dens, no requisition, no forge, one weapon each, no repair, a different roster (prologue_roster fb_f1). Protect the copyists in the scriptorium (cargo_needed 3 of 4) for 8 turns against the quarter's raiders, who come in by the three gates. A clerk writes each deed down as it happens. On the win a page of the copy is lost and nothing ever says which.</t>
+        </is>
+      </c>
+      <c r="J52" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K52" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L52" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M52" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="N52" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="R52" s="17" t="inlineStr">
+        <is>
+          <t>the north gate|the west gate|the east gate</t>
+        </is>
+      </c>
+      <c r="S52" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
+        <is>
+          <t>map_f02</t>
+        </is>
+      </c>
+      <c r="B53" s="17" t="inlineStr">
+        <is>
+          <t>The last court of the Long Reign</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="n">
+        <v>20</v>
+      </c>
+      <c r="D53" s="17" t="n">
+        <v>14</v>
+      </c>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>defend</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G53" s="17" t="inlineStr">
+        <is>
+          <t>a basilica court under a high dais; columns, a nave, two doors to the street</t>
+        </is>
+      </c>
+      <c r="H53" s="17" t="inlineStr">
+        <is>
+          <t>ch_f02</t>
+        </is>
+      </c>
+      <c r="I53" s="17" t="inlineStr">
+        <is>
+          <t>FLASHBACK F2 (DRAFTED 2026-11-02). A defence with no reinforcements and no supply: every enemy is on the field at the start and nothing refills. Every pact answers once, free, and weapons never wear. The court falls whatever you do: the turn limit is dawn and the memory ends then, or sooner if the company is gone. Either way the chapter is complete (losing is the ending of the memory).</t>
+        </is>
+      </c>
+      <c r="J53" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K53" s="17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L53" s="17" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M53" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="R53" s="17" t="inlineStr">
+        <is>
+          <t>the street doors|the side doors</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="25" t="inlineStr">
         <is>
           <t>Sizing band 20x25 to 30x20. Act 3 embeds reuse_in_act3 tilemaps into larger battlefields.</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="25" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="25" t="inlineStr">
         <is>
           <t>MAP LAWS. 1) Every reinforcement has an address: a visible den, ideally capturable, and it may never arrive inside the movement range of a unit who could not have seen it. 2) No single unit solves a map: min_solution_units &gt;= 2, enforced by non-atomic objectives (two seize points, a seal stripped before damage lands, three tiles held at once). 3) A set-piece boss is unreachable for N turns FOR A VISIBLE REASON. 4) Forced deploys are budgeted (&lt;= 1/3 of slots), named, and never a unit held under three chapters. Diversity is an optimized choice, never a constraint: &gt;= 2 approaches favouring different movement types.</t>
         </is>

</xml_diff>

<commit_message>
Build Anna's fixed scene and the enrolment of the dead
Canon gives Anna one fixed scene instead of a support chain, and an off-screen purpose in the March's
rebaptism fieldwork. A drafted pre-battle scene on the eve of the Reunion (the scene pipeline now
understands guests), and a closing line on the fallen roll once she has gone. Her Act 3 payoff stays
the reconstruction gap canon says it is.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -11682,7 +11682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I38"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="17" min="1" max="1"/>
@@ -13063,7 +13063,49 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="25" t="inlineStr">
+      <c r="A38" s="17" t="inlineStr">
+        <is>
+          <t>sc_anna_fixed</t>
+        </is>
+      </c>
+      <c r="B38" s="17" t="inlineStr">
+        <is>
+          <t>ch_rf20</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>pre-battle</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>u_avatar|gst_anna</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>gst_anna</t>
+        </is>
+      </c>
+      <c r="G38" s="17" t="inlineStr">
+        <is>
+          <t>ANNA'S ONE FIXED SCENE (DRAFTED 2026-11-04; stands in for a support chain, which guest_units.support_shape says she has none of). On the eve of the Reunion, before she leaves, Anna lays the parish lists she has been cross-referencing beside the decan tables for the avatar and shows the places where the two will not agree; she does not say what the disagreement means, only that someone must go on enrolling the dead by name, and that it will be her. Nothing here settles the calendar: her Act 3 payoff (the decan token) is still the reconstruction gap in guest_units.gst_anna.act3_payoff.</t>
+        </is>
+      </c>
+      <c r="H38" s="17" t="inlineStr">
+        <is>
+          <t>drafted</t>
+        </is>
+      </c>
+      <c r="I38" s="17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="inlineStr">
         <is>
           <t>One row per generated scene. depends_on_* columns are the coherence contract: the validator fails any scene naming a unit that has not joined by its chapter.</t>
         </is>
@@ -15993,12 +16035,12 @@
       </c>
       <c r="I2" s="17" t="inlineStr">
         <is>
-          <t>No tiered support chain -- one fixed scene instead.</t>
+          <t>No tiered support chain -- one fixed scene instead. ADDENDUM (2026-11-04): built as scenes.sc_anna_fixed, a drafted pre-battle scene on the eve of the Reunion (ch_rf20), shown while she is with the company (SCENES_DESIGN.md / ANNA_DESIGN.md).</t>
         </is>
       </c>
       <c r="J2" s="17" t="inlineStr">
         <is>
-          <t>Continues the Continuing Word's rebaptism fieldwork (prc_rebaptism) off-screen after departing -- cross-referencing parish/decan lists to enroll the plague dead by name.</t>
+          <t>Continues the Continuing Word's rebaptism fieldwork (prc_rebaptism) off-screen after departing -- cross-referencing parish/decan lists to enroll the plague dead by name. ADDENDUM (2026-11-04): built as the closing line of the fallen roll once she has departed (epilogue_text.epi_roll_enrolled): the dead are entered by name.</t>
         </is>
       </c>
       <c r="K2" s="17" t="inlineStr">
@@ -23110,10 +23152,11 @@
       </c>
       <c r="H5" s="23" t="inlineStr">
         <is>
-          <t>puts the prophets and the crown's clerks in the same archive, for opposite reasons</t>
-        </is>
-      </c>
-    </row>
+          <t>puts the prophets and the crown's clerks in the same archive, for opposite reasons ADDENDUM (2026-11-04): the one practice the game carries: once Anna (gst_anna) has gone, the fallen roll closes with the dead entered by name (epilogue_text.epi_roll_enrolled).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="18">
       <c r="A7" s="25" t="inlineStr">
         <is>
@@ -26782,7 +26825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" style="18" min="1" max="1"/>
@@ -27334,8 +27377,26 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="17" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="17" t="inlineStr">
+        <is>
+          <t>epi_roll_enrolled</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>Each of them is entered by name in the parish lists, and the name is spoken.</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>closes the fallen roll once Anna has gone: she continues the Continuing Word's rebaptism fieldwork (prc_rebaptism: nobody is enrolled without their name being spoken) off-screen after departing (guest_units.gst_anna.off_screen_purpose_on_exit)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
         <is>
           <t>IMPLEMENTATION NOTES (2026-10-09). The text of epilogue_generation, built as scripts/epilogue.gd. Wording is DRAFT; placeholders in {BRACES} are filled by the generator, and {A} becomes 'a' or 'an' by the word after it. No line uses a pronoun for the fallen or the partner -- they/them is avoided by naming. TWO EXTENSIONS to the killed_by_type enum, which the original schema did not list: 'band' (an unaffiliated armed band -- looters, relic hunters, privateers, or a soldier on a map that names no polity) and 'hazard' (a death with no hand in it: the cold on map_a03). maps.enemy_polity_id is a DRAFT: state-affiliated enemies belong to the polity opposite the chapter's route (a Diadem-route map fields Assembly soldiers); both-route maps name none, so those soldiers read as a band. Tune it map by map. ADDENDUM (2026-10-20): {WEAPON} is the weapon's provenance name (epithets.weapon_form), which may already read as a possessive ("Taker's Iron Axe"), so the weapon lines say 'The {WEAPON}' rather than '{NAME}'s {WEAPON}'.</t>
         </is>

</xml_diff>

<commit_message>
Build the image, and show proc odds in the forecast
THE IMAGE: one procedural silhouette that grows across the prologue statue, the synod's colossus,
the Hierophant's image and the Idol, with a halo holding 1, 12, 36 and 72 patrons, placed from canon
maps.image_* columns and broken when the prologue's statue is. The forecast panel now shows each
side's patron favour and burden odds. Validator rule c07i, tests and a design note.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -32462,7 +32462,6 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
         <is>
@@ -52471,7 +52470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U55"/>
+  <dimension ref="A1:AA55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="17" min="1" max="1"/>
@@ -52601,6 +52600,36 @@
           <t>breach_symbols</t>
         </is>
       </c>
+      <c r="V1" s="21" t="inlineStr">
+        <is>
+          <t>image_stage</t>
+        </is>
+      </c>
+      <c r="W1" s="21" t="inlineStr">
+        <is>
+          <t>image_col</t>
+        </is>
+      </c>
+      <c r="X1" s="21" t="inlineStr">
+        <is>
+          <t>image_row</t>
+        </is>
+      </c>
+      <c r="Y1" s="21" t="inlineStr">
+        <is>
+          <t>image_w</t>
+        </is>
+      </c>
+      <c r="Z1" s="21" t="inlineStr">
+        <is>
+          <t>image_h</t>
+        </is>
+      </c>
+      <c r="AA1" s="21" t="inlineStr">
+        <is>
+          <t>image_note</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -53372,6 +53401,26 @@
           <t>the terraces (foot)|the aqueduct span (one tile)|the channels (flying only)</t>
         </is>
       </c>
+      <c r="V11" t="n">
+        <v>1</v>
+      </c>
+      <c r="W11" t="n">
+        <v>8</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>the statue of the patron, the one people can still see; it goes still only once it is rubble (the figure breaks when the statue does)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="23" t="inlineStr">
@@ -54040,6 +54089,26 @@
           <t>the approach (foot)|the colossus itself (any)</t>
         </is>
       </c>
+      <c r="V20" t="n">
+        <v>4</v>
+      </c>
+      <c r="W20" t="n">
+        <v>10</v>
+      </c>
+      <c r="X20" t="n">
+        <v>7</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>the Idol: a false godhood assembled from what was taken</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="23" t="inlineStr">
@@ -54184,6 +54253,26 @@
           <t>the hidden approach (foot)|the open field (riding)</t>
         </is>
       </c>
+      <c r="V22" t="n">
+        <v>3</v>
+      </c>
+      <c r="W22" t="n">
+        <v>8</v>
+      </c>
+      <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>the movement gone underground: the same image kept in hiding (a visual callback to the Idol)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="23" t="inlineStr">
@@ -54400,6 +54489,26 @@
           <t>the last field (foot)|the high ground (riding)</t>
         </is>
       </c>
+      <c r="V25" t="n">
+        <v>3</v>
+      </c>
+      <c r="W25" t="n">
+        <v>8</v>
+      </c>
+      <c r="X25" t="n">
+        <v>2</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>6</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>4</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>the Hierophant's colossus, convergent with the Idol</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="23" t="inlineStr">
@@ -56119,6 +56228,26 @@
           <t>the rubble field (all movement, hazard)|the colossus base (foot, riding)</t>
         </is>
       </c>
+      <c r="V48" t="n">
+        <v>2</v>
+      </c>
+      <c r="W48" t="n">
+        <v>15</v>
+      </c>
+      <c r="X48" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>4</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>6</v>
+      </c>
+      <c r="AA48" t="inlineStr">
+        <is>
+          <t>the synod's colossus, fed from the granary district</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="17" t="inlineStr">
@@ -56472,6 +56601,26 @@
           <t>the street doors|the side doors</t>
         </is>
       </c>
+      <c r="V53" t="n">
+        <v>1</v>
+      </c>
+      <c r="W53" t="n">
+        <v>8</v>
+      </c>
+      <c r="X53" t="n">
+        <v>1</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>3</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>3</v>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>the church's image on its dais, on the day it stopped being believed</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
@@ -56483,7 +56632,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>MAP LAWS. 1) Every reinforcement has an address: a visible den, ideally capturable, and it may never arrive inside the movement range of a unit who could not have seen it. 2) No single unit solves a map: min_solution_units &gt;= 2, enforced by non-atomic objectives (two seize points, a seal stripped before damage lands, three tiles held at once). 3) A set-piece boss is unreachable for N turns FOR A VISIBLE REASON. 4) Forced deploys are budgeted (&lt;= 1/3 of slots), named, and never a unit held under three chapters. Diversity is an optimized choice, never a constraint: &gt;= 2 approaches favouring different movement types.</t>
+          <t>MAP LAWS. 1) Every reinforcement has an address: a visible den, ideally capturable, and it may never arrive inside the movement range of a unit who could not have seen it. 2) No single unit solves a map: min_solution_units &gt;= 2, enforced by non-atomic objectives (two seize points, a seal stripped before damage lands, three tiles held at once). 3) A set-piece boss is unreachable for N turns FOR A VISIBLE REASON. 4) Forced deploys are budgeted (&lt;= 1/3 of slots), named, and never a unit held under three chapters. Diversity is an optimized choice, never a constraint: &gt;= 2 approaches favouring different movement types. ADDENDUM (2026-11-07, IMAGE_DESIGN.md): image_stage/col/row/w/h/note place THE IMAGE on the maps where canon shows it: one silhouette that grows with the register (stage 1 the prologue statue and the last court's image; 2 the synod's colossus; 3 the Hierophant's and the movement-underground callback; 4 the Idol), because canon makes the Idol, the colossus and the Hierophant's image deliberately convergent. col/row/w/h are tiles of the map.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build bound ground: seals on map ground scale a patron's gifts by who holds it
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -30364,7 +30364,7 @@
       </c>
       <c r="L36" s="17" t="inlineStr">
         <is>
-          <t>capture</t>
+          <t>capture|unseal</t>
         </is>
       </c>
     </row>
@@ -31508,6 +31508,7 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
@@ -44525,7 +44526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -46657,7 +46658,103 @@
     <row r="134">
       <c r="A134" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus. ADDENDUM (2026-11-02): flashback_register_pages. ADDENDUM (2026-11-05): patron parameters (patron_chance_*, patron_lean_*, patron_chance_min/max, patron_reveal_map). ADDENDUM (2026-11-06): the Morph gamble (morph_*).</t>
+          <t>prm_seal_angel_blessing_pct</t>
+        </is>
+      </c>
+      <c r="B134" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C134" s="17" t="n"/>
+      <c r="D134" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: on a seal held by the angel, blessing chances go to this percent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="17" t="inlineStr">
+        <is>
+          <t>prm_seal_angel_curse_pct</t>
+        </is>
+      </c>
+      <c r="B135" s="17" t="n">
+        <v>50</v>
+      </c>
+      <c r="C135" s="17" t="n"/>
+      <c r="D135" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: ... and curse chances to this percent (the angel's ground softens the price).</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="17" t="inlineStr">
+        <is>
+          <t>prm_seal_demon_blessing_pct</t>
+        </is>
+      </c>
+      <c r="B136" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C136" s="17" t="n"/>
+      <c r="D136" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: on a seal held by the demon, blessing chances go to this percent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="17" t="inlineStr">
+        <is>
+          <t>prm_seal_demon_curse_pct</t>
+        </is>
+      </c>
+      <c r="B137" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C137" s="17" t="n"/>
+      <c r="D137" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: ... and curse chances to this percent (the demon's ground raises everything).</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="inlineStr">
+        <is>
+          <t>prm_seal_balanced_pct</t>
+        </is>
+      </c>
+      <c r="B138" s="17" t="n">
+        <v>125</v>
+      </c>
+      <c r="C138" s="17" t="n"/>
+      <c r="D138" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: on a seal shared by the pair, both blessing and curse chances go to this percent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="inlineStr">
+        <is>
+          <t>prm_seal_home_pct</t>
+        </is>
+      </c>
+      <c r="B139" s="17" t="n">
+        <v>150</v>
+      </c>
+      <c r="C139" s="17" t="n"/>
+      <c r="D139" s="17" t="inlineStr">
+        <is>
+          <t>Bound ground: a bearer born under the very pair the seal belongs to is at home: their blessings are scaled by this percent on top.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus. ADDENDUM (2026-11-02): flashback_register_pages. ADDENDUM (2026-11-05): patron parameters (patron_chance_*, patron_lean_*, patron_chance_min/max, patron_reveal_map). ADDENDUM (2026-11-06): the Morph gamble (morph_*). ADDENDUM (2026-11-08): bound ground (seal_*).</t>
         </is>
       </c>
     </row>
@@ -52470,7 +52567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:AA55"/>
+  <dimension ref="A1:AB55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="17" min="1" max="1"/>
@@ -52630,6 +52727,11 @@
           <t>image_note</t>
         </is>
       </c>
+      <c r="AB1" s="21" t="inlineStr">
+        <is>
+          <t>seal_tiles</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="15" customHeight="1" s="18">
       <c r="A2" s="23" t="inlineStr">
@@ -52712,6 +52814,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB2" t="inlineStr">
+        <is>
+          <t>5:5|9:5</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="15" customHeight="1" s="18">
       <c r="A3" s="23" t="inlineStr">
@@ -52789,6 +52896,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>6:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="18">
       <c r="A4" s="23" t="inlineStr">
@@ -52869,6 +52981,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
       <c r="A5" s="23" t="inlineStr">
@@ -52949,6 +53066,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>6:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="15" customHeight="1" s="18">
       <c r="A6" s="23" t="inlineStr">
@@ -53031,6 +53153,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>6:5|12:5</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="18">
       <c r="A7" s="23" t="inlineStr">
@@ -53180,6 +53307,11 @@
           <t>west crossing|east crossing</t>
         </is>
       </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>8:7|16:7</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="23.25" customHeight="1" s="18">
       <c r="A9" s="23" t="inlineStr">
@@ -53252,6 +53384,11 @@
           <t>the arcade (blocks bows)|the open bazaar|the porters' alley</t>
         </is>
       </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>6:7|12:7</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="79.5" customHeight="1" s="18">
       <c r="A10" s="23" t="inlineStr">
@@ -53329,6 +53466,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>8:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
       <c r="A11" s="23" t="inlineStr">
@@ -53401,22 +53543,22 @@
           <t>the terraces (foot)|the aqueduct span (one tile)|the channels (flying only)</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="V11" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="W11" t="n">
+      <c r="W11" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="X11" t="n">
+      <c r="X11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="Y11" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="Z11" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="AA11" t="inlineStr">
+      <c r="AA11" s="17" t="inlineStr">
         <is>
           <t>the statue of the patron, the one people can still see; it goes still only once it is rubble (the figure breaks when the statue does)</t>
         </is>
@@ -53498,6 +53640,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>6:6|12:6</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="18">
       <c r="A13" s="23" t="inlineStr">
@@ -53575,6 +53722,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>6:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="15" customHeight="1" s="18">
       <c r="A14" s="23" t="inlineStr">
@@ -53647,6 +53799,11 @@
           <t>the hall (foot)|the courtyard (riding)</t>
         </is>
       </c>
+      <c r="AB14" t="inlineStr">
+        <is>
+          <t>6:6|12:6</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="23" t="inlineStr">
@@ -53724,6 +53881,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB15" t="inlineStr">
+        <is>
+          <t>8:7|11:7</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="23" t="inlineStr">
@@ -53801,6 +53963,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB16" t="inlineStr">
+        <is>
+          <t>4:6|9:6</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="23" t="inlineStr">
@@ -53873,6 +54040,11 @@
           <t>the toll road (riding)|the counting house (foot)</t>
         </is>
       </c>
+      <c r="AB17" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="inlineStr">
@@ -53945,6 +54117,11 @@
           <t>the counting floor (foot)|the loading yard (riding)</t>
         </is>
       </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>8:8|14:8</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="23" t="inlineStr">
@@ -54017,6 +54194,11 @@
           <t>the processional (foot)|the high road (riding)|open sky (flying)</t>
         </is>
       </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>9:9|17:9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="23" t="inlineStr">
@@ -54089,24 +54271,29 @@
           <t>the approach (foot)|the colossus itself (any)</t>
         </is>
       </c>
-      <c r="V20" t="n">
+      <c r="V20" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="W20" t="n">
+      <c r="W20" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="X20" t="n">
+      <c r="X20" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="Y20" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="Z20" t="n">
+      <c r="Z20" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="AA20" t="inlineStr">
+      <c r="AA20" s="17" t="inlineStr">
         <is>
           <t>the Idol: a false godhood assembled from what was taken</t>
+        </is>
+      </c>
+      <c r="AB20" s="17" t="inlineStr">
+        <is>
+          <t>8:9|16:9</t>
         </is>
       </c>
     </row>
@@ -54181,6 +54368,11 @@
           <t>the muster line (foot)|the siege road (riding)</t>
         </is>
       </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>8:8|14:8</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="23" t="inlineStr">
@@ -54253,24 +54445,29 @@
           <t>the hidden approach (foot)|the open field (riding)</t>
         </is>
       </c>
-      <c r="V22" t="n">
+      <c r="V22" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="W22" t="n">
+      <c r="W22" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="X22" t="n">
+      <c r="X22" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="Y22" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="Z22" t="n">
+      <c r="Z22" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="AA22" t="inlineStr">
+      <c r="AA22" s="17" t="inlineStr">
         <is>
           <t>the movement gone underground: the same image kept in hiding (a visual callback to the Idol)</t>
+        </is>
+      </c>
+      <c r="AB22" s="17" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
         </is>
       </c>
     </row>
@@ -54345,6 +54542,11 @@
           <t>the front line (foot)|the flank road (riding)</t>
         </is>
       </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
@@ -54417,6 +54619,11 @@
           <t>the front line (foot)|the flank road (riding)</t>
         </is>
       </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="23" t="inlineStr">
@@ -54489,24 +54696,29 @@
           <t>the last field (foot)|the high ground (riding)</t>
         </is>
       </c>
-      <c r="V25" t="n">
+      <c r="V25" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="W25" t="n">
+      <c r="W25" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="X25" t="n">
+      <c r="X25" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="Y25" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="Z25" t="n">
+      <c r="Z25" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="AA25" t="inlineStr">
+      <c r="AA25" s="17" t="inlineStr">
         <is>
           <t>the Hierophant's colossus, convergent with the Idol</t>
+        </is>
+      </c>
+      <c r="AB25" s="17" t="inlineStr">
+        <is>
+          <t>8:8|14:8</t>
         </is>
       </c>
     </row>
@@ -54581,6 +54793,11 @@
           <t>the shoreline farmland (foot)|the lake (flying only, ground blocked around the tower)</t>
         </is>
       </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>4:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="23" t="inlineStr">
@@ -54653,6 +54870,11 @@
           <t>the shores (foot)|the ford, 3 tiles wide (foot only)|open water (flying only)</t>
         </is>
       </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>7:7|14:7</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="17" t="inlineStr">
@@ -54723,6 +54945,11 @@
           <t>the lowest terrace (foot, riding)|the upper terraces (riding blocked)|the sea (flying only)</t>
         </is>
       </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>6:5|10:5</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
@@ -54793,6 +55020,11 @@
           <t>the nest plateau (foot, riding)|the slopes (riding blocked)|the lake far below (flying only)</t>
         </is>
       </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>6:7|10:7</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
@@ -54863,6 +55095,11 @@
           <t>the clearing (foot, riding, safe)|the ash field (all movement, 2 HP/turn hazard)</t>
         </is>
       </c>
+      <c r="AB30" t="inlineStr">
+        <is>
+          <t>6:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
@@ -54933,6 +55170,11 @@
           <t>the open flat (all movement, no cover, no chokepoints)</t>
         </is>
       </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>6:6|12:6</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="17" t="inlineStr">
@@ -55003,6 +55245,11 @@
           <t>the road (all movement, open, no cover)</t>
         </is>
       </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>7:5|13:5</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="17" t="inlineStr">
@@ -55078,6 +55325,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>5:6|10:6</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
@@ -55153,6 +55405,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB34" t="inlineStr">
+        <is>
+          <t>6:3|10:3</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
@@ -55233,6 +55490,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB35" t="inlineStr">
+        <is>
+          <t>6:4|10:4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="17" t="inlineStr">
@@ -55313,6 +55575,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB36" t="inlineStr">
+        <is>
+          <t>5:3|9:3</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="17" t="inlineStr">
@@ -55388,6 +55655,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB37" t="inlineStr">
+        <is>
+          <t>7:5|13:5</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="17" t="inlineStr">
@@ -55463,6 +55735,11 @@
           <t>pol_assembly</t>
         </is>
       </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>7:5|13:5</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
@@ -55543,6 +55820,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="AB39" t="inlineStr">
+        <is>
+          <t>7:5|10:5</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
@@ -55618,6 +55900,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB40" t="inlineStr">
+        <is>
+          <t>6:3|10:3</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="17" t="inlineStr">
@@ -55693,6 +55980,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB41" t="inlineStr">
+        <is>
+          <t>6:3|10:3</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
@@ -55773,6 +56065,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB42" t="inlineStr">
+        <is>
+          <t>6:5|11:5</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="17" t="inlineStr">
@@ -55848,6 +56145,11 @@
           <t>pol_diadem</t>
         </is>
       </c>
+      <c r="AB43" t="inlineStr">
+        <is>
+          <t>6:3|12:3</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="17" t="inlineStr">
@@ -56003,6 +56305,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="AB45" t="inlineStr">
+        <is>
+          <t>6:5|10:5</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
@@ -56083,6 +56390,11 @@
           <t>x</t>
         </is>
       </c>
+      <c r="AB46" t="inlineStr">
+        <is>
+          <t>6:5|10:5</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="17" t="inlineStr">
@@ -56158,6 +56470,11 @@
           <t>b</t>
         </is>
       </c>
+      <c r="AB47" t="inlineStr">
+        <is>
+          <t>8:8|14:8</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="17" t="inlineStr">
@@ -56228,24 +56545,29 @@
           <t>the rubble field (all movement, hazard)|the colossus base (foot, riding)</t>
         </is>
       </c>
-      <c r="V48" t="n">
+      <c r="V48" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="W48" t="n">
+      <c r="W48" s="17" t="n">
         <v>15</v>
       </c>
-      <c r="X48" t="n">
+      <c r="X48" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="Y48" t="n">
+      <c r="Y48" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="Z48" t="n">
+      <c r="Z48" s="17" t="n">
         <v>6</v>
       </c>
-      <c r="AA48" t="inlineStr">
+      <c r="AA48" s="17" t="inlineStr">
         <is>
           <t>the synod's colossus, fed from the granary district</t>
+        </is>
+      </c>
+      <c r="AB48" s="17" t="inlineStr">
+        <is>
+          <t>8:8|14:8</t>
         </is>
       </c>
     </row>
@@ -56318,6 +56640,11 @@
           <t>the clear ground (foot, riding)|the ash band (all movement, hazard)</t>
         </is>
       </c>
+      <c r="AB49" t="inlineStr">
+        <is>
+          <t>7:5|13:5</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="17" t="inlineStr">
@@ -56388,6 +56715,11 @@
           <t>the channel (foot, riding)|the flanking cliffs (impassable, flying passes)</t>
         </is>
       </c>
+      <c r="AB50" t="inlineStr">
+        <is>
+          <t>6:4|12:4</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
@@ -56458,6 +56790,11 @@
           <t>the open field (all movement)|the camps (blocks flying)</t>
         </is>
       </c>
+      <c r="AB51" t="inlineStr">
+        <is>
+          <t>7:7|13:7</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
@@ -56601,22 +56938,22 @@
           <t>the street doors|the side doors</t>
         </is>
       </c>
-      <c r="V53" t="n">
+      <c r="V53" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="W53" t="n">
+      <c r="W53" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="X53" t="n">
+      <c r="X53" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="Y53" t="n">
+      <c r="Y53" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="Z53" t="n">
+      <c r="Z53" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="AA53" t="inlineStr">
+      <c r="AA53" s="17" t="inlineStr">
         <is>
           <t>the church's image on its dais, on the day it stopped being believed</t>
         </is>
@@ -56632,7 +56969,7 @@
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>MAP LAWS. 1) Every reinforcement has an address: a visible den, ideally capturable, and it may never arrive inside the movement range of a unit who could not have seen it. 2) No single unit solves a map: min_solution_units &gt;= 2, enforced by non-atomic objectives (two seize points, a seal stripped before damage lands, three tiles held at once). 3) A set-piece boss is unreachable for N turns FOR A VISIBLE REASON. 4) Forced deploys are budgeted (&lt;= 1/3 of slots), named, and never a unit held under three chapters. Diversity is an optimized choice, never a constraint: &gt;= 2 approaches favouring different movement types. ADDENDUM (2026-11-07, IMAGE_DESIGN.md): image_stage/col/row/w/h/note place THE IMAGE on the maps where canon shows it: one silhouette that grows with the register (stage 1 the prologue statue and the last court's image; 2 the synod's colossus; 3 the Hierophant's and the movement-underground callback; 4 the Idol), because canon makes the Idol, the colossus and the Hierophant's image deliberately convergent. col/row/w/h are tiles of the map.</t>
+          <t>MAP LAWS. 1) Every reinforcement has an address: a visible den, ideally capturable, and it may never arrive inside the movement range of a unit who could not have seen it. 2) No single unit solves a map: min_solution_units &gt;= 2, enforced by non-atomic objectives (two seize points, a seal stripped before damage lands, three tiles held at once). 3) A set-piece boss is unreachable for N turns FOR A VISIBLE REASON. 4) Forced deploys are budgeted (&lt;= 1/3 of slots), named, and never a unit held under three chapters. Diversity is an optimized choice, never a constraint: &gt;= 2 approaches favouring different movement types. ADDENDUM (2026-11-07, IMAGE_DESIGN.md): image_stage/col/row/w/h/note place THE IMAGE on the maps where canon shows it: one silhouette that grows with the register (stage 1 the prologue statue and the last court's image; 2 the synod's colossus; 3 the Hierophant's and the movement-underground callback; 4 the Idol), because canon makes the Idol, the colossus and the Hierophant's image deliberately convergent. col/row/w/h are tiles of the map. ADDENDUM (2026-11-08, BOUND_GROUND_DESIGN.md): seal_tiles ('col:row|col:row') are the BOUND GROUND of a map: seals of the patron pair of the chapter's location (locations.patron_id and patron_side). Whoever stands on one (either side) has its patron gifts scaled by the side that holds it; a Pardoner can break one. DRAFTED: the placements were generated (two passable tiles near the middle, clear of the deploy row, spawns and objectives) and are yours to move.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Build the patron of the day: a chapter's day falls to one pair, whose bearers' blessings run louder
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E6FGS7u3N7gLp8oZBSsLDj
</commit_message>
<xml_diff>
--- a/canon.xlsx
+++ b/canon.xlsx
@@ -31508,7 +31508,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
@@ -44526,7 +44525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D140"/>
+  <dimension ref="A1:D141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="18" min="1" max="1"/>
@@ -46754,7 +46753,23 @@
     <row r="140">
       <c r="A140" s="17" t="inlineStr">
         <is>
-          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus. ADDENDUM (2026-11-02): flashback_register_pages. ADDENDUM (2026-11-05): patron parameters (patron_chance_*, patron_lean_*, patron_chance_min/max, patron_reveal_map). ADDENDUM (2026-11-06): the Morph gamble (morph_*). ADDENDUM (2026-11-08): bound ground (seal_*).</t>
+          <t>prm_patron_day_bonus</t>
+        </is>
+      </c>
+      <c r="B140" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="C140" s="17" t="n"/>
+      <c r="D140" s="17" t="inlineStr">
+        <is>
+          <t>Patron of the day: on a chapter whose calendar names a day, the patron holding that five-day band (the sign's six bands in turn, one band each time the wheel comes round) answers louder for its own bearers: their blessing chances rise by this many points (capped at twice patron_chance_max). Curses are untouched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="inlineStr">
+        <is>
+          <t>NOTE -- draft promotion/levelling/income parameters, review before treating as canon. Everything here is a design proposal (PROMOTION_DESIGN.md), not sourced from the setting; numbers are tuned for playtesting. Drafted by a Claude Code session, 2026-10-05. ADDENDUM (2026-10-06): paragon-tier parameters (level 30, one deed, 1000 gold + 150 a level, +30 stat jump, +5 more growth, +1 slot) and the deed-tracking thresholds. ADDENDUM (2026-10-07): Capture action parameters (capture_hp_pct, income_per_capture). ADDENDUM (2026-10-08): Shove/Smite parameters (shove_distance, smite_distance, shove_armor_resist). ADDENDUM (2026-10-09): collision_pct (Shove/Smite collision damage). ADDENDUM (2026-10-10): Bribe parameters (bribe_cost_base, bribe_cost_per_level, bribe_per_map). ADDENDUM (2026-10-12): delivery_radius. ADDENDUM (2026-10-13): Talk parameters and the rout/talk income rates. ADDENDUM (2026-10-17): forge parameters. ADDENDUM (2026-10-18): guest_level_gap. ADDENDUM (2026-10-19): deputy scoring parameters. ADDENDUM (2026-10-20): weapon-name parameters (weapon_marks_max, reforge_fee). ADDENDUM (2026-10-21): Sapper parameters (sapper_charges, mine_damage). ADDENDUM (2026-10-22): weapon-effect parameters (renew_heal, drain_pct, recoil_damage). ADDENDUM (2026-10-24): Skald parameters (steal_base, steal_per_spd, aura_radius, aura_per_deed, aura_cap). ADDENDUM (2026-10-25): miracle_per_map. ADDENDUM (2026-10-26): requisition tier and standard-forge parameters. ADDENDUM (2026-10-27): mount parameters (capture_intact_hp_pct, mount_heal, charge_distance, charge_bonus, mount_capture_per_map). ADDENDUM (2026-10-28): Huma parameters (huma_maps, huma_radius, huma_drift, huma_start_col, huma_bonus). ADDENDUM (2026-10-29): named_wary_kills. ADDENDUM (2026-10-31): trial_mercy_weight. ADDENDUM (2026-11-01): calendar_bonus. ADDENDUM (2026-11-02): flashback_register_pages. ADDENDUM (2026-11-05): patron parameters (patron_chance_*, patron_lean_*, patron_chance_min/max, patron_reveal_map). ADDENDUM (2026-11-06): the Morph gamble (morph_*). ADDENDUM (2026-11-08): bound ground (seal_*). ADDENDUM (2026-11-09): patron_day_bonus (PATRON_DAY_DESIGN.md).</t>
         </is>
       </c>
     </row>
@@ -52814,7 +52829,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AB2" s="17" t="inlineStr">
         <is>
           <t>5:5|9:5</t>
         </is>
@@ -52896,7 +52911,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AB3" s="17" t="inlineStr">
         <is>
           <t>6:6|10:6</t>
         </is>
@@ -52981,7 +52996,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AB4" s="17" t="inlineStr">
         <is>
           <t>7:7|13:7</t>
         </is>
@@ -53066,7 +53081,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AB5" s="17" t="inlineStr">
         <is>
           <t>6:6|10:6</t>
         </is>
@@ -53153,7 +53168,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AB6" s="17" t="inlineStr">
         <is>
           <t>6:5|12:5</t>
         </is>
@@ -53307,7 +53322,7 @@
           <t>west crossing|east crossing</t>
         </is>
       </c>
-      <c r="AB8" t="inlineStr">
+      <c r="AB8" s="17" t="inlineStr">
         <is>
           <t>8:7|16:7</t>
         </is>
@@ -53384,7 +53399,7 @@
           <t>the arcade (blocks bows)|the open bazaar|the porters' alley</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
+      <c r="AB9" s="17" t="inlineStr">
         <is>
           <t>6:7|12:7</t>
         </is>
@@ -53466,7 +53481,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB10" t="inlineStr">
+      <c r="AB10" s="17" t="inlineStr">
         <is>
           <t>8:7|13:7</t>
         </is>
@@ -53640,7 +53655,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
+      <c r="AB12" s="17" t="inlineStr">
         <is>
           <t>6:6|12:6</t>
         </is>
@@ -53722,7 +53737,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB13" t="inlineStr">
+      <c r="AB13" s="17" t="inlineStr">
         <is>
           <t>6:6|10:6</t>
         </is>
@@ -53799,7 +53814,7 @@
           <t>the hall (foot)|the courtyard (riding)</t>
         </is>
       </c>
-      <c r="AB14" t="inlineStr">
+      <c r="AB14" s="17" t="inlineStr">
         <is>
           <t>6:6|12:6</t>
         </is>
@@ -53881,7 +53896,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB15" t="inlineStr">
+      <c r="AB15" s="17" t="inlineStr">
         <is>
           <t>8:7|11:7</t>
         </is>
@@ -53963,7 +53978,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB16" t="inlineStr">
+      <c r="AB16" s="17" t="inlineStr">
         <is>
           <t>4:6|9:6</t>
         </is>
@@ -54040,7 +54055,7 @@
           <t>the toll road (riding)|the counting house (foot)</t>
         </is>
       </c>
-      <c r="AB17" t="inlineStr">
+      <c r="AB17" s="17" t="inlineStr">
         <is>
           <t>7:7|13:7</t>
         </is>
@@ -54117,7 +54132,7 @@
           <t>the counting floor (foot)|the loading yard (riding)</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
+      <c r="AB18" s="17" t="inlineStr">
         <is>
           <t>8:8|14:8</t>
         </is>
@@ -54194,7 +54209,7 @@
           <t>the processional (foot)|the high road (riding)|open sky (flying)</t>
         </is>
       </c>
-      <c r="AB19" t="inlineStr">
+      <c r="AB19" s="17" t="inlineStr">
         <is>
           <t>9:9|17:9</t>
         </is>
@@ -54368,7 +54383,7 @@
           <t>the muster line (foot)|the siege road (riding)</t>
         </is>
       </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AB21" s="17" t="inlineStr">
         <is>
           <t>8:8|14:8</t>
         </is>
@@ -54542,7 +54557,7 @@
           <t>the front line (foot)|the flank road (riding)</t>
         </is>
       </c>
-      <c r="AB23" t="inlineStr">
+      <c r="AB23" s="17" t="inlineStr">
         <is>
           <t>7:7|13:7</t>
         </is>
@@ -54619,7 +54634,7 @@
           <t>the front line (foot)|the flank road (riding)</t>
         </is>
       </c>
-      <c r="AB24" t="inlineStr">
+      <c r="AB24" s="17" t="inlineStr">
         <is>
           <t>7:7|13:7</t>
         </is>
@@ -54793,7 +54808,7 @@
           <t>the shoreline farmland (foot)|the lake (flying only, ground blocked around the tower)</t>
         </is>
       </c>
-      <c r="AB26" t="inlineStr">
+      <c r="AB26" s="17" t="inlineStr">
         <is>
           <t>4:6|10:6</t>
         </is>
@@ -54870,7 +54885,7 @@
           <t>the shores (foot)|the ford, 3 tiles wide (foot only)|open water (flying only)</t>
         </is>
       </c>
-      <c r="AB27" t="inlineStr">
+      <c r="AB27" s="17" t="inlineStr">
         <is>
           <t>7:7|14:7</t>
         </is>
@@ -54945,7 +54960,7 @@
           <t>the lowest terrace (foot, riding)|the upper terraces (riding blocked)|the sea (flying only)</t>
         </is>
       </c>
-      <c r="AB28" t="inlineStr">
+      <c r="AB28" s="17" t="inlineStr">
         <is>
           <t>6:5|10:5</t>
         </is>
@@ -55020,7 +55035,7 @@
           <t>the nest plateau (foot, riding)|the slopes (riding blocked)|the lake far below (flying only)</t>
         </is>
       </c>
-      <c r="AB29" t="inlineStr">
+      <c r="AB29" s="17" t="inlineStr">
         <is>
           <t>6:7|10:7</t>
         </is>
@@ -55095,7 +55110,7 @@
           <t>the clearing (foot, riding, safe)|the ash field (all movement, 2 HP/turn hazard)</t>
         </is>
       </c>
-      <c r="AB30" t="inlineStr">
+      <c r="AB30" s="17" t="inlineStr">
         <is>
           <t>6:6|10:6</t>
         </is>
@@ -55170,7 +55185,7 @@
           <t>the open flat (all movement, no cover, no chokepoints)</t>
         </is>
       </c>
-      <c r="AB31" t="inlineStr">
+      <c r="AB31" s="17" t="inlineStr">
         <is>
           <t>6:6|12:6</t>
         </is>
@@ -55245,7 +55260,7 @@
           <t>the road (all movement, open, no cover)</t>
         </is>
       </c>
-      <c r="AB32" t="inlineStr">
+      <c r="AB32" s="17" t="inlineStr">
         <is>
           <t>7:5|13:5</t>
         </is>
@@ -55325,7 +55340,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AB33" t="inlineStr">
+      <c r="AB33" s="17" t="inlineStr">
         <is>
           <t>5:6|10:6</t>
         </is>
@@ -55405,7 +55420,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB34" t="inlineStr">
+      <c r="AB34" s="17" t="inlineStr">
         <is>
           <t>6:3|10:3</t>
         </is>
@@ -55490,7 +55505,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB35" t="inlineStr">
+      <c r="AB35" s="17" t="inlineStr">
         <is>
           <t>6:4|10:4</t>
         </is>
@@ -55575,7 +55590,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB36" t="inlineStr">
+      <c r="AB36" s="17" t="inlineStr">
         <is>
           <t>5:3|9:3</t>
         </is>
@@ -55655,7 +55670,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB37" t="inlineStr">
+      <c r="AB37" s="17" t="inlineStr">
         <is>
           <t>7:5|13:5</t>
         </is>
@@ -55735,7 +55750,7 @@
           <t>pol_assembly</t>
         </is>
       </c>
-      <c r="AB38" t="inlineStr">
+      <c r="AB38" s="17" t="inlineStr">
         <is>
           <t>7:5|13:5</t>
         </is>
@@ -55820,7 +55835,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AB39" t="inlineStr">
+      <c r="AB39" s="17" t="inlineStr">
         <is>
           <t>7:5|10:5</t>
         </is>
@@ -55900,7 +55915,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB40" t="inlineStr">
+      <c r="AB40" s="17" t="inlineStr">
         <is>
           <t>6:3|10:3</t>
         </is>
@@ -55980,7 +55995,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB41" t="inlineStr">
+      <c r="AB41" s="17" t="inlineStr">
         <is>
           <t>6:3|10:3</t>
         </is>
@@ -56065,7 +56080,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB42" t="inlineStr">
+      <c r="AB42" s="17" t="inlineStr">
         <is>
           <t>6:5|11:5</t>
         </is>
@@ -56145,7 +56160,7 @@
           <t>pol_diadem</t>
         </is>
       </c>
-      <c r="AB43" t="inlineStr">
+      <c r="AB43" s="17" t="inlineStr">
         <is>
           <t>6:3|12:3</t>
         </is>
@@ -56305,7 +56320,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AB45" t="inlineStr">
+      <c r="AB45" s="17" t="inlineStr">
         <is>
           <t>6:5|10:5</t>
         </is>
@@ -56390,7 +56405,7 @@
           <t>x</t>
         </is>
       </c>
-      <c r="AB46" t="inlineStr">
+      <c r="AB46" s="17" t="inlineStr">
         <is>
           <t>6:5|10:5</t>
         </is>
@@ -56470,7 +56485,7 @@
           <t>b</t>
         </is>
       </c>
-      <c r="AB47" t="inlineStr">
+      <c r="AB47" s="17" t="inlineStr">
         <is>
           <t>8:8|14:8</t>
         </is>
@@ -56640,7 +56655,7 @@
           <t>the clear ground (foot, riding)|the ash band (all movement, hazard)</t>
         </is>
       </c>
-      <c r="AB49" t="inlineStr">
+      <c r="AB49" s="17" t="inlineStr">
         <is>
           <t>7:5|13:5</t>
         </is>
@@ -56715,7 +56730,7 @@
           <t>the channel (foot, riding)|the flanking cliffs (impassable, flying passes)</t>
         </is>
       </c>
-      <c r="AB50" t="inlineStr">
+      <c r="AB50" s="17" t="inlineStr">
         <is>
           <t>6:4|12:4</t>
         </is>
@@ -56790,7 +56805,7 @@
           <t>the open field (all movement)|the camps (blocks flying)</t>
         </is>
       </c>
-      <c r="AB51" t="inlineStr">
+      <c r="AB51" s="17" t="inlineStr">
         <is>
           <t>7:7|13:7</t>
         </is>

</xml_diff>